<commit_message>
overall_tier_score py file code finalized
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -9,13 +9,13 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="tier_score_sheet" sheetId="1" r:id="rId1"/>
     <sheet name="comment_table" sheetId="2" r:id="rId2"/>
-    <sheet name="overall_tier_scores" sheetId="5" r:id="rId3"/>
-    <sheet name="tier_score_sheet_copy" sheetId="3" r:id="rId4"/>
+    <sheet name="overall_tier_scores" sheetId="3" r:id="rId3"/>
+    <sheet name="tier_score_sheet_copy" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="overall_tier_score" localSheetId="2">overall_tier_scores!$A$1:$M$53</definedName>
@@ -24,32 +24,8 @@
 </workbook>
 </file>
 
-<file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" name="overall_tier_score" type="6" refreshedVersion="6" background="1" saveData="1">
-    <textPr codePage="850" sourceFile="D:\Project\GPU_Project\overall_tier_score.csv" tab="0" comma="1">
-      <textFields count="13">
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-        <textField/>
-      </textFields>
-    </textPr>
-  </connection>
-</connections>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="117">
   <si>
     <t>gpu_name</t>
   </si>
@@ -357,7 +333,7 @@
     <t>currently Intel Arc GPU drivers have several issues affecting performance and stability</t>
   </si>
   <si>
-    <t>the Radeon RX 7900 XT and 7900 XTX currently having high junction temperature issues</t>
+    <t>some of the Radeon RX 7900 XT and 7900 XTX currently having high junction temperature issues; AMD has acknowledged them and replace them under warranty</t>
   </si>
   <si>
     <t>low_profile</t>
@@ -369,31 +345,37 @@
     <t>graphics card is very large and may require a case upgrade (over 300 mm in length and/or 60 mm in height)</t>
   </si>
   <si>
+    <t>radeon_high_idle_power</t>
+  </si>
+  <si>
+    <t>when connecting to high resolution and high refresh rate monitors (sometimes up to 100 W); this is a known issue and AMD is working on a driver fix for this</t>
+  </si>
+  <si>
+    <t>positive_additional_score_multiplier</t>
+  </si>
+  <si>
+    <t>negative_additional_score_multiplier</t>
+  </si>
+  <si>
+    <t>overall_additional_score</t>
+  </si>
+  <si>
+    <t>net_tier_score</t>
+  </si>
+  <si>
+    <t>non_rt_positive_score_multiplier</t>
+  </si>
+  <si>
+    <t>non_rt_additional_score</t>
+  </si>
+  <si>
+    <t>non_rt_net_score</t>
+  </si>
+  <si>
     <t>gpu_name_tpu</t>
   </si>
   <si>
     <t>Geforce RTX 3060</t>
-  </si>
-  <si>
-    <t>positive_additional_score_multiplier</t>
-  </si>
-  <si>
-    <t>negative_additional_score_multiplier</t>
-  </si>
-  <si>
-    <t>overall_additional_score</t>
-  </si>
-  <si>
-    <t>net_tier_score</t>
-  </si>
-  <si>
-    <t>non_rt_positive_score_multiplier</t>
-  </si>
-  <si>
-    <t>non_rt_net_score</t>
-  </si>
-  <si>
-    <t>non_rt_additional_score</t>
   </si>
 </sst>
 </file>
@@ -569,10 +551,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="overall_tier_score" connectionId="1" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2775,7 +2753,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
@@ -2879,7 +2857,7 @@
         <v>102</v>
       </c>
       <c r="C9">
-        <v>-10</v>
+        <v>-5</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -2902,6 +2880,17 @@
       </c>
       <c r="C11">
         <v>-5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B12" t="s">
+        <v>107</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2914,20 +2903,20 @@
   <dimension ref="A1:O53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="31.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -2968,10 +2957,10 @@
         <v>112</v>
       </c>
       <c r="N1" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>114</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -3012,11 +3001,11 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <f>(M2+J2)*D2</f>
+        <f t="shared" ref="N2:N33" si="0">(M2+J2)*D2</f>
         <v>-0.121</v>
       </c>
       <c r="O2">
-        <f>D2+N2</f>
+        <f t="shared" ref="O2:O33" si="1">D2+N2</f>
         <v>1.089</v>
       </c>
     </row>
@@ -3051,12 +3040,12 @@
       <c r="M3">
         <v>0</v>
       </c>
-      <c r="N3" s="2">
-        <f t="shared" ref="N3:N53" si="0">(M3+J3)*D3</f>
+      <c r="N3">
+        <f t="shared" si="0"/>
         <v>-0.28100000000000003</v>
       </c>
-      <c r="O3" s="2">
-        <f t="shared" ref="O3:O53" si="1">D3+N3</f>
+      <c r="O3">
+        <f t="shared" si="1"/>
         <v>2.5289999999999999</v>
       </c>
     </row>
@@ -3091,11 +3080,11 @@
       <c r="M4">
         <v>0</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4">
         <f t="shared" si="0"/>
         <v>-0.30099999999999999</v>
       </c>
-      <c r="O4" s="2">
+      <c r="O4">
         <f t="shared" si="1"/>
         <v>2.7089999999999996</v>
       </c>
@@ -3134,11 +3123,11 @@
       <c r="M5">
         <v>0</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O5" s="2">
+      <c r="O5">
         <f t="shared" si="1"/>
         <v>1</v>
       </c>
@@ -3177,11 +3166,11 @@
       <c r="M6">
         <v>0</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O6" s="2">
+      <c r="O6">
         <f t="shared" si="1"/>
         <v>1.6</v>
       </c>
@@ -3223,11 +3212,11 @@
       <c r="M7">
         <v>0.05</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7">
         <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
-      <c r="O7" s="2">
+      <c r="O7">
         <f t="shared" si="1"/>
         <v>1.3125</v>
       </c>
@@ -3269,11 +3258,11 @@
       <c r="M8">
         <v>0.05</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8">
         <f t="shared" si="0"/>
         <v>6.9499999999999992E-2</v>
       </c>
-      <c r="O8" s="2">
+      <c r="O8">
         <f t="shared" si="1"/>
         <v>1.4594999999999998</v>
       </c>
@@ -3312,11 +3301,11 @@
       <c r="M9">
         <v>0</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O9" s="2">
+      <c r="O9">
         <f t="shared" si="1"/>
         <v>1.69</v>
       </c>
@@ -3355,11 +3344,11 @@
       <c r="M10">
         <v>0</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O10" s="2">
+      <c r="O10">
         <f t="shared" si="1"/>
         <v>1.87</v>
       </c>
@@ -3398,11 +3387,11 @@
       <c r="M11">
         <v>0</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O11" s="2">
+      <c r="O11">
         <f t="shared" si="1"/>
         <v>2.1</v>
       </c>
@@ -3441,11 +3430,11 @@
       <c r="M12">
         <v>0</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O12" s="2">
+      <c r="O12">
         <f t="shared" si="1"/>
         <v>2.15</v>
       </c>
@@ -3487,11 +3476,11 @@
       <c r="M13">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13">
         <f t="shared" si="0"/>
         <v>0.17710000000000001</v>
       </c>
-      <c r="O13" s="2">
+      <c r="O13">
         <f t="shared" si="1"/>
         <v>2.7070999999999996</v>
       </c>
@@ -3533,11 +3522,11 @@
       <c r="M14">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N14" s="2">
+      <c r="N14">
         <f t="shared" si="0"/>
         <v>0.1988</v>
       </c>
-      <c r="O14" s="2">
+      <c r="O14">
         <f t="shared" si="1"/>
         <v>3.0387999999999997</v>
       </c>
@@ -3576,11 +3565,11 @@
       <c r="M15">
         <v>0</v>
       </c>
-      <c r="N15" s="2">
+      <c r="N15">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O15" s="2">
+      <c r="O15">
         <f t="shared" si="1"/>
         <v>2.95</v>
       </c>
@@ -3622,11 +3611,11 @@
       <c r="M16">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N16" s="2">
+      <c r="N16">
         <f t="shared" si="0"/>
         <v>0.22820000000000001</v>
       </c>
-      <c r="O16" s="2">
+      <c r="O16">
         <f t="shared" si="1"/>
         <v>3.4882</v>
       </c>
@@ -3668,11 +3657,11 @@
       <c r="M17">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N17" s="2">
+      <c r="N17">
         <f t="shared" si="0"/>
         <v>0.24500000000000002</v>
       </c>
-      <c r="O17" s="2">
+      <c r="O17">
         <f t="shared" si="1"/>
         <v>3.7450000000000001</v>
       </c>
@@ -3714,11 +3703,11 @@
       <c r="M18">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N18" s="2">
+      <c r="N18">
         <f t="shared" si="0"/>
         <v>0.25690000000000002</v>
       </c>
-      <c r="O18" s="2">
+      <c r="O18">
         <f t="shared" si="1"/>
         <v>3.9268999999999998</v>
       </c>
@@ -3760,11 +3749,11 @@
       <c r="M19">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N19" s="2">
+      <c r="N19">
         <f t="shared" si="0"/>
         <v>0.28910000000000002</v>
       </c>
-      <c r="O19" s="2">
+      <c r="O19">
         <f t="shared" si="1"/>
         <v>4.4191000000000003</v>
       </c>
@@ -3806,11 +3795,11 @@
       <c r="M20">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N20" s="2">
+      <c r="N20">
         <f t="shared" si="0"/>
         <v>0.15260000000000001</v>
       </c>
-      <c r="O20" s="2">
+      <c r="O20">
         <f t="shared" si="1"/>
         <v>2.3326000000000002</v>
       </c>
@@ -3852,11 +3841,11 @@
       <c r="M21">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N21" s="2">
+      <c r="N21">
         <f t="shared" si="0"/>
         <v>0.18900000000000003</v>
       </c>
-      <c r="O21" s="2">
+      <c r="O21">
         <f t="shared" si="1"/>
         <v>2.8890000000000002</v>
       </c>
@@ -3898,11 +3887,11 @@
       <c r="M22">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N22" s="2">
+      <c r="N22">
         <f t="shared" si="0"/>
         <v>0.2107</v>
       </c>
-      <c r="O22" s="2">
+      <c r="O22">
         <f t="shared" si="1"/>
         <v>3.2206999999999999</v>
       </c>
@@ -3944,11 +3933,11 @@
       <c r="M23">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N23" s="2">
+      <c r="N23">
         <f t="shared" si="0"/>
         <v>0.26319999999999999</v>
       </c>
-      <c r="O23" s="2">
+      <c r="O23">
         <f t="shared" si="1"/>
         <v>4.0232000000000001</v>
       </c>
@@ -3990,11 +3979,11 @@
       <c r="M24">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N24" s="2">
+      <c r="N24">
         <f t="shared" si="0"/>
         <v>0.30870000000000003</v>
       </c>
-      <c r="O24" s="2">
+      <c r="O24">
         <f t="shared" si="1"/>
         <v>4.7187000000000001</v>
       </c>
@@ -4036,11 +4025,11 @@
       <c r="M25">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N25" s="2">
+      <c r="N25">
         <f t="shared" si="0"/>
         <v>0.33040000000000003</v>
       </c>
-      <c r="O25" s="2">
+      <c r="O25">
         <f t="shared" si="1"/>
         <v>5.0503999999999998</v>
       </c>
@@ -4082,11 +4071,11 @@
       <c r="M26">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N26" s="2">
+      <c r="N26">
         <f t="shared" si="0"/>
         <v>0.38220000000000004</v>
       </c>
-      <c r="O26" s="2">
+      <c r="O26">
         <f t="shared" si="1"/>
         <v>5.8422000000000001</v>
       </c>
@@ -4128,11 +4117,11 @@
       <c r="M27">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N27" s="2">
+      <c r="N27">
         <f t="shared" si="0"/>
         <v>0.40110000000000007</v>
       </c>
-      <c r="O27" s="2">
+      <c r="O27">
         <f t="shared" si="1"/>
         <v>6.1311000000000009</v>
       </c>
@@ -4174,11 +4163,11 @@
       <c r="M28">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N28" s="2">
+      <c r="N28">
         <f t="shared" si="0"/>
         <v>0.44940000000000002</v>
       </c>
-      <c r="O28" s="2">
+      <c r="O28">
         <f t="shared" si="1"/>
         <v>6.8693999999999997</v>
       </c>
@@ -4223,11 +4212,11 @@
       <c r="M29">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N29" s="2">
+      <c r="N29">
         <f t="shared" si="0"/>
         <v>0.12960000000000002</v>
       </c>
-      <c r="O29" s="2">
+      <c r="O29">
         <f t="shared" si="1"/>
         <v>6.6096000000000004</v>
       </c>
@@ -4272,11 +4261,11 @@
       <c r="M30">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N30" s="2">
+      <c r="N30">
         <f t="shared" si="0"/>
         <v>0.14000000000000001</v>
       </c>
-      <c r="O30" s="2">
+      <c r="O30">
         <f t="shared" si="1"/>
         <v>7.14</v>
       </c>
@@ -4321,11 +4310,11 @@
       <c r="M31">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N31" s="2">
+      <c r="N31">
         <f t="shared" si="0"/>
         <v>0.16220000000000001</v>
       </c>
-      <c r="O31" s="2">
+      <c r="O31">
         <f t="shared" si="1"/>
         <v>8.2721999999999998</v>
       </c>
@@ -4370,11 +4359,11 @@
       <c r="M32">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N32" s="2">
+      <c r="N32">
         <f t="shared" si="0"/>
         <v>0.20280000000000006</v>
       </c>
-      <c r="O32" s="2">
+      <c r="O32">
         <f t="shared" si="1"/>
         <v>10.3428</v>
       </c>
@@ -4416,11 +4405,11 @@
       <c r="M33">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="N33" s="2">
+      <c r="N33">
         <f t="shared" si="0"/>
         <v>0.46760000000000002</v>
       </c>
-      <c r="O33" s="2">
+      <c r="O33">
         <f t="shared" si="1"/>
         <v>7.1475999999999997</v>
       </c>
@@ -4453,12 +4442,12 @@
       <c r="M34">
         <v>0</v>
       </c>
-      <c r="N34" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O34" s="2">
-        <f t="shared" si="1"/>
+      <c r="N34">
+        <f t="shared" ref="N34:N65" si="2">(M34+J34)*D34</f>
+        <v>0</v>
+      </c>
+      <c r="O34">
+        <f t="shared" ref="O34:O65" si="3">D34+N34</f>
         <v>1.62</v>
       </c>
     </row>
@@ -4496,12 +4485,12 @@
       <c r="M35">
         <v>0</v>
       </c>
-      <c r="N35" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O35" s="2">
-        <f t="shared" si="1"/>
+      <c r="N35">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O35">
+        <f t="shared" si="3"/>
         <v>1.42</v>
       </c>
     </row>
@@ -4539,12 +4528,12 @@
       <c r="M36">
         <v>0</v>
       </c>
-      <c r="N36" s="2">
-        <f>(M36+J36)*D36</f>
-        <v>0</v>
-      </c>
-      <c r="O36" s="2">
-        <f t="shared" si="1"/>
+      <c r="N36">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O36">
+        <f t="shared" si="3"/>
         <v>1.65</v>
       </c>
     </row>
@@ -4582,12 +4571,12 @@
       <c r="M37">
         <v>0</v>
       </c>
-      <c r="N37" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O37" s="2">
-        <f>D37+N37</f>
+      <c r="N37">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O37">
+        <f t="shared" si="3"/>
         <v>2.46</v>
       </c>
     </row>
@@ -4625,12 +4614,12 @@
       <c r="M38">
         <v>0</v>
       </c>
-      <c r="N38" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O38" s="2">
-        <f t="shared" si="1"/>
+      <c r="N38">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O38">
+        <f t="shared" si="3"/>
         <v>1.42</v>
       </c>
     </row>
@@ -4668,12 +4657,12 @@
       <c r="M39">
         <v>0</v>
       </c>
-      <c r="N39" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O39" s="2">
-        <f t="shared" si="1"/>
+      <c r="N39">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O39">
+        <f t="shared" si="3"/>
         <v>2.63</v>
       </c>
     </row>
@@ -4711,12 +4700,12 @@
       <c r="M40">
         <v>0</v>
       </c>
-      <c r="N40" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O40" s="2">
-        <f t="shared" si="1"/>
+      <c r="N40">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O40">
+        <f t="shared" si="3"/>
         <v>3.02</v>
       </c>
     </row>
@@ -4754,12 +4743,12 @@
       <c r="M41">
         <v>0</v>
       </c>
-      <c r="N41" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O41" s="2">
-        <f t="shared" si="1"/>
+      <c r="N41">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O41">
+        <f t="shared" si="3"/>
         <v>1.64</v>
       </c>
     </row>
@@ -4797,12 +4786,12 @@
       <c r="M42">
         <v>0</v>
       </c>
-      <c r="N42" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O42" s="2">
-        <f t="shared" si="1"/>
+      <c r="N42">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O42">
+        <f t="shared" si="3"/>
         <v>1.77</v>
       </c>
     </row>
@@ -4843,12 +4832,12 @@
       <c r="M43">
         <v>0</v>
       </c>
-      <c r="N43" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O43" s="2">
-        <f t="shared" si="1"/>
+      <c r="N43">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O43">
+        <f t="shared" si="3"/>
         <v>2.82</v>
       </c>
     </row>
@@ -4889,12 +4878,12 @@
       <c r="M44">
         <v>0</v>
       </c>
-      <c r="N44" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O44" s="2">
-        <f t="shared" si="1"/>
+      <c r="N44">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O44">
+        <f t="shared" si="3"/>
         <v>3.36</v>
       </c>
     </row>
@@ -4935,12 +4924,12 @@
       <c r="M45">
         <v>0</v>
       </c>
-      <c r="N45" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O45" s="2">
-        <f t="shared" si="1"/>
+      <c r="N45">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O45">
+        <f t="shared" si="3"/>
         <v>3.43</v>
       </c>
     </row>
@@ -4981,12 +4970,12 @@
       <c r="M46">
         <v>0</v>
       </c>
-      <c r="N46" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O46" s="2">
-        <f t="shared" si="1"/>
+      <c r="N46">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O46">
+        <f t="shared" si="3"/>
         <v>3.83</v>
       </c>
     </row>
@@ -5027,12 +5016,12 @@
       <c r="M47">
         <v>0</v>
       </c>
-      <c r="N47" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O47" s="2">
-        <f t="shared" si="1"/>
+      <c r="N47">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O47">
+        <f t="shared" si="3"/>
         <v>4.1399999999999997</v>
       </c>
     </row>
@@ -5073,12 +5062,12 @@
       <c r="M48">
         <v>0</v>
       </c>
-      <c r="N48" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O48" s="2">
-        <f t="shared" si="1"/>
+      <c r="N48">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O48">
+        <f t="shared" si="3"/>
         <v>4.8600000000000003</v>
       </c>
     </row>
@@ -5119,12 +5108,12 @@
       <c r="M49">
         <v>0</v>
       </c>
-      <c r="N49" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O49" s="2">
-        <f t="shared" si="1"/>
+      <c r="N49">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O49">
+        <f t="shared" si="3"/>
         <v>5.58</v>
       </c>
     </row>
@@ -5165,12 +5154,12 @@
       <c r="M50">
         <v>0</v>
       </c>
-      <c r="N50" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O50" s="2">
-        <f t="shared" si="1"/>
+      <c r="N50">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O50">
+        <f t="shared" si="3"/>
         <v>6.06</v>
       </c>
     </row>
@@ -5211,12 +5200,12 @@
       <c r="M51">
         <v>0</v>
       </c>
-      <c r="N51" s="2">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="O51" s="2">
-        <f t="shared" si="1"/>
+      <c r="N51">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="O51">
+        <f t="shared" si="3"/>
         <v>6.43</v>
       </c>
     </row>
@@ -5260,12 +5249,12 @@
       <c r="M52">
         <v>0</v>
       </c>
-      <c r="N52" s="2">
-        <f t="shared" si="0"/>
+      <c r="N52">
+        <f t="shared" si="2"/>
         <v>-0.70599999999999996</v>
       </c>
-      <c r="O52" s="2">
-        <f t="shared" si="1"/>
+      <c r="O52">
+        <f t="shared" si="3"/>
         <v>6.3539999999999992</v>
       </c>
     </row>
@@ -5309,18 +5298,18 @@
       <c r="M53">
         <v>0</v>
       </c>
-      <c r="N53" s="2">
-        <f t="shared" si="0"/>
+      <c r="N53">
+        <f t="shared" si="2"/>
         <v>-0.84399999999999997</v>
       </c>
-      <c r="O53" s="2">
-        <f t="shared" si="1"/>
+      <c r="O53">
+        <f t="shared" si="3"/>
         <v>7.5959999999999992</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
 
@@ -5338,7 +5327,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -5748,7 +5737,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="B26">
         <v>301</v>

</xml_diff>

<commit_message>
changed the 'gpu_name' column to 'gpu_unit_name'
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="tier_score_sheet" sheetId="1" r:id="rId1"/>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="117">
   <si>
-    <t>gpu_name</t>
-  </si>
-  <si>
     <t>performance</t>
   </si>
   <si>
@@ -376,6 +373,9 @@
   </si>
   <si>
     <t>Geforce RTX 3060</t>
+  </si>
+  <si>
+    <t>gpu_unit_name</t>
   </si>
 </sst>
 </file>
@@ -557,7 +557,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G53" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:G53"/>
   <tableColumns count="7">
-    <tableColumn id="1" name="gpu_name"/>
+    <tableColumn id="1" name="gpu_unit_name"/>
     <tableColumn id="2" name="performance" dataDxfId="1"/>
     <tableColumn id="3" name="base_tier_score">
       <calculatedColumnFormula>B2/100</calculatedColumnFormula>
@@ -881,45 +881,45 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="D1" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="U1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="U1" s="4" t="s">
+      <c r="V1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="W1" s="4" t="s">
+      <c r="X1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="X1" s="4" t="s">
+      <c r="Y1" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="Y1" s="4" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2">
         <v>121</v>
@@ -941,7 +941,7 @@
         <v>17500</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5"/>
@@ -955,7 +955,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3">
         <v>281</v>
@@ -965,10 +965,10 @@
         <v>2.81</v>
       </c>
       <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="U3" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="U3" s="5" t="s">
-        <v>16</v>
       </c>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
@@ -982,7 +982,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4">
         <v>301</v>
@@ -992,13 +992,13 @@
         <v>3.01</v>
       </c>
       <c r="E4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="U4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="V4" s="5" t="s">
         <v>18</v>
-      </c>
-      <c r="V4" s="5" t="s">
-        <v>19</v>
       </c>
       <c r="W4" s="5"/>
       <c r="X4" s="5">
@@ -1011,7 +1011,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>100</v>
@@ -1029,10 +1029,10 @@
         <v>17500</v>
       </c>
       <c r="U5" s="5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="V5" s="5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="W5" s="5"/>
       <c r="X5" s="5">
@@ -1045,7 +1045,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6">
         <v>160</v>
@@ -1063,7 +1063,7 @@
         <v>37500</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
@@ -1077,7 +1077,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7">
         <v>125</v>
@@ -1099,7 +1099,7 @@
         <v>18750</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
@@ -1113,7 +1113,7 @@
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B8">
         <v>139</v>
@@ -1135,7 +1135,7 @@
         <v>18750</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
@@ -1149,7 +1149,7 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9">
         <v>169</v>
@@ -1167,7 +1167,7 @@
         <v>20000</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
@@ -1181,7 +1181,7 @@
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B10">
         <v>187</v>
@@ -1199,10 +1199,10 @@
         <v>27500</v>
       </c>
       <c r="U10" t="s">
+        <v>25</v>
+      </c>
+      <c r="V10" t="s">
         <v>26</v>
-      </c>
-      <c r="V10" t="s">
-        <v>27</v>
       </c>
       <c r="X10">
         <v>300</v>
@@ -1214,7 +1214,7 @@
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B11">
         <v>210</v>
@@ -1232,10 +1232,10 @@
         <v>28750</v>
       </c>
       <c r="U11" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="V11" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="X11">
         <v>400</v>
@@ -1247,7 +1247,7 @@
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>215</v>
@@ -1265,10 +1265,10 @@
         <v>35000</v>
       </c>
       <c r="U12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="V12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="X12">
         <v>500</v>
@@ -1280,7 +1280,7 @@
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>253</v>
@@ -1302,10 +1302,10 @@
         <v>37500</v>
       </c>
       <c r="U13" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="V13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="X13">
         <v>500</v>
@@ -1317,7 +1317,7 @@
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>284</v>
@@ -1339,10 +1339,10 @@
         <v>50000</v>
       </c>
       <c r="U14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="V14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="X14">
         <v>700</v>
@@ -1354,7 +1354,7 @@
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B15">
         <v>295</v>
@@ -1371,10 +1371,10 @@
         <v>62500</v>
       </c>
       <c r="U15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="V15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="X15">
         <v>700</v>
@@ -1386,7 +1386,7 @@
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B16">
         <v>326</v>
@@ -1408,10 +1408,10 @@
         <v>62500</v>
       </c>
       <c r="U16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="V16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="X16">
         <v>1000</v>
@@ -1423,7 +1423,7 @@
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17">
         <v>350</v>
@@ -1445,10 +1445,10 @@
         <v>87500</v>
       </c>
       <c r="U17" t="s">
+        <v>37</v>
+      </c>
+      <c r="V17" t="s">
         <v>38</v>
-      </c>
-      <c r="V17" t="s">
-        <v>39</v>
       </c>
       <c r="X17">
         <v>250</v>
@@ -1460,7 +1460,7 @@
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18">
         <v>367</v>
@@ -1482,10 +1482,10 @@
         <v>87500</v>
       </c>
       <c r="U18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="V18" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X18">
         <v>330</v>
@@ -1497,7 +1497,7 @@
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B19">
         <v>413</v>
@@ -1519,10 +1519,10 @@
         <v>125000</v>
       </c>
       <c r="U19" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="V19" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X19">
         <v>330</v>
@@ -1534,7 +1534,7 @@
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B20">
         <v>218</v>
@@ -1556,10 +1556,10 @@
         <v>31250</v>
       </c>
       <c r="U20" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="V20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X20">
         <v>400</v>
@@ -1571,7 +1571,7 @@
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B21">
         <v>270</v>
@@ -1593,10 +1593,10 @@
         <v>41250</v>
       </c>
       <c r="U21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="V21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X21">
         <v>500</v>
@@ -1608,7 +1608,7 @@
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B22">
         <v>301</v>
@@ -1630,10 +1630,10 @@
         <v>41250</v>
       </c>
       <c r="U22" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="V22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X22">
         <v>600</v>
@@ -1645,7 +1645,7 @@
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B23">
         <v>376</v>
@@ -1667,10 +1667,10 @@
         <v>50000</v>
       </c>
       <c r="U23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X23">
         <v>700</v>
@@ -1682,7 +1682,7 @@
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B24">
         <v>441</v>
@@ -1704,10 +1704,10 @@
         <v>62500</v>
       </c>
       <c r="U24" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="V24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X24">
         <v>800</v>
@@ -1719,7 +1719,7 @@
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B25">
         <v>472</v>
@@ -1741,10 +1741,10 @@
         <v>75000</v>
       </c>
       <c r="U25" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="V25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X25">
         <v>1200</v>
@@ -1756,7 +1756,7 @@
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B26">
         <v>546</v>
@@ -1778,10 +1778,10 @@
         <v>87500</v>
       </c>
       <c r="U26" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="V26" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X26">
         <v>1500</v>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B27">
         <v>573</v>
@@ -1815,10 +1815,10 @@
         <v>100000</v>
       </c>
       <c r="U27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="V27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="X27">
         <v>2000</v>
@@ -1830,7 +1830,7 @@
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B28">
         <v>642</v>
@@ -1852,10 +1852,10 @@
         <v>150000</v>
       </c>
       <c r="U28" t="s">
+        <v>50</v>
+      </c>
+      <c r="V28" t="s">
         <v>51</v>
-      </c>
-      <c r="V28" t="s">
-        <v>52</v>
       </c>
       <c r="X28">
         <v>800</v>
@@ -1867,7 +1867,7 @@
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B29">
         <v>648</v>
@@ -1881,7 +1881,7 @@
         <v>rt_2 dlss_2</v>
       </c>
       <c r="E29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F29">
         <f t="shared" si="5"/>
@@ -1892,10 +1892,10 @@
         <v>187500</v>
       </c>
       <c r="U29" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="X29">
         <v>1200</v>
@@ -1907,7 +1907,7 @@
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B30">
         <v>700</v>
@@ -1921,7 +1921,7 @@
         <v>rt_2 dlss_2</v>
       </c>
       <c r="E30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F30">
         <f t="shared" si="5"/>
@@ -1932,10 +1932,10 @@
         <v>250000</v>
       </c>
       <c r="U30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="V30" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="X30">
         <v>1600</v>
@@ -1947,7 +1947,7 @@
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B31">
         <v>811</v>
@@ -1961,7 +1961,7 @@
         <v>rt_3 dlss_2 dlss_3</v>
       </c>
       <c r="E31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F31">
         <f t="shared" si="5"/>
@@ -1972,7 +1972,7 @@
         <v>150000</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="V31" s="5"/>
       <c r="W31" s="5"/>
@@ -1986,7 +1986,7 @@
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B32">
         <v>1014</v>
@@ -2000,7 +2000,7 @@
         <v>rt_3 dlss_2 dlss_3</v>
       </c>
       <c r="E32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F32">
         <f t="shared" si="5"/>
@@ -2011,7 +2011,7 @@
         <v>200000</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="V32" s="5"/>
       <c r="W32" s="5"/>
@@ -2025,7 +2025,7 @@
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B33">
         <v>668</v>
@@ -2047,7 +2047,7 @@
         <v>100000</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="V33" s="5"/>
       <c r="W33" s="5"/>
@@ -2061,23 +2061,23 @@
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B34">
         <v>162</v>
       </c>
       <c r="C34">
-        <f t="shared" ref="C34:C65" si="6">B34/100</f>
+        <f t="shared" ref="C34:C53" si="6">B34/100</f>
         <v>1.62</v>
       </c>
       <c r="U34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B35">
         <v>142</v>
@@ -2095,7 +2095,7 @@
         <v>21250</v>
       </c>
       <c r="U35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="X35">
         <v>170</v>
@@ -2107,7 +2107,7 @@
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B36">
         <v>165</v>
@@ -2125,7 +2125,7 @@
         <v>25000</v>
       </c>
       <c r="U36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="X36">
         <v>200</v>
@@ -2137,7 +2137,7 @@
     </row>
     <row r="37" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B37">
         <v>246</v>
@@ -2155,13 +2155,13 @@
         <v>35000</v>
       </c>
       <c r="U37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Y37" s="7"/>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B38">
         <v>142</v>
@@ -2179,7 +2179,7 @@
         <v>21250</v>
       </c>
       <c r="U38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="X38">
         <v>280</v>
@@ -2191,7 +2191,7 @@
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B39">
         <v>263</v>
@@ -2209,7 +2209,7 @@
         <v>43750</v>
       </c>
       <c r="U39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="X39">
         <v>350</v>
@@ -2221,7 +2221,7 @@
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B40">
         <v>302</v>
@@ -2239,7 +2239,7 @@
         <v>50000</v>
       </c>
       <c r="U40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="X40">
         <v>400</v>
@@ -2251,7 +2251,7 @@
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B41">
         <v>164</v>
@@ -2269,10 +2269,10 @@
         <v>28750</v>
       </c>
       <c r="U41" t="s">
+        <v>65</v>
+      </c>
+      <c r="V41" t="s">
         <v>66</v>
-      </c>
-      <c r="V41" t="s">
-        <v>67</v>
       </c>
       <c r="X41">
         <v>330</v>
@@ -2284,7 +2284,7 @@
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B42">
         <v>177</v>
@@ -2302,10 +2302,10 @@
         <v>35000</v>
       </c>
       <c r="U42" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="V42" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X42">
         <v>380</v>
@@ -2317,7 +2317,7 @@
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B43">
         <v>282</v>
@@ -2327,7 +2327,7 @@
         <v>2.82</v>
       </c>
       <c r="D43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F43">
         <v>330</v>
@@ -2337,10 +2337,10 @@
         <v>41250</v>
       </c>
       <c r="U43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="V43" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X43">
         <v>400</v>
@@ -2352,7 +2352,7 @@
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B44">
         <v>336</v>
@@ -2374,13 +2374,13 @@
         <v>47500</v>
       </c>
       <c r="U44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="Y44" s="7"/>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B45">
         <v>343</v>
@@ -2402,10 +2402,10 @@
         <v>50000</v>
       </c>
       <c r="U45" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="V45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X45">
         <v>480</v>
@@ -2417,7 +2417,7 @@
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B46">
         <v>383</v>
@@ -2439,10 +2439,10 @@
         <v>60000</v>
       </c>
       <c r="U46" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="V46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X46">
         <v>550</v>
@@ -2454,7 +2454,7 @@
     </row>
     <row r="47" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B47">
         <v>414</v>
@@ -2476,10 +2476,10 @@
         <v>68750</v>
       </c>
       <c r="U47" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="V47" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X47">
         <v>580</v>
@@ -2491,7 +2491,7 @@
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B48">
         <v>486</v>
@@ -2513,10 +2513,10 @@
         <v>72500</v>
       </c>
       <c r="U48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="V48" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X48">
         <v>650</v>
@@ -2528,7 +2528,7 @@
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B49">
         <v>558</v>
@@ -2550,10 +2550,10 @@
         <v>81250</v>
       </c>
       <c r="U49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="V49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X49">
         <v>1000</v>
@@ -2565,7 +2565,7 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B50">
         <v>606</v>
@@ -2587,10 +2587,10 @@
         <v>125000</v>
       </c>
       <c r="U50" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="V50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="X50">
         <v>1100</v>
@@ -2602,7 +2602,7 @@
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B51">
         <v>643</v>
@@ -2624,10 +2624,10 @@
         <v>137500</v>
       </c>
       <c r="U51" t="s">
+        <v>78</v>
+      </c>
+      <c r="V51" t="s">
         <v>79</v>
-      </c>
-      <c r="V51" t="s">
-        <v>80</v>
       </c>
       <c r="X51">
         <v>900</v>
@@ -2639,7 +2639,7 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B52">
         <v>706</v>
@@ -2653,7 +2653,7 @@
         <v xml:space="preserve">rt_2  </v>
       </c>
       <c r="E52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F52">
         <f t="shared" si="11"/>
@@ -2664,10 +2664,10 @@
         <v>112500</v>
       </c>
       <c r="U52" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="V52" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="X52">
         <v>1000</v>
@@ -2679,7 +2679,7 @@
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B53">
         <v>844</v>
@@ -2693,7 +2693,7 @@
         <v xml:space="preserve">rt_2  </v>
       </c>
       <c r="E53" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F53">
         <f t="shared" si="11"/>
@@ -2704,15 +2704,15 @@
         <v>125000</v>
       </c>
       <c r="U53" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U54" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="W54" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="X54">
         <v>140</v>
@@ -2724,22 +2724,22 @@
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U55" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U56" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U57" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U58" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2763,21 +2763,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>88</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -2785,10 +2785,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B3" t="s">
         <v>91</v>
-      </c>
-      <c r="B3" t="s">
-        <v>92</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -2796,10 +2796,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" t="s">
         <v>93</v>
-      </c>
-      <c r="B4" t="s">
-        <v>94</v>
       </c>
       <c r="C4">
         <v>15</v>
@@ -2807,10 +2807,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>94</v>
+      </c>
+      <c r="B5" t="s">
         <v>95</v>
-      </c>
-      <c r="B5" t="s">
-        <v>96</v>
       </c>
       <c r="C5">
         <v>7</v>
@@ -2818,10 +2818,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>96</v>
+      </c>
+      <c r="B6" t="s">
         <v>97</v>
-      </c>
-      <c r="B6" t="s">
-        <v>98</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -2829,10 +2829,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>98</v>
+      </c>
+      <c r="B7" t="s">
         <v>99</v>
-      </c>
-      <c r="B7" t="s">
-        <v>100</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -2840,10 +2840,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8">
         <v>-10</v>
@@ -2851,10 +2851,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C9">
         <v>-5</v>
@@ -2862,10 +2862,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B10" t="s">
         <v>103</v>
-      </c>
-      <c r="B10" t="s">
-        <v>104</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -2873,10 +2873,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C11">
         <v>-5</v>
@@ -2884,10 +2884,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>105</v>
+      </c>
+      <c r="B12" t="s">
         <v>106</v>
-      </c>
-      <c r="B12" t="s">
-        <v>107</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -2921,46 +2921,46 @@
   <sheetData>
     <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B1" s="4" t="s">
-        <v>0</v>
+        <v>116</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>6</v>
-      </c>
       <c r="I1" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="J1" s="4" t="s">
         <v>108</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="K1" s="4" t="s">
         <v>109</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="L1" s="4" t="s">
         <v>110</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="M1" s="4" t="s">
         <v>111</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="O1" s="4" t="s">
         <v>113</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
@@ -2968,7 +2968,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>121</v>
@@ -2977,7 +2977,7 @@
         <v>1.21</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G2">
         <v>140</v>
@@ -3014,7 +3014,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>281</v>
@@ -3023,7 +3023,7 @@
         <v>2.81</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -3054,7 +3054,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4">
         <v>301</v>
@@ -3063,7 +3063,7 @@
         <v>3.01</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -3094,7 +3094,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -3137,7 +3137,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C6">
         <v>160</v>
@@ -3180,7 +3180,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C7">
         <v>125</v>
@@ -3189,7 +3189,7 @@
         <v>1.25</v>
       </c>
       <c r="E7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7">
         <v>150</v>
@@ -3226,7 +3226,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8">
         <v>139</v>
@@ -3235,7 +3235,7 @@
         <v>1.39</v>
       </c>
       <c r="E8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G8">
         <v>150</v>
@@ -3272,7 +3272,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9">
         <v>169</v>
@@ -3315,7 +3315,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C10">
         <v>187</v>
@@ -3358,7 +3358,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11">
         <v>210</v>
@@ -3401,7 +3401,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12">
         <v>215</v>
@@ -3444,7 +3444,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13">
         <v>253</v>
@@ -3453,7 +3453,7 @@
         <v>2.5299999999999998</v>
       </c>
       <c r="E13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G13">
         <v>300</v>
@@ -3490,7 +3490,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C14">
         <v>284</v>
@@ -3499,7 +3499,7 @@
         <v>2.84</v>
       </c>
       <c r="E14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G14">
         <v>400</v>
@@ -3536,7 +3536,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C15">
         <v>295</v>
@@ -3579,7 +3579,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C16">
         <v>326</v>
@@ -3588,7 +3588,7 @@
         <v>3.26</v>
       </c>
       <c r="E16" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G16">
         <v>500</v>
@@ -3625,7 +3625,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17">
         <v>350</v>
@@ -3634,7 +3634,7 @@
         <v>3.5</v>
       </c>
       <c r="E17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G17">
         <v>700</v>
@@ -3671,7 +3671,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C18">
         <v>367</v>
@@ -3680,7 +3680,7 @@
         <v>3.67</v>
       </c>
       <c r="E18" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G18">
         <v>700</v>
@@ -3717,7 +3717,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C19">
         <v>413</v>
@@ -3726,7 +3726,7 @@
         <v>4.13</v>
       </c>
       <c r="E19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G19">
         <v>1000</v>
@@ -3763,7 +3763,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C20">
         <v>218</v>
@@ -3772,7 +3772,7 @@
         <v>2.1800000000000002</v>
       </c>
       <c r="E20" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G20">
         <v>250</v>
@@ -3809,7 +3809,7 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C21">
         <v>270</v>
@@ -3818,7 +3818,7 @@
         <v>2.7</v>
       </c>
       <c r="E21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G21">
         <v>330</v>
@@ -3855,7 +3855,7 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C22">
         <v>301</v>
@@ -3864,7 +3864,7 @@
         <v>3.01</v>
       </c>
       <c r="E22" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G22">
         <v>330</v>
@@ -3901,7 +3901,7 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C23">
         <v>376</v>
@@ -3910,7 +3910,7 @@
         <v>3.76</v>
       </c>
       <c r="E23" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G23">
         <v>400</v>
@@ -3947,7 +3947,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C24">
         <v>441</v>
@@ -3956,7 +3956,7 @@
         <v>4.41</v>
       </c>
       <c r="E24" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G24">
         <v>500</v>
@@ -3993,7 +3993,7 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C25">
         <v>472</v>
@@ -4002,7 +4002,7 @@
         <v>4.72</v>
       </c>
       <c r="E25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G25">
         <v>600</v>
@@ -4039,7 +4039,7 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C26">
         <v>546</v>
@@ -4048,7 +4048,7 @@
         <v>5.46</v>
       </c>
       <c r="E26" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G26">
         <v>700</v>
@@ -4085,7 +4085,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C27">
         <v>573</v>
@@ -4094,7 +4094,7 @@
         <v>5.73</v>
       </c>
       <c r="E27" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G27">
         <v>800</v>
@@ -4131,7 +4131,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C28">
         <v>642</v>
@@ -4140,7 +4140,7 @@
         <v>6.42</v>
       </c>
       <c r="E28" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G28">
         <v>1200</v>
@@ -4177,7 +4177,7 @@
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29">
         <v>648</v>
@@ -4186,10 +4186,10 @@
         <v>6.48</v>
       </c>
       <c r="E29" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F29" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G29">
         <v>1500</v>
@@ -4226,7 +4226,7 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C30">
         <v>700</v>
@@ -4235,10 +4235,10 @@
         <v>7</v>
       </c>
       <c r="E30" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G30">
         <v>2000</v>
@@ -4275,7 +4275,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C31">
         <v>811</v>
@@ -4284,10 +4284,10 @@
         <v>8.11</v>
       </c>
       <c r="E31" t="s">
+        <v>51</v>
+      </c>
+      <c r="F31" t="s">
         <v>52</v>
-      </c>
-      <c r="F31" t="s">
-        <v>53</v>
       </c>
       <c r="G31">
         <v>1200</v>
@@ -4324,7 +4324,7 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C32">
         <v>1014</v>
@@ -4333,10 +4333,10 @@
         <v>10.14</v>
       </c>
       <c r="E32" t="s">
+        <v>51</v>
+      </c>
+      <c r="F32" t="s">
         <v>52</v>
-      </c>
-      <c r="F32" t="s">
-        <v>53</v>
       </c>
       <c r="G32">
         <v>1600</v>
@@ -4373,7 +4373,7 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C33">
         <v>668</v>
@@ -4382,7 +4382,7 @@
         <v>6.68</v>
       </c>
       <c r="E33" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G33">
         <v>800</v>
@@ -4419,7 +4419,7 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C34">
         <v>162</v>
@@ -4443,11 +4443,11 @@
         <v>0</v>
       </c>
       <c r="N34">
-        <f t="shared" ref="N34:N65" si="2">(M34+J34)*D34</f>
+        <f t="shared" ref="N34:N53" si="2">(M34+J34)*D34</f>
         <v>0</v>
       </c>
       <c r="O34">
-        <f t="shared" ref="O34:O65" si="3">D34+N34</f>
+        <f t="shared" ref="O34:O53" si="3">D34+N34</f>
         <v>1.62</v>
       </c>
     </row>
@@ -4456,7 +4456,7 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C35">
         <v>142</v>
@@ -4499,7 +4499,7 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C36">
         <v>165</v>
@@ -4542,7 +4542,7 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C37">
         <v>246</v>
@@ -4585,7 +4585,7 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C38">
         <v>142</v>
@@ -4628,7 +4628,7 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C39">
         <v>263</v>
@@ -4671,7 +4671,7 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C40">
         <v>302</v>
@@ -4714,7 +4714,7 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C41">
         <v>164</v>
@@ -4757,7 +4757,7 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C42">
         <v>177</v>
@@ -4800,7 +4800,7 @@
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C43">
         <v>282</v>
@@ -4809,7 +4809,7 @@
         <v>2.82</v>
       </c>
       <c r="E43" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G43">
         <v>330</v>
@@ -4846,7 +4846,7 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C44">
         <v>336</v>
@@ -4855,7 +4855,7 @@
         <v>3.36</v>
       </c>
       <c r="E44" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G44">
         <v>380</v>
@@ -4892,7 +4892,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C45">
         <v>343</v>
@@ -4901,7 +4901,7 @@
         <v>3.43</v>
       </c>
       <c r="E45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G45">
         <v>400</v>
@@ -4938,7 +4938,7 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C46">
         <v>383</v>
@@ -4947,7 +4947,7 @@
         <v>3.83</v>
       </c>
       <c r="E46" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G46">
         <v>480</v>
@@ -4984,7 +4984,7 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C47">
         <v>414</v>
@@ -4993,7 +4993,7 @@
         <v>4.1399999999999997</v>
       </c>
       <c r="E47" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G47">
         <v>550</v>
@@ -5030,7 +5030,7 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C48">
         <v>486</v>
@@ -5039,7 +5039,7 @@
         <v>4.8600000000000003</v>
       </c>
       <c r="E48" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G48">
         <v>580</v>
@@ -5076,7 +5076,7 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C49">
         <v>558</v>
@@ -5085,7 +5085,7 @@
         <v>5.58</v>
       </c>
       <c r="E49" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G49">
         <v>650</v>
@@ -5122,7 +5122,7 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C50">
         <v>606</v>
@@ -5131,7 +5131,7 @@
         <v>6.06</v>
       </c>
       <c r="E50" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G50">
         <v>1000</v>
@@ -5168,7 +5168,7 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C51">
         <v>643</v>
@@ -5177,7 +5177,7 @@
         <v>6.43</v>
       </c>
       <c r="E51" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G51">
         <v>1100</v>
@@ -5214,7 +5214,7 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C52">
         <v>706</v>
@@ -5223,10 +5223,10 @@
         <v>7.06</v>
       </c>
       <c r="E52" t="s">
+        <v>79</v>
+      </c>
+      <c r="F52" t="s">
         <v>80</v>
-      </c>
-      <c r="F52" t="s">
-        <v>81</v>
       </c>
       <c r="G52">
         <v>900</v>
@@ -5263,7 +5263,7 @@
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C53">
         <v>844</v>
@@ -5272,10 +5272,10 @@
         <v>8.44</v>
       </c>
       <c r="E53" t="s">
+        <v>79</v>
+      </c>
+      <c r="F53" t="s">
         <v>80</v>
-      </c>
-      <c r="F53" t="s">
-        <v>81</v>
       </c>
       <c r="G53">
         <v>1000</v>
@@ -5327,19 +5327,19 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -5347,7 +5347,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -5364,7 +5364,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3">
         <v>121</v>
@@ -5381,7 +5381,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>125</v>
@@ -5398,7 +5398,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5">
         <v>139</v>
@@ -5415,7 +5415,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B6">
         <v>142</v>
@@ -5432,7 +5432,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7">
         <v>142</v>
@@ -5449,7 +5449,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>160</v>
@@ -5466,7 +5466,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B9">
         <v>162</v>
@@ -5477,7 +5477,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B10">
         <v>164</v>
@@ -5494,7 +5494,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B11">
         <v>165</v>
@@ -5511,7 +5511,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B12">
         <v>169</v>
@@ -5528,7 +5528,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B13">
         <v>177</v>
@@ -5545,7 +5545,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B14">
         <v>187</v>
@@ -5562,7 +5562,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15">
         <v>210</v>
@@ -5579,7 +5579,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B16">
         <v>215</v>
@@ -5596,7 +5596,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B17">
         <v>218</v>
@@ -5613,7 +5613,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B18">
         <v>246</v>
@@ -5630,7 +5630,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19">
         <v>253</v>
@@ -5647,7 +5647,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B20">
         <v>263</v>
@@ -5664,7 +5664,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B21">
         <v>281</v>
@@ -5675,7 +5675,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B22">
         <v>282</v>
@@ -5692,7 +5692,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23">
         <v>284</v>
@@ -5709,7 +5709,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24">
         <v>295</v>
@@ -5726,7 +5726,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B25">
         <v>301</v>
@@ -5737,7 +5737,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B26">
         <v>301</v>
@@ -5754,7 +5754,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B27">
         <v>302</v>
@@ -5771,7 +5771,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B28">
         <v>326</v>
@@ -5788,7 +5788,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B29">
         <v>336</v>
@@ -5805,7 +5805,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B30">
         <v>343</v>
@@ -5822,7 +5822,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B31">
         <v>350</v>
@@ -5839,7 +5839,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B32">
         <v>367</v>
@@ -5856,7 +5856,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B33">
         <v>376</v>
@@ -5873,7 +5873,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B34">
         <v>383</v>
@@ -5890,7 +5890,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B35">
         <v>413</v>
@@ -5907,7 +5907,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B36">
         <v>414</v>
@@ -5924,7 +5924,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B37">
         <v>441</v>
@@ -5941,7 +5941,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B38">
         <v>472</v>
@@ -5958,7 +5958,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B39">
         <v>486</v>
@@ -5975,7 +5975,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B40">
         <v>546</v>
@@ -5992,7 +5992,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B41">
         <v>558</v>
@@ -6009,7 +6009,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B42">
         <v>573</v>
@@ -6026,7 +6026,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B43">
         <v>606</v>
@@ -6043,7 +6043,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B44">
         <v>642</v>
@@ -6060,7 +6060,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B45">
         <v>643</v>
@@ -6077,7 +6077,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B46">
         <v>648</v>
@@ -6094,7 +6094,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B47">
         <v>700</v>
@@ -6111,7 +6111,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B48">
         <v>706</v>
@@ -6128,7 +6128,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B49">
         <v>811</v>
@@ -6145,7 +6145,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B50">
         <v>844</v>
@@ -6162,7 +6162,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B51">
         <v>1014</v>

</xml_diff>

<commit_message>
changed the SUPER to Super (only first letter cap) in overall_tier_scores sheet
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -3272,7 +3272,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C9">
         <v>169</v>
@@ -3358,7 +3358,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="C11">
         <v>210</v>
@@ -3490,7 +3490,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C14">
         <v>284</v>
@@ -3579,7 +3579,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="C16">
         <v>326</v>
@@ -3671,7 +3671,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C18">
         <v>367</v>

</xml_diff>

<commit_message>
feb 8 data & overall_tier_score correction data added for February 8, 2023 overall_tier_score had a slight issue preventing data_coll_script from reading it - now fixed
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -17,9 +17,6 @@
     <sheet name="overall_tier_scores" sheetId="3" r:id="rId3"/>
     <sheet name="tier_score_sheet_copy" sheetId="4" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="overall_tier_score" localSheetId="2">overall_tier_scores!$A$1:$M$53</definedName>
-  </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
@@ -27,6 +24,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="117">
   <si>
+    <t>gpu_unit_name</t>
+  </si>
+  <si>
     <t>performance</t>
   </si>
   <si>
@@ -373,9 +373,6 @@
   </si>
   <si>
     <t>Geforce RTX 3060</t>
-  </si>
-  <si>
-    <t>gpu_unit_name</t>
   </si>
 </sst>
 </file>
@@ -385,7 +382,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -426,6 +423,11 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -440,7 +442,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -474,13 +476,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -494,6 +511,9 @@
     <xf numFmtId="43" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -881,45 +901,45 @@
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F1" s="8" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U1" s="4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="V1" s="4" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Y1" s="4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>121</v>
@@ -941,7 +961,7 @@
         <v>17500</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="V2" s="5"/>
       <c r="W2" s="5"/>
@@ -955,7 +975,7 @@
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>281</v>
@@ -965,10 +985,10 @@
         <v>2.81</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U3" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="V3" s="5"/>
       <c r="W3" s="5"/>
@@ -982,7 +1002,7 @@
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4">
         <v>301</v>
@@ -992,13 +1012,13 @@
         <v>3.01</v>
       </c>
       <c r="E4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="U4" s="5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="V4" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="W4" s="5"/>
       <c r="X4" s="5">
@@ -1011,7 +1031,7 @@
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B5">
         <v>100</v>
@@ -1029,10 +1049,10 @@
         <v>17500</v>
       </c>
       <c r="U5" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="V5" s="5" t="s">
         <v>19</v>
-      </c>
-      <c r="V5" s="5" t="s">
-        <v>18</v>
       </c>
       <c r="W5" s="5"/>
       <c r="X5" s="5">
@@ -1045,7 +1065,7 @@
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6">
         <v>160</v>
@@ -1063,7 +1083,7 @@
         <v>37500</v>
       </c>
       <c r="U6" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="V6" s="5"/>
       <c r="W6" s="5"/>
@@ -1077,7 +1097,7 @@
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B7">
         <v>125</v>
@@ -1099,7 +1119,7 @@
         <v>18750</v>
       </c>
       <c r="U7" s="5" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="V7" s="5"/>
       <c r="W7" s="5"/>
@@ -1113,7 +1133,7 @@
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>139</v>
@@ -1135,7 +1155,7 @@
         <v>18750</v>
       </c>
       <c r="U8" s="5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="V8" s="5"/>
       <c r="W8" s="5"/>
@@ -1149,7 +1169,7 @@
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B9">
         <v>169</v>
@@ -1167,7 +1187,7 @@
         <v>20000</v>
       </c>
       <c r="U9" s="5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="V9" s="5"/>
       <c r="W9" s="5"/>
@@ -1181,7 +1201,7 @@
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>187</v>
@@ -1199,10 +1219,10 @@
         <v>27500</v>
       </c>
       <c r="U10" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="V10" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X10">
         <v>300</v>
@@ -1214,7 +1234,7 @@
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B11">
         <v>210</v>
@@ -1232,10 +1252,10 @@
         <v>28750</v>
       </c>
       <c r="U11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="V11" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X11">
         <v>400</v>
@@ -1247,7 +1267,7 @@
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B12">
         <v>215</v>
@@ -1265,10 +1285,10 @@
         <v>35000</v>
       </c>
       <c r="U12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="V12" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X12">
         <v>500</v>
@@ -1280,7 +1300,7 @@
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B13">
         <v>253</v>
@@ -1302,10 +1322,10 @@
         <v>37500</v>
       </c>
       <c r="U13" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="V13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X13">
         <v>500</v>
@@ -1317,7 +1337,7 @@
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B14">
         <v>284</v>
@@ -1339,10 +1359,10 @@
         <v>50000</v>
       </c>
       <c r="U14" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="V14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X14">
         <v>700</v>
@@ -1354,7 +1374,7 @@
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15">
         <v>295</v>
@@ -1371,10 +1391,10 @@
         <v>62500</v>
       </c>
       <c r="U15" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X15">
         <v>700</v>
@@ -1386,7 +1406,7 @@
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B16">
         <v>326</v>
@@ -1408,10 +1428,10 @@
         <v>62500</v>
       </c>
       <c r="U16" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="V16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="X16">
         <v>1000</v>
@@ -1423,7 +1443,7 @@
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>350</v>
@@ -1445,10 +1465,10 @@
         <v>87500</v>
       </c>
       <c r="U17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="V17" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X17">
         <v>250</v>
@@ -1460,7 +1480,7 @@
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B18">
         <v>367</v>
@@ -1482,10 +1502,10 @@
         <v>87500</v>
       </c>
       <c r="U18" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="V18" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X18">
         <v>330</v>
@@ -1497,7 +1517,7 @@
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B19">
         <v>413</v>
@@ -1519,10 +1539,10 @@
         <v>125000</v>
       </c>
       <c r="U19" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="V19" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X19">
         <v>330</v>
@@ -1534,7 +1554,7 @@
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B20">
         <v>218</v>
@@ -1556,10 +1576,10 @@
         <v>31250</v>
       </c>
       <c r="U20" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="V20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X20">
         <v>400</v>
@@ -1571,7 +1591,7 @@
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B21">
         <v>270</v>
@@ -1593,10 +1613,10 @@
         <v>41250</v>
       </c>
       <c r="U21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="V21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X21">
         <v>500</v>
@@ -1608,7 +1628,7 @@
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B22">
         <v>301</v>
@@ -1630,10 +1650,10 @@
         <v>41250</v>
       </c>
       <c r="U22" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X22">
         <v>600</v>
@@ -1645,7 +1665,7 @@
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B23">
         <v>376</v>
@@ -1667,10 +1687,10 @@
         <v>50000</v>
       </c>
       <c r="U23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="V23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X23">
         <v>700</v>
@@ -1682,7 +1702,7 @@
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B24">
         <v>441</v>
@@ -1704,10 +1724,10 @@
         <v>62500</v>
       </c>
       <c r="U24" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="V24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X24">
         <v>800</v>
@@ -1719,7 +1739,7 @@
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25">
         <v>472</v>
@@ -1741,10 +1761,10 @@
         <v>75000</v>
       </c>
       <c r="U25" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="V25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X25">
         <v>1200</v>
@@ -1756,7 +1776,7 @@
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B26">
         <v>546</v>
@@ -1778,10 +1798,10 @@
         <v>87500</v>
       </c>
       <c r="U26" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="V26" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X26">
         <v>1500</v>
@@ -1793,7 +1813,7 @@
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B27">
         <v>573</v>
@@ -1815,10 +1835,10 @@
         <v>100000</v>
       </c>
       <c r="U27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="V27" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="X27">
         <v>2000</v>
@@ -1830,7 +1850,7 @@
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B28">
         <v>642</v>
@@ -1852,10 +1872,10 @@
         <v>150000</v>
       </c>
       <c r="U28" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="V28" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X28">
         <v>800</v>
@@ -1867,7 +1887,7 @@
     </row>
     <row r="29" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B29">
         <v>648</v>
@@ -1881,7 +1901,7 @@
         <v>rt_2 dlss_2</v>
       </c>
       <c r="E29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F29">
         <f t="shared" si="5"/>
@@ -1892,10 +1912,10 @@
         <v>187500</v>
       </c>
       <c r="U29" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="V29" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X29">
         <v>1200</v>
@@ -1907,7 +1927,7 @@
     </row>
     <row r="30" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B30">
         <v>700</v>
@@ -1921,7 +1941,7 @@
         <v>rt_2 dlss_2</v>
       </c>
       <c r="E30" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F30">
         <f t="shared" si="5"/>
@@ -1932,10 +1952,10 @@
         <v>250000</v>
       </c>
       <c r="U30" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="V30" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="X30">
         <v>1600</v>
@@ -1947,7 +1967,7 @@
     </row>
     <row r="31" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B31">
         <v>811</v>
@@ -1961,7 +1981,7 @@
         <v>rt_3 dlss_2 dlss_3</v>
       </c>
       <c r="E31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F31">
         <f t="shared" si="5"/>
@@ -1972,7 +1992,7 @@
         <v>150000</v>
       </c>
       <c r="U31" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="V31" s="5"/>
       <c r="W31" s="5"/>
@@ -1986,7 +2006,7 @@
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B32">
         <v>1014</v>
@@ -2000,7 +2020,7 @@
         <v>rt_3 dlss_2 dlss_3</v>
       </c>
       <c r="E32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F32">
         <f t="shared" si="5"/>
@@ -2011,7 +2031,7 @@
         <v>200000</v>
       </c>
       <c r="U32" s="5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="V32" s="5"/>
       <c r="W32" s="5"/>
@@ -2025,7 +2045,7 @@
     </row>
     <row r="33" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B33">
         <v>668</v>
@@ -2047,7 +2067,7 @@
         <v>100000</v>
       </c>
       <c r="U33" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="V33" s="5"/>
       <c r="W33" s="5"/>
@@ -2061,23 +2081,23 @@
     </row>
     <row r="34" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B34">
         <v>162</v>
       </c>
       <c r="C34">
-        <f t="shared" ref="C34:C53" si="6">B34/100</f>
+        <f t="shared" ref="C34:C65" si="6">B34/100</f>
         <v>1.62</v>
       </c>
       <c r="U34" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="Y34" s="7"/>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B35">
         <v>142</v>
@@ -2095,7 +2115,7 @@
         <v>21250</v>
       </c>
       <c r="U35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="X35">
         <v>170</v>
@@ -2107,7 +2127,7 @@
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B36">
         <v>165</v>
@@ -2125,7 +2145,7 @@
         <v>25000</v>
       </c>
       <c r="U36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="X36">
         <v>200</v>
@@ -2137,7 +2157,7 @@
     </row>
     <row r="37" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B37">
         <v>246</v>
@@ -2155,13 +2175,13 @@
         <v>35000</v>
       </c>
       <c r="U37" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="Y37" s="7"/>
     </row>
     <row r="38" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B38">
         <v>142</v>
@@ -2179,7 +2199,7 @@
         <v>21250</v>
       </c>
       <c r="U38" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="X38">
         <v>280</v>
@@ -2191,7 +2211,7 @@
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B39">
         <v>263</v>
@@ -2209,7 +2229,7 @@
         <v>43750</v>
       </c>
       <c r="U39" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="X39">
         <v>350</v>
@@ -2221,7 +2241,7 @@
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B40">
         <v>302</v>
@@ -2239,7 +2259,7 @@
         <v>50000</v>
       </c>
       <c r="U40" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="X40">
         <v>400</v>
@@ -2251,7 +2271,7 @@
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B41">
         <v>164</v>
@@ -2269,10 +2289,10 @@
         <v>28750</v>
       </c>
       <c r="U41" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="V41" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X41">
         <v>330</v>
@@ -2284,7 +2304,7 @@
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B42">
         <v>177</v>
@@ -2302,10 +2322,10 @@
         <v>35000</v>
       </c>
       <c r="U42" t="s">
+        <v>68</v>
+      </c>
+      <c r="V42" t="s">
         <v>67</v>
-      </c>
-      <c r="V42" t="s">
-        <v>66</v>
       </c>
       <c r="X42">
         <v>380</v>
@@ -2317,7 +2337,7 @@
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B43">
         <v>282</v>
@@ -2327,7 +2347,7 @@
         <v>2.82</v>
       </c>
       <c r="D43" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F43">
         <v>330</v>
@@ -2337,10 +2357,10 @@
         <v>41250</v>
       </c>
       <c r="U43" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="V43" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X43">
         <v>400</v>
@@ -2352,7 +2372,7 @@
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B44">
         <v>336</v>
@@ -2374,13 +2394,13 @@
         <v>47500</v>
       </c>
       <c r="U44" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="Y44" s="7"/>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B45">
         <v>343</v>
@@ -2402,10 +2422,10 @@
         <v>50000</v>
       </c>
       <c r="U45" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="V45" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X45">
         <v>480</v>
@@ -2417,7 +2437,7 @@
     </row>
     <row r="46" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B46">
         <v>383</v>
@@ -2439,10 +2459,10 @@
         <v>60000</v>
       </c>
       <c r="U46" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="V46" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X46">
         <v>550</v>
@@ -2454,7 +2474,7 @@
     </row>
     <row r="47" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B47">
         <v>414</v>
@@ -2476,10 +2496,10 @@
         <v>68750</v>
       </c>
       <c r="U47" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="V47" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X47">
         <v>580</v>
@@ -2491,7 +2511,7 @@
     </row>
     <row r="48" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B48">
         <v>486</v>
@@ -2513,10 +2533,10 @@
         <v>72500</v>
       </c>
       <c r="U48" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="V48" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X48">
         <v>650</v>
@@ -2528,7 +2548,7 @@
     </row>
     <row r="49" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B49">
         <v>558</v>
@@ -2550,10 +2570,10 @@
         <v>81250</v>
       </c>
       <c r="U49" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="V49" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X49">
         <v>1000</v>
@@ -2565,7 +2585,7 @@
     </row>
     <row r="50" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B50">
         <v>606</v>
@@ -2587,10 +2607,10 @@
         <v>125000</v>
       </c>
       <c r="U50" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="V50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="X50">
         <v>1100</v>
@@ -2602,7 +2622,7 @@
     </row>
     <row r="51" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B51">
         <v>643</v>
@@ -2624,10 +2644,10 @@
         <v>137500</v>
       </c>
       <c r="U51" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="V51" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="X51">
         <v>900</v>
@@ -2639,7 +2659,7 @@
     </row>
     <row r="52" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B52">
         <v>706</v>
@@ -2653,7 +2673,7 @@
         <v xml:space="preserve">rt_2  </v>
       </c>
       <c r="E52" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F52">
         <f t="shared" si="11"/>
@@ -2664,10 +2684,10 @@
         <v>112500</v>
       </c>
       <c r="U52" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="V52" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="X52">
         <v>1000</v>
@@ -2679,7 +2699,7 @@
     </row>
     <row r="53" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B53">
         <v>844</v>
@@ -2693,7 +2713,7 @@
         <v xml:space="preserve">rt_2  </v>
       </c>
       <c r="E53" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="F53">
         <f t="shared" si="11"/>
@@ -2704,15 +2724,15 @@
         <v>125000</v>
       </c>
       <c r="U53" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U54" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="W54" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="X54">
         <v>140</v>
@@ -2724,22 +2744,22 @@
     </row>
     <row r="55" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U55" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="56" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U56" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="57" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U57" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="58" spans="1:25" x14ac:dyDescent="0.25">
       <c r="U58" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -2763,21 +2783,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -2785,10 +2805,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -2796,10 +2816,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C4">
         <v>15</v>
@@ -2807,10 +2827,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C5">
         <v>7</v>
@@ -2818,10 +2838,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -2829,10 +2849,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -2840,10 +2860,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C8">
         <v>-10</v>
@@ -2851,10 +2871,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C9">
         <v>-5</v>
@@ -2862,10 +2882,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -2873,10 +2893,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C11">
         <v>-5</v>
@@ -2884,10 +2904,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -2903,72 +2923,63 @@
   <dimension ref="A1:O53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="31.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="15" width="16.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.42578125" customWidth="1"/>
+    <col min="15" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" s="4" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="D1" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="E1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="F1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="G1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="J1" s="4" t="s">
+      <c r="H1" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="I1" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="K1" s="4" t="s">
+      <c r="J1" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="K1" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="L1" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="M1" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="O1" s="4" t="s">
+      <c r="N1" s="9" t="s">
         <v>113</v>
       </c>
+      <c r="O1" s="9" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2">
+      <c r="A2" s="9">
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C2">
         <v>121</v>
@@ -2977,7 +2988,7 @@
         <v>1.21</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2">
         <v>140</v>
@@ -3001,20 +3012,18 @@
         <v>0</v>
       </c>
       <c r="N2">
-        <f t="shared" ref="N2:N33" si="0">(M2+J2)*D2</f>
         <v>-0.121</v>
       </c>
       <c r="O2">
-        <f t="shared" ref="O2:O33" si="1">D2+N2</f>
         <v>1.089</v>
       </c>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C3">
         <v>281</v>
@@ -3023,7 +3032,7 @@
         <v>2.81</v>
       </c>
       <c r="F3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I3">
         <v>0</v>
@@ -3041,20 +3050,18 @@
         <v>0</v>
       </c>
       <c r="N3">
-        <f t="shared" si="0"/>
         <v>-0.28100000000000003</v>
       </c>
       <c r="O3">
-        <f t="shared" si="1"/>
         <v>2.5289999999999999</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4">
+      <c r="A4" s="9">
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>301</v>
@@ -3063,7 +3070,7 @@
         <v>3.01</v>
       </c>
       <c r="F4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I4">
         <v>0</v>
@@ -3075,26 +3082,24 @@
         <v>-0.30099999999999999</v>
       </c>
       <c r="L4">
-        <v>2.7089999999999899</v>
+        <v>2.7090000000000001</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <f t="shared" si="0"/>
         <v>-0.30099999999999999</v>
       </c>
       <c r="O4">
-        <f t="shared" si="1"/>
-        <v>2.7089999999999996</v>
+        <v>2.7090000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5">
+      <c r="A5" s="9">
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -3124,20 +3129,18 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O5">
-        <f t="shared" si="1"/>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6">
+      <c r="A6" s="9">
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6">
         <v>160</v>
@@ -3167,20 +3170,18 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O6">
-        <f t="shared" si="1"/>
         <v>1.6</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="9">
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C7">
         <v>125</v>
@@ -3189,7 +3190,7 @@
         <v>1.25</v>
       </c>
       <c r="E7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G7">
         <v>150</v>
@@ -3213,20 +3214,18 @@
         <v>0.05</v>
       </c>
       <c r="N7">
-        <f t="shared" si="0"/>
         <v>6.25E-2</v>
       </c>
       <c r="O7">
-        <f t="shared" si="1"/>
         <v>1.3125</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8">
+      <c r="A8" s="9">
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C8">
         <v>139</v>
@@ -3235,7 +3234,7 @@
         <v>1.39</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G8">
         <v>150</v>
@@ -3250,29 +3249,27 @@
         <v>0</v>
       </c>
       <c r="K8">
-        <v>6.9499999999999895E-2</v>
+        <v>6.9499999999999992E-2</v>
       </c>
       <c r="L8">
-        <v>1.45949999999999</v>
+        <v>1.4595</v>
       </c>
       <c r="M8">
         <v>0.05</v>
       </c>
       <c r="N8">
-        <f t="shared" si="0"/>
         <v>6.9499999999999992E-2</v>
       </c>
       <c r="O8">
-        <f t="shared" si="1"/>
-        <v>1.4594999999999998</v>
+        <v>1.4595</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9">
+      <c r="A9" s="9">
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C9">
         <v>169</v>
@@ -3302,20 +3299,18 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O9">
-        <f t="shared" si="1"/>
         <v>1.69</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A10">
+      <c r="A10" s="9">
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C10">
         <v>187</v>
@@ -3345,20 +3340,18 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O10">
-        <f t="shared" si="1"/>
         <v>1.87</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11">
+      <c r="A11" s="9">
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C11">
         <v>210</v>
@@ -3388,20 +3381,18 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O11">
-        <f t="shared" si="1"/>
         <v>2.1</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12">
+      <c r="A12" s="9">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12">
         <v>215</v>
@@ -3431,20 +3422,18 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O12">
-        <f t="shared" si="1"/>
         <v>2.15</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13">
+      <c r="A13" s="9">
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C13">
         <v>253</v>
@@ -3453,7 +3442,7 @@
         <v>2.5299999999999998</v>
       </c>
       <c r="E13" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G13">
         <v>300</v>
@@ -3471,26 +3460,24 @@
         <v>0.30359999999999998</v>
       </c>
       <c r="L13">
-        <v>2.8335999999999899</v>
+        <v>2.8336000000000001</v>
       </c>
       <c r="M13">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N13">
-        <f t="shared" si="0"/>
         <v>0.17710000000000001</v>
       </c>
       <c r="O13">
-        <f t="shared" si="1"/>
-        <v>2.7070999999999996</v>
+        <v>2.7071000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14">
+      <c r="A14" s="9">
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C14">
         <v>284</v>
@@ -3499,7 +3486,7 @@
         <v>2.84</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G14">
         <v>400</v>
@@ -3517,26 +3504,24 @@
         <v>0.34079999999999999</v>
       </c>
       <c r="L14">
-        <v>3.1807999999999899</v>
+        <v>3.1808000000000001</v>
       </c>
       <c r="M14">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N14">
-        <f t="shared" si="0"/>
         <v>0.1988</v>
       </c>
       <c r="O14">
-        <f t="shared" si="1"/>
-        <v>3.0387999999999997</v>
+        <v>3.0388000000000002</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15">
+      <c r="A15" s="9">
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C15">
         <v>295</v>
@@ -3566,20 +3551,18 @@
         <v>0</v>
       </c>
       <c r="N15">
-        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="O15">
-        <f t="shared" si="1"/>
         <v>2.95</v>
       </c>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16">
+      <c r="A16" s="9">
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C16">
         <v>326</v>
@@ -3588,7 +3571,7 @@
         <v>3.26</v>
       </c>
       <c r="E16" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G16">
         <v>500</v>
@@ -3603,7 +3586,7 @@
         <v>0</v>
       </c>
       <c r="K16">
-        <v>0.39119999999999899</v>
+        <v>0.39119999999999988</v>
       </c>
       <c r="L16">
         <v>3.6511999999999998</v>
@@ -3612,20 +3595,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N16">
-        <f t="shared" si="0"/>
-        <v>0.22820000000000001</v>
+        <v>0.22819999999999999</v>
       </c>
       <c r="O16">
-        <f t="shared" si="1"/>
         <v>3.4882</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17">
+      <c r="A17" s="9">
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C17">
         <v>350</v>
@@ -3634,7 +3615,7 @@
         <v>3.5</v>
       </c>
       <c r="E17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G17">
         <v>700</v>
@@ -3658,20 +3639,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N17">
-        <f t="shared" si="0"/>
-        <v>0.24500000000000002</v>
+        <v>0.245</v>
       </c>
       <c r="O17">
-        <f t="shared" si="1"/>
         <v>3.7450000000000001</v>
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18">
+      <c r="A18" s="9">
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="C18">
         <v>367</v>
@@ -3680,7 +3659,7 @@
         <v>3.67</v>
       </c>
       <c r="E18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G18">
         <v>700</v>
@@ -3695,7 +3674,7 @@
         <v>0</v>
       </c>
       <c r="K18">
-        <v>0.44039999999999901</v>
+        <v>0.44040000000000001</v>
       </c>
       <c r="L18">
         <v>4.1104000000000003</v>
@@ -3704,20 +3683,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N18">
-        <f t="shared" si="0"/>
         <v>0.25690000000000002</v>
       </c>
       <c r="O18">
-        <f t="shared" si="1"/>
         <v>3.9268999999999998</v>
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A19">
+      <c r="A19" s="9">
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C19">
         <v>413</v>
@@ -3726,7 +3703,7 @@
         <v>4.13</v>
       </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G19">
         <v>1000</v>
@@ -3744,26 +3721,24 @@
         <v>0.49559999999999998</v>
       </c>
       <c r="L19">
-        <v>4.6255999999999897</v>
+        <v>4.6255999999999986</v>
       </c>
       <c r="M19">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N19">
-        <f t="shared" si="0"/>
         <v>0.28910000000000002</v>
       </c>
       <c r="O19">
-        <f t="shared" si="1"/>
         <v>4.4191000000000003</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20">
+      <c r="A20" s="9">
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C20">
         <v>218</v>
@@ -3772,7 +3747,7 @@
         <v>2.1800000000000002</v>
       </c>
       <c r="E20" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G20">
         <v>250</v>
@@ -3796,20 +3771,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N20">
-        <f t="shared" si="0"/>
         <v>0.15260000000000001</v>
       </c>
       <c r="O20">
-        <f t="shared" si="1"/>
-        <v>2.3326000000000002</v>
+        <v>2.3325999999999998</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21">
+      <c r="A21" s="9">
         <v>19</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C21">
         <v>270</v>
@@ -3818,7 +3791,7 @@
         <v>2.7</v>
       </c>
       <c r="E21" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G21">
         <v>330</v>
@@ -3833,7 +3806,7 @@
         <v>0</v>
       </c>
       <c r="K21">
-        <v>0.45900000000000002</v>
+        <v>0.45900000000000007</v>
       </c>
       <c r="L21">
         <v>3.1589999999999998</v>
@@ -3842,20 +3815,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N21">
-        <f t="shared" si="0"/>
-        <v>0.18900000000000003</v>
+        <v>0.189</v>
       </c>
       <c r="O21">
-        <f t="shared" si="1"/>
-        <v>2.8890000000000002</v>
+        <v>2.8889999999999998</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22">
+      <c r="A22" s="9">
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C22">
         <v>301</v>
@@ -3864,7 +3835,7 @@
         <v>3.01</v>
       </c>
       <c r="E22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G22">
         <v>330</v>
@@ -3888,20 +3859,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N22">
-        <f t="shared" si="0"/>
         <v>0.2107</v>
       </c>
       <c r="O22">
-        <f t="shared" si="1"/>
         <v>3.2206999999999999</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23">
+      <c r="A23" s="9">
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C23">
         <v>376</v>
@@ -3910,7 +3879,7 @@
         <v>3.76</v>
       </c>
       <c r="E23" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G23">
         <v>400</v>
@@ -3928,26 +3897,24 @@
         <v>0.63919999999999999</v>
       </c>
       <c r="L23">
-        <v>4.3991999999999898</v>
+        <v>4.3992000000000004</v>
       </c>
       <c r="M23">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N23">
-        <f t="shared" si="0"/>
         <v>0.26319999999999999</v>
       </c>
       <c r="O23">
-        <f t="shared" si="1"/>
         <v>4.0232000000000001</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24">
+      <c r="A24" s="9">
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C24">
         <v>441</v>
@@ -3956,7 +3923,7 @@
         <v>4.41</v>
       </c>
       <c r="E24" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G24">
         <v>500</v>
@@ -3980,20 +3947,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N24">
-        <f t="shared" si="0"/>
-        <v>0.30870000000000003</v>
+        <v>0.30869999999999997</v>
       </c>
       <c r="O24">
-        <f t="shared" si="1"/>
         <v>4.7187000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25">
+      <c r="A25" s="9">
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C25">
         <v>472</v>
@@ -4002,7 +3967,7 @@
         <v>4.72</v>
       </c>
       <c r="E25" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G25">
         <v>600</v>
@@ -4020,26 +3985,24 @@
         <v>0.8024</v>
       </c>
       <c r="L25">
-        <v>5.5223999999999904</v>
+        <v>5.5223999999999993</v>
       </c>
       <c r="M25">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N25">
-        <f t="shared" si="0"/>
         <v>0.33040000000000003</v>
       </c>
       <c r="O25">
-        <f t="shared" si="1"/>
         <v>5.0503999999999998</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26">
+      <c r="A26" s="9">
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C26">
         <v>546</v>
@@ -4048,7 +4011,7 @@
         <v>5.46</v>
       </c>
       <c r="E26" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G26">
         <v>700</v>
@@ -4072,20 +4035,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N26">
-        <f t="shared" si="0"/>
-        <v>0.38220000000000004</v>
+        <v>0.38219999999999998</v>
       </c>
       <c r="O26">
-        <f t="shared" si="1"/>
         <v>5.8422000000000001</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27">
+      <c r="A27" s="9">
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C27">
         <v>573</v>
@@ -4094,7 +4055,7 @@
         <v>5.73</v>
       </c>
       <c r="E27" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G27">
         <v>800</v>
@@ -4109,7 +4070,7 @@
         <v>0</v>
       </c>
       <c r="K27">
-        <v>0.97409999999999997</v>
+        <v>0.97410000000000019</v>
       </c>
       <c r="L27">
         <v>6.7041000000000004</v>
@@ -4118,20 +4079,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N27">
-        <f t="shared" si="0"/>
-        <v>0.40110000000000007</v>
+        <v>0.40110000000000012</v>
       </c>
       <c r="O27">
-        <f t="shared" si="1"/>
         <v>6.1311000000000009</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28">
+      <c r="A28" s="9">
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C28">
         <v>642</v>
@@ -4140,7 +4099,7 @@
         <v>6.42</v>
       </c>
       <c r="E28" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G28">
         <v>1200</v>
@@ -4164,20 +4123,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N28">
-        <f t="shared" si="0"/>
         <v>0.44940000000000002</v>
       </c>
       <c r="O28">
-        <f t="shared" si="1"/>
         <v>6.8693999999999997</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29">
+      <c r="A29" s="9">
         <v>27</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C29">
         <v>648</v>
@@ -4186,10 +4143,10 @@
         <v>6.48</v>
       </c>
       <c r="E29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F29" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G29">
         <v>1500</v>
@@ -4204,7 +4161,7 @@
         <v>-0.05</v>
       </c>
       <c r="K29">
-        <v>0.77759999999999996</v>
+        <v>0.77760000000000007</v>
       </c>
       <c r="L29">
         <v>7.2576000000000001</v>
@@ -4213,20 +4170,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N29">
-        <f t="shared" si="0"/>
-        <v>0.12960000000000002</v>
+        <v>0.12959999999999999</v>
       </c>
       <c r="O29">
-        <f t="shared" si="1"/>
         <v>6.6096000000000004</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30">
+      <c r="A30" s="9">
         <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C30">
         <v>700</v>
@@ -4235,10 +4190,10 @@
         <v>7</v>
       </c>
       <c r="E30" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F30" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G30">
         <v>2000</v>
@@ -4253,7 +4208,7 @@
         <v>-0.05</v>
       </c>
       <c r="K30">
-        <v>0.84</v>
+        <v>0.84000000000000008</v>
       </c>
       <c r="L30">
         <v>7.84</v>
@@ -4262,20 +4217,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N30">
-        <f t="shared" si="0"/>
         <v>0.14000000000000001</v>
       </c>
       <c r="O30">
-        <f t="shared" si="1"/>
         <v>7.14</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31">
+      <c r="A31" s="9">
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C31">
         <v>811</v>
@@ -4284,10 +4237,10 @@
         <v>8.11</v>
       </c>
       <c r="E31" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F31" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G31">
         <v>1200</v>
@@ -4302,7 +4255,7 @@
         <v>-0.05</v>
       </c>
       <c r="K31">
-        <v>1.37869999999999</v>
+        <v>1.3787</v>
       </c>
       <c r="L31">
         <v>9.4886999999999997</v>
@@ -4311,20 +4264,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N31">
-        <f t="shared" si="0"/>
         <v>0.16220000000000001</v>
       </c>
       <c r="O31">
-        <f t="shared" si="1"/>
         <v>8.2721999999999998</v>
       </c>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32">
+      <c r="A32" s="9">
         <v>30</v>
       </c>
       <c r="B32" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C32">
         <v>1014</v>
@@ -4333,10 +4284,10 @@
         <v>10.14</v>
       </c>
       <c r="E32" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F32" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G32">
         <v>1600</v>
@@ -4360,20 +4311,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N32">
-        <f t="shared" si="0"/>
-        <v>0.20280000000000006</v>
+        <v>0.20280000000000009</v>
       </c>
       <c r="O32">
-        <f t="shared" si="1"/>
         <v>10.3428</v>
       </c>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33">
+      <c r="A33" s="9">
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C33">
         <v>668</v>
@@ -4382,7 +4331,7 @@
         <v>6.68</v>
       </c>
       <c r="E33" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G33">
         <v>800</v>
@@ -4406,20 +4355,18 @@
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="N33">
-        <f t="shared" si="0"/>
         <v>0.46760000000000002</v>
       </c>
       <c r="O33">
-        <f t="shared" si="1"/>
         <v>7.1475999999999997</v>
       </c>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34">
+      <c r="A34" s="9">
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C34">
         <v>162</v>
@@ -4443,20 +4390,18 @@
         <v>0</v>
       </c>
       <c r="N34">
-        <f t="shared" ref="N34:N53" si="2">(M34+J34)*D34</f>
         <v>0</v>
       </c>
       <c r="O34">
-        <f t="shared" ref="O34:O53" si="3">D34+N34</f>
         <v>1.62</v>
       </c>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35">
+      <c r="A35" s="9">
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C35">
         <v>142</v>
@@ -4486,20 +4431,18 @@
         <v>0</v>
       </c>
       <c r="N35">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O35">
-        <f t="shared" si="3"/>
         <v>1.42</v>
       </c>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36">
+      <c r="A36" s="9">
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C36">
         <v>165</v>
@@ -4529,20 +4472,18 @@
         <v>0</v>
       </c>
       <c r="N36">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O36">
-        <f t="shared" si="3"/>
         <v>1.65</v>
       </c>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37">
+      <c r="A37" s="9">
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C37">
         <v>246</v>
@@ -4572,20 +4513,18 @@
         <v>0</v>
       </c>
       <c r="N37">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O37">
-        <f t="shared" si="3"/>
         <v>2.46</v>
       </c>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38">
+      <c r="A38" s="9">
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C38">
         <v>142</v>
@@ -4615,20 +4554,18 @@
         <v>0</v>
       </c>
       <c r="N38">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O38">
-        <f t="shared" si="3"/>
         <v>1.42</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39">
+      <c r="A39" s="9">
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C39">
         <v>263</v>
@@ -4658,20 +4595,18 @@
         <v>0</v>
       </c>
       <c r="N39">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O39">
-        <f t="shared" si="3"/>
         <v>2.63</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40">
+      <c r="A40" s="9">
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C40">
         <v>302</v>
@@ -4701,20 +4636,18 @@
         <v>0</v>
       </c>
       <c r="N40">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O40">
-        <f t="shared" si="3"/>
         <v>3.02</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41">
+      <c r="A41" s="9">
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C41">
         <v>164</v>
@@ -4744,20 +4677,18 @@
         <v>0</v>
       </c>
       <c r="N41">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O41">
-        <f t="shared" si="3"/>
         <v>1.64</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42">
+      <c r="A42" s="9">
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C42">
         <v>177</v>
@@ -4787,20 +4718,18 @@
         <v>0</v>
       </c>
       <c r="N42">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O42">
-        <f t="shared" si="3"/>
         <v>1.77</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43">
+      <c r="A43" s="9">
         <v>41</v>
       </c>
       <c r="B43" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C43">
         <v>282</v>
@@ -4809,7 +4738,7 @@
         <v>2.82</v>
       </c>
       <c r="E43" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G43">
         <v>330</v>
@@ -4833,20 +4762,18 @@
         <v>0</v>
       </c>
       <c r="N43">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O43">
-        <f t="shared" si="3"/>
         <v>2.82</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44">
+      <c r="A44" s="9">
         <v>42</v>
       </c>
       <c r="B44" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C44">
         <v>336</v>
@@ -4855,7 +4782,7 @@
         <v>3.36</v>
       </c>
       <c r="E44" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G44">
         <v>380</v>
@@ -4879,20 +4806,18 @@
         <v>0</v>
       </c>
       <c r="N44">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O44">
-        <f t="shared" si="3"/>
         <v>3.36</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45">
+      <c r="A45" s="9">
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C45">
         <v>343</v>
@@ -4901,7 +4826,7 @@
         <v>3.43</v>
       </c>
       <c r="E45" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G45">
         <v>400</v>
@@ -4925,20 +4850,18 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O45">
-        <f t="shared" si="3"/>
         <v>3.43</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46">
+      <c r="A46" s="9">
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C46">
         <v>383</v>
@@ -4947,7 +4870,7 @@
         <v>3.83</v>
       </c>
       <c r="E46" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G46">
         <v>480</v>
@@ -4971,20 +4894,18 @@
         <v>0</v>
       </c>
       <c r="N46">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O46">
-        <f t="shared" si="3"/>
         <v>3.83</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A47">
+      <c r="A47" s="9">
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C47">
         <v>414</v>
@@ -4993,7 +4914,7 @@
         <v>4.1399999999999997</v>
       </c>
       <c r="E47" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G47">
         <v>550</v>
@@ -5011,26 +4932,24 @@
         <v>0.20699999999999999</v>
       </c>
       <c r="L47">
-        <v>4.3469999999999898</v>
+        <v>4.3470000000000004</v>
       </c>
       <c r="M47">
         <v>0</v>
       </c>
       <c r="N47">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O47">
-        <f t="shared" si="3"/>
         <v>4.1399999999999997</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A48">
+      <c r="A48" s="9">
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C48">
         <v>486</v>
@@ -5039,7 +4958,7 @@
         <v>4.8600000000000003</v>
       </c>
       <c r="E48" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G48">
         <v>580</v>
@@ -5057,26 +4976,24 @@
         <v>0.24299999999999999</v>
       </c>
       <c r="L48">
-        <v>5.1029999999999998</v>
+        <v>5.1030000000000006</v>
       </c>
       <c r="M48">
         <v>0</v>
       </c>
       <c r="N48">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O48">
-        <f t="shared" si="3"/>
         <v>4.8600000000000003</v>
       </c>
     </row>
     <row r="49" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A49">
+      <c r="A49" s="9">
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C49">
         <v>558</v>
@@ -5085,7 +5002,7 @@
         <v>5.58</v>
       </c>
       <c r="E49" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G49">
         <v>650</v>
@@ -5109,20 +5026,18 @@
         <v>0</v>
       </c>
       <c r="N49">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O49">
-        <f t="shared" si="3"/>
         <v>5.58</v>
       </c>
     </row>
     <row r="50" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A50">
+      <c r="A50" s="9">
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C50">
         <v>606</v>
@@ -5131,7 +5046,7 @@
         <v>6.06</v>
       </c>
       <c r="E50" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G50">
         <v>1000</v>
@@ -5149,26 +5064,24 @@
         <v>0.30299999999999999</v>
       </c>
       <c r="L50">
-        <v>6.3629999999999898</v>
+        <v>6.3630000000000004</v>
       </c>
       <c r="M50">
         <v>0</v>
       </c>
       <c r="N50">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O50">
-        <f t="shared" si="3"/>
         <v>6.06</v>
       </c>
     </row>
     <row r="51" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A51">
+      <c r="A51" s="9">
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C51">
         <v>643</v>
@@ -5177,7 +5090,7 @@
         <v>6.43</v>
       </c>
       <c r="E51" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G51">
         <v>1100</v>
@@ -5201,20 +5114,18 @@
         <v>0</v>
       </c>
       <c r="N51">
-        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="O51">
-        <f t="shared" si="3"/>
         <v>6.43</v>
       </c>
     </row>
     <row r="52" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A52">
+      <c r="A52" s="9">
         <v>50</v>
       </c>
       <c r="B52" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C52">
         <v>706</v>
@@ -5223,10 +5134,10 @@
         <v>7.06</v>
       </c>
       <c r="E52" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F52" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G52">
         <v>900</v>
@@ -5238,32 +5149,30 @@
         <v>0.1</v>
       </c>
       <c r="J52">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="K52">
-        <v>0</v>
+        <v>0.35299999999999998</v>
       </c>
       <c r="L52">
-        <v>7.06</v>
+        <v>7.4129999999999994</v>
       </c>
       <c r="M52">
         <v>0</v>
       </c>
       <c r="N52">
-        <f t="shared" si="2"/>
-        <v>-0.70599999999999996</v>
+        <v>-0.35299999999999998</v>
       </c>
       <c r="O52">
-        <f t="shared" si="3"/>
-        <v>6.3539999999999992</v>
+        <v>6.7069999999999999</v>
       </c>
     </row>
     <row r="53" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A53">
+      <c r="A53" s="9">
         <v>51</v>
       </c>
       <c r="B53" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C53">
         <v>844</v>
@@ -5272,10 +5181,10 @@
         <v>8.44</v>
       </c>
       <c r="E53" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F53" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G53">
         <v>1000</v>
@@ -5287,29 +5196,26 @@
         <v>0.1</v>
       </c>
       <c r="J53">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="K53">
-        <v>0</v>
+        <v>0.42199999999999999</v>
       </c>
       <c r="L53">
-        <v>8.44</v>
+        <v>8.8620000000000001</v>
       </c>
       <c r="M53">
         <v>0</v>
       </c>
       <c r="N53">
-        <f t="shared" si="2"/>
-        <v>-0.84399999999999997</v>
+        <v>-0.42199999999999999</v>
       </c>
       <c r="O53">
-        <f t="shared" si="3"/>
-        <v>7.5959999999999992</v>
+        <v>8.0179999999999989</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -5327,19 +5233,19 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -5347,7 +5253,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -5364,7 +5270,7 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3">
         <v>121</v>
@@ -5381,7 +5287,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4">
         <v>125</v>
@@ -5398,7 +5304,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B5">
         <v>139</v>
@@ -5415,7 +5321,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B6">
         <v>142</v>
@@ -5432,7 +5338,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B7">
         <v>142</v>
@@ -5449,7 +5355,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>160</v>
@@ -5466,7 +5372,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B9">
         <v>162</v>
@@ -5477,7 +5383,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B10">
         <v>164</v>
@@ -5494,7 +5400,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B11">
         <v>165</v>
@@ -5511,7 +5417,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>169</v>
@@ -5528,7 +5434,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B13">
         <v>177</v>
@@ -5545,7 +5451,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B14">
         <v>187</v>
@@ -5562,7 +5468,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B15">
         <v>210</v>
@@ -5579,7 +5485,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16">
         <v>215</v>
@@ -5596,7 +5502,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B17">
         <v>218</v>
@@ -5613,7 +5519,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B18">
         <v>246</v>
@@ -5630,7 +5536,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B19">
         <v>253</v>
@@ -5647,7 +5553,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B20">
         <v>263</v>
@@ -5664,7 +5570,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B21">
         <v>281</v>
@@ -5675,7 +5581,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B22">
         <v>282</v>
@@ -5692,7 +5598,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B23">
         <v>284</v>
@@ -5709,7 +5615,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B24">
         <v>295</v>
@@ -5726,7 +5632,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B25">
         <v>301</v>
@@ -5737,7 +5643,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B26">
         <v>301</v>
@@ -5754,7 +5660,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B27">
         <v>302</v>
@@ -5771,7 +5677,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B28">
         <v>326</v>
@@ -5788,7 +5694,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B29">
         <v>336</v>
@@ -5805,7 +5711,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B30">
         <v>343</v>
@@ -5822,7 +5728,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B31">
         <v>350</v>
@@ -5839,7 +5745,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B32">
         <v>367</v>
@@ -5856,7 +5762,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B33">
         <v>376</v>
@@ -5873,7 +5779,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B34">
         <v>383</v>
@@ -5890,7 +5796,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B35">
         <v>413</v>
@@ -5907,7 +5813,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B36">
         <v>414</v>
@@ -5924,7 +5830,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B37">
         <v>441</v>
@@ -5941,7 +5847,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B38">
         <v>472</v>
@@ -5958,7 +5864,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B39">
         <v>486</v>
@@ -5975,7 +5881,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B40">
         <v>546</v>
@@ -5992,7 +5898,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B41">
         <v>558</v>
@@ -6009,7 +5915,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B42">
         <v>573</v>
@@ -6026,7 +5932,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B43">
         <v>606</v>
@@ -6043,7 +5949,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B44">
         <v>642</v>
@@ -6060,7 +5966,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B45">
         <v>643</v>
@@ -6077,7 +5983,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B46">
         <v>648</v>
@@ -6094,7 +6000,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B47">
         <v>700</v>
@@ -6111,7 +6017,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B48">
         <v>706</v>
@@ -6128,7 +6034,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B49">
         <v>811</v>
@@ -6145,7 +6051,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B50">
         <v>844</v>
@@ -6162,7 +6068,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B51">
         <v>1014</v>

</xml_diff>

<commit_message>
RX 6500 XT added to GPU of interest: the price of the 6500 XT might make it somewhat of a value proposition around its price point, especially at BDT 20,000 rough EDA shows lowest 6500 XT may cost BDT. 22,500
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="120">
   <si>
     <t>gpu_unit_name</t>
   </si>
@@ -373,6 +373,15 @@
   </si>
   <si>
     <t>Geforce RTX 3060</t>
+  </si>
+  <si>
+    <t>Radeon RX 6500 XT</t>
+  </si>
+  <si>
+    <t>rx_6500_xt_problems</t>
+  </si>
+  <si>
+    <t>poor PCI. E 3.0 performance, no hardware encoding ( thus, screen capturing on gpu not supported), only 2 display output ports; it's basically a laptop card turned into a desktop card)</t>
   </si>
 </sst>
 </file>
@@ -497,7 +506,7 @@
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -516,6 +525,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -574,8 +584,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G53" totalsRowShown="0" headerRowDxfId="2">
-  <autoFilter ref="A1:G53"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:G54" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:G54"/>
   <tableColumns count="7">
     <tableColumn id="1" name="gpu_unit_name"/>
     <tableColumn id="2" name="performance" dataDxfId="1"/>
@@ -2728,6 +2738,29 @@
       </c>
     </row>
     <row r="54" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B54" s="10">
+        <v>166</v>
+      </c>
+      <c r="C54" s="2">
+        <f>B54/100</f>
+        <v>1.66</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>70</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="F54" s="2">
+        <v>200</v>
+      </c>
+      <c r="G54" s="2">
+        <f>F54*125</f>
+        <v>25000</v>
+      </c>
       <c r="U54" t="s">
         <v>12</v>
       </c>
@@ -2773,7 +2806,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
@@ -2911,6 +2944,17 @@
       </c>
       <c r="C12">
         <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="2">
+        <v>-10</v>
       </c>
     </row>
   </sheetData>
@@ -2924,10 +2968,6 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="14" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="9.42578125" customWidth="1"/>
-    <col min="15" max="15" width="16.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
code changes for better documentation some column of overall_tier_df changed for better documentation tier_score.xlsx now contain those updated column names in the overall_tier_score sheet
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -3065,7 +3065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O54"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3106,35 +3106,40 @@
       </c>
       <c r="I1" s="10" t="inlineStr">
         <is>
-          <t>positive_additional_score_multiplier</t>
+          <t>positive_score_multiplier</t>
         </is>
       </c>
       <c r="J1" s="10" t="inlineStr">
         <is>
-          <t>negative_additional_score_multiplier</t>
+          <t>negative_score_multiplier</t>
         </is>
       </c>
       <c r="K1" s="10" t="inlineStr">
         <is>
+          <t>overall_score_multiplier</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
           <t>overall_additional_score</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="M1" s="10" t="inlineStr">
         <is>
           <t>net_tier_score</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="N1" s="10" t="inlineStr">
         <is>
           <t>non_rt_positive_score_multiplier</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="O1" s="10" t="inlineStr">
         <is>
           <t>non_rt_additional_score</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="P1" s="10" t="inlineStr">
         <is>
           <t>non_rt_net_score</t>
         </is>
@@ -3152,42 +3157,27 @@
       <c r="C2" t="n">
         <v>121</v>
       </c>
-      <c r="D2" t="n">
-        <v>1.21</v>
-      </c>
+      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>arc_driver_issues</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>140</v>
-      </c>
-      <c r="H2" t="n">
-        <v>17500</v>
-      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="n">
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>-0.121</v>
-      </c>
-      <c r="L2" t="n">
-        <v>1.089</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
       <c r="N2" t="n">
-        <v>-0.121</v>
-      </c>
-      <c r="O2" t="n">
-        <v>1.089</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="n">
@@ -3201,9 +3191,7 @@
       <c r="C3" t="n">
         <v>281</v>
       </c>
-      <c r="D3" t="n">
-        <v>2.81</v>
-      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
@@ -3219,20 +3207,15 @@
         <v>-0.1</v>
       </c>
       <c r="K3" t="n">
-        <v>-0.281</v>
-      </c>
-      <c r="L3" t="n">
-        <v>2.529</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.1</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="n">
-        <v>-0.281</v>
-      </c>
-      <c r="O3" t="n">
-        <v>2.529</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="n">
@@ -3246,9 +3229,7 @@
       <c r="C4" t="n">
         <v>301</v>
       </c>
-      <c r="D4" t="n">
-        <v>3.01</v>
-      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
@@ -3264,20 +3245,15 @@
         <v>-0.1</v>
       </c>
       <c r="K4" t="n">
-        <v>-0.301</v>
-      </c>
-      <c r="L4" t="n">
-        <v>2.709</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.1</v>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="n">
-        <v>-0.301</v>
-      </c>
-      <c r="O4" t="n">
-        <v>2.709</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="n">
@@ -3291,17 +3267,11 @@
       <c r="C5" t="n">
         <v>100</v>
       </c>
-      <c r="D5" t="n">
-        <v>1</v>
-      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
-      <c r="G5" t="n">
-        <v>140</v>
-      </c>
-      <c r="H5" t="n">
-        <v>17500</v>
-      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="n">
         <v>0</v>
       </c>
@@ -3311,18 +3281,13 @@
       <c r="K5" t="n">
         <v>0</v>
       </c>
-      <c r="L5" t="n">
-        <v>1</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
       <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="n">
@@ -3336,17 +3301,11 @@
       <c r="C6" t="n">
         <v>160</v>
       </c>
-      <c r="D6" t="n">
-        <v>1.6</v>
-      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
-      <c r="G6" t="n">
-        <v>300</v>
-      </c>
-      <c r="H6" t="n">
-        <v>37500</v>
-      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
       <c r="I6" t="n">
         <v>0</v>
       </c>
@@ -3356,18 +3315,13 @@
       <c r="K6" t="n">
         <v>0</v>
       </c>
-      <c r="L6" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>0</v>
       </c>
-      <c r="O6" t="n">
-        <v>1.6</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n">
@@ -3381,42 +3335,27 @@
       <c r="C7" t="n">
         <v>125</v>
       </c>
-      <c r="D7" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>low_power low_profile</t>
-        </is>
-      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
-      <c r="G7" t="n">
-        <v>150</v>
-      </c>
-      <c r="H7" t="n">
-        <v>18750</v>
-      </c>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
       <c r="I7" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="L7" t="n">
-        <v>1.3125</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0.05</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
-        <v>0.0625</v>
-      </c>
-      <c r="O7" t="n">
-        <v>1.3125</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n">
@@ -3430,42 +3369,27 @@
       <c r="C8" t="n">
         <v>139</v>
       </c>
-      <c r="D8" t="n">
-        <v>1.39</v>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>low_power low_profile</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
-      <c r="G8" t="n">
-        <v>150</v>
-      </c>
-      <c r="H8" t="n">
-        <v>18750</v>
-      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
       <c r="K8" t="n">
-        <v>0.06949999999999999</v>
-      </c>
-      <c r="L8" t="n">
-        <v>1.4595</v>
-      </c>
-      <c r="M8" t="n">
-        <v>0.05</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
-        <v>0.06949999999999999</v>
-      </c>
-      <c r="O8" t="n">
-        <v>1.4595</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n">
@@ -3479,17 +3403,11 @@
       <c r="C9" t="n">
         <v>169</v>
       </c>
-      <c r="D9" t="n">
-        <v>1.69</v>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
-      <c r="G9" t="n">
-        <v>160</v>
-      </c>
-      <c r="H9" t="n">
-        <v>20000</v>
-      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="n">
         <v>0</v>
       </c>
@@ -3499,18 +3417,13 @@
       <c r="K9" t="n">
         <v>0</v>
       </c>
-      <c r="L9" t="n">
-        <v>1.69</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
       <c r="N9" t="n">
         <v>0</v>
       </c>
-      <c r="O9" t="n">
-        <v>1.69</v>
-      </c>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n">
@@ -3524,17 +3437,11 @@
       <c r="C10" t="n">
         <v>187</v>
       </c>
-      <c r="D10" t="n">
-        <v>1.87</v>
-      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
-      <c r="G10" t="n">
-        <v>220</v>
-      </c>
-      <c r="H10" t="n">
-        <v>27500</v>
-      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="n">
         <v>0</v>
       </c>
@@ -3544,18 +3451,13 @@
       <c r="K10" t="n">
         <v>0</v>
       </c>
-      <c r="L10" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
       <c r="N10" t="n">
         <v>0</v>
       </c>
-      <c r="O10" t="n">
-        <v>1.87</v>
-      </c>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n">
@@ -3569,17 +3471,11 @@
       <c r="C11" t="n">
         <v>210</v>
       </c>
-      <c r="D11" t="n">
-        <v>2.1</v>
-      </c>
+      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
-      <c r="G11" t="n">
-        <v>230</v>
-      </c>
-      <c r="H11" t="n">
-        <v>28750</v>
-      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="n">
         <v>0</v>
       </c>
@@ -3589,18 +3485,13 @@
       <c r="K11" t="n">
         <v>0</v>
       </c>
-      <c r="L11" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
         <v>0</v>
       </c>
-      <c r="O11" t="n">
-        <v>2.1</v>
-      </c>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n">
@@ -3614,17 +3505,11 @@
       <c r="C12" t="n">
         <v>215</v>
       </c>
-      <c r="D12" t="n">
-        <v>2.15</v>
-      </c>
+      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
-      <c r="G12" t="n">
-        <v>280</v>
-      </c>
-      <c r="H12" t="n">
-        <v>35000</v>
-      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
       <c r="I12" t="n">
         <v>0</v>
       </c>
@@ -3634,18 +3519,13 @@
       <c r="K12" t="n">
         <v>0</v>
       </c>
-      <c r="L12" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="M12" t="n">
-        <v>0</v>
-      </c>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
         <v>0</v>
       </c>
-      <c r="O12" t="n">
-        <v>2.15</v>
-      </c>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n">
@@ -3659,42 +3539,27 @@
       <c r="C13" t="n">
         <v>253</v>
       </c>
-      <c r="D13" t="n">
-        <v>2.53</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>rt_1 dlss_2</t>
-        </is>
-      </c>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
-      <c r="G13" t="n">
-        <v>300</v>
-      </c>
-      <c r="H13" t="n">
-        <v>37500</v>
-      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>0.3036</v>
-      </c>
-      <c r="L13" t="n">
-        <v>2.8336</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
-        <v>0.1771</v>
-      </c>
-      <c r="O13" t="n">
-        <v>2.7071</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n">
@@ -3708,42 +3573,27 @@
       <c r="C14" t="n">
         <v>284</v>
       </c>
-      <c r="D14" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>rt_1 dlss_2</t>
-        </is>
-      </c>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
-      <c r="G14" t="n">
-        <v>400</v>
-      </c>
-      <c r="H14" t="n">
-        <v>50000</v>
-      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
       </c>
       <c r="K14" t="n">
-        <v>0.3408</v>
-      </c>
-      <c r="L14" t="n">
-        <v>3.1808</v>
-      </c>
-      <c r="M14" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
-        <v>0.1988</v>
-      </c>
-      <c r="O14" t="n">
-        <v>3.0388</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n">
@@ -3757,17 +3607,13 @@
       <c r="C15" t="n">
         <v>295</v>
       </c>
-      <c r="D15" t="n">
-        <v>2.95</v>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="n">
         <v>500</v>
       </c>
-      <c r="H15" t="n">
-        <v>62500</v>
-      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="n">
         <v>0</v>
       </c>
@@ -3777,18 +3623,13 @@
       <c r="K15" t="n">
         <v>0</v>
       </c>
-      <c r="L15" t="n">
-        <v>2.95</v>
-      </c>
-      <c r="M15" t="n">
-        <v>0</v>
-      </c>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
       <c r="N15" t="n">
         <v>0</v>
       </c>
-      <c r="O15" t="n">
-        <v>2.95</v>
-      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
@@ -3802,42 +3643,27 @@
       <c r="C16" t="n">
         <v>326</v>
       </c>
-      <c r="D16" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>rt_1 dlss_2</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="n">
-        <v>500</v>
-      </c>
-      <c r="H16" t="n">
-        <v>62500</v>
-      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0.3911999999999999</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3.6512</v>
-      </c>
-      <c r="M16" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
-        <v>0.2282</v>
-      </c>
-      <c r="O16" t="n">
-        <v>3.4882</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n">
@@ -3851,42 +3677,27 @@
       <c r="C17" t="n">
         <v>350</v>
       </c>
-      <c r="D17" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>rt_1 dlss_2</t>
-        </is>
-      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="n">
-        <v>700</v>
-      </c>
-      <c r="H17" t="n">
-        <v>87500</v>
-      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="L17" t="n">
-        <v>3.92</v>
-      </c>
-      <c r="M17" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
-        <v>0.245</v>
-      </c>
-      <c r="O17" t="n">
-        <v>3.745</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
@@ -3900,42 +3711,27 @@
       <c r="C18" t="n">
         <v>367</v>
       </c>
-      <c r="D18" t="n">
-        <v>3.67</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>rt_1 dlss_2</t>
-        </is>
-      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr"/>
-      <c r="G18" t="n">
-        <v>700</v>
-      </c>
-      <c r="H18" t="n">
-        <v>87500</v>
-      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
         <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>0.4404</v>
-      </c>
-      <c r="L18" t="n">
-        <v>4.1104</v>
-      </c>
-      <c r="M18" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
-        <v>0.2569</v>
-      </c>
-      <c r="O18" t="n">
-        <v>3.9269</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n">
@@ -3949,42 +3745,27 @@
       <c r="C19" t="n">
         <v>413</v>
       </c>
-      <c r="D19" t="n">
-        <v>4.13</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>rt_1 dlss_2</t>
-        </is>
-      </c>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr"/>
-      <c r="G19" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H19" t="n">
-        <v>125000</v>
-      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>0.4956</v>
-      </c>
-      <c r="L19" t="n">
-        <v>4.625599999999999</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L19" t="inlineStr"/>
+      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
-        <v>0.2891</v>
-      </c>
-      <c r="O19" t="n">
-        <v>4.4191</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
@@ -3998,42 +3779,27 @@
       <c r="C20" t="n">
         <v>218</v>
       </c>
-      <c r="D20" t="n">
-        <v>2.18</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr"/>
-      <c r="G20" t="n">
-        <v>250</v>
-      </c>
-      <c r="H20" t="n">
-        <v>31250</v>
-      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>0.3706</v>
-      </c>
-      <c r="L20" t="n">
-        <v>2.5506</v>
-      </c>
-      <c r="M20" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L20" t="inlineStr"/>
+      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
-        <v>0.1526</v>
-      </c>
-      <c r="O20" t="n">
-        <v>2.3326</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n">
@@ -4047,42 +3813,27 @@
       <c r="C21" t="n">
         <v>270</v>
       </c>
-      <c r="D21" t="n">
-        <v>2.7</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
-        <v>330</v>
-      </c>
-      <c r="H21" t="n">
-        <v>41250</v>
-      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0.4590000000000001</v>
-      </c>
-      <c r="L21" t="n">
-        <v>3.159</v>
-      </c>
-      <c r="M21" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L21" t="inlineStr"/>
+      <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="O21" t="n">
-        <v>2.889</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
@@ -4096,42 +3847,27 @@
       <c r="C22" t="n">
         <v>301</v>
       </c>
-      <c r="D22" t="n">
-        <v>3.01</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="n">
-        <v>330</v>
-      </c>
-      <c r="H22" t="n">
-        <v>41250</v>
-      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J22" t="n">
         <v>0</v>
       </c>
       <c r="K22" t="n">
-        <v>0.5117</v>
-      </c>
-      <c r="L22" t="n">
-        <v>3.5217</v>
-      </c>
-      <c r="M22" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L22" t="inlineStr"/>
+      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
-        <v>0.2107</v>
-      </c>
-      <c r="O22" t="n">
-        <v>3.2207</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -4145,42 +3881,27 @@
       <c r="C23" t="n">
         <v>376</v>
       </c>
-      <c r="D23" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr"/>
-      <c r="G23" t="n">
-        <v>400</v>
-      </c>
-      <c r="H23" t="n">
-        <v>50000</v>
-      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
       <c r="I23" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
         <v>0</v>
       </c>
       <c r="K23" t="n">
-        <v>0.6392</v>
-      </c>
-      <c r="L23" t="n">
-        <v>4.3992</v>
-      </c>
-      <c r="M23" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L23" t="inlineStr"/>
+      <c r="M23" t="inlineStr"/>
       <c r="N23" t="n">
-        <v>0.2632</v>
-      </c>
-      <c r="O23" t="n">
-        <v>4.0232</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
@@ -4194,42 +3915,27 @@
       <c r="C24" t="n">
         <v>441</v>
       </c>
-      <c r="D24" t="n">
-        <v>4.41</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr"/>
-      <c r="G24" t="n">
-        <v>500</v>
-      </c>
-      <c r="H24" t="n">
-        <v>62500</v>
-      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
       <c r="I24" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>0.7497</v>
-      </c>
-      <c r="L24" t="n">
-        <v>5.1597</v>
-      </c>
-      <c r="M24" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L24" t="inlineStr"/>
+      <c r="M24" t="inlineStr"/>
       <c r="N24" t="n">
-        <v>0.3087</v>
-      </c>
-      <c r="O24" t="n">
-        <v>4.7187</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n">
@@ -4243,42 +3949,27 @@
       <c r="C25" t="n">
         <v>472</v>
       </c>
-      <c r="D25" t="n">
-        <v>4.72</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr"/>
-      <c r="G25" t="n">
-        <v>600</v>
-      </c>
-      <c r="H25" t="n">
-        <v>75000</v>
-      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
       <c r="I25" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
       </c>
       <c r="K25" t="n">
-        <v>0.8024</v>
-      </c>
-      <c r="L25" t="n">
-        <v>5.522399999999999</v>
-      </c>
-      <c r="M25" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L25" t="inlineStr"/>
+      <c r="M25" t="inlineStr"/>
       <c r="N25" t="n">
-        <v>0.3304</v>
-      </c>
-      <c r="O25" t="n">
-        <v>5.0504</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
@@ -4292,42 +3983,27 @@
       <c r="C26" t="n">
         <v>546</v>
       </c>
-      <c r="D26" t="n">
-        <v>5.46</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
-      <c r="G26" t="n">
-        <v>700</v>
-      </c>
-      <c r="H26" t="n">
-        <v>87500</v>
-      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
       </c>
       <c r="K26" t="n">
-        <v>0.9282</v>
-      </c>
-      <c r="L26" t="n">
-        <v>6.3882</v>
-      </c>
-      <c r="M26" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L26" t="inlineStr"/>
+      <c r="M26" t="inlineStr"/>
       <c r="N26" t="n">
-        <v>0.3822</v>
-      </c>
-      <c r="O26" t="n">
-        <v>5.8422</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n">
@@ -4341,42 +4017,27 @@
       <c r="C27" t="n">
         <v>573</v>
       </c>
-      <c r="D27" t="n">
-        <v>5.73</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="n">
-        <v>800</v>
-      </c>
-      <c r="H27" t="n">
-        <v>100000</v>
-      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
       </c>
       <c r="K27" t="n">
-        <v>0.9741000000000002</v>
-      </c>
-      <c r="L27" t="n">
-        <v>6.7041</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr"/>
       <c r="N27" t="n">
-        <v>0.4011000000000001</v>
-      </c>
-      <c r="O27" t="n">
-        <v>6.131100000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
@@ -4390,42 +4051,27 @@
       <c r="C28" t="n">
         <v>642</v>
       </c>
-      <c r="D28" t="n">
-        <v>6.42</v>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr"/>
-      <c r="G28" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H28" t="n">
-        <v>150000</v>
-      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
       </c>
       <c r="K28" t="n">
-        <v>1.0914</v>
-      </c>
-      <c r="L28" t="n">
-        <v>7.5114</v>
-      </c>
-      <c r="M28" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
       <c r="N28" t="n">
-        <v>0.4494</v>
-      </c>
-      <c r="O28" t="n">
-        <v>6.8694</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n">
@@ -4439,46 +4085,31 @@
       <c r="C29" t="n">
         <v>648</v>
       </c>
-      <c r="D29" t="n">
-        <v>6.48</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>monster_size</t>
         </is>
       </c>
-      <c r="G29" t="n">
-        <v>1500</v>
-      </c>
-      <c r="H29" t="n">
-        <v>187500</v>
-      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
       <c r="I29" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J29" t="n">
         <v>-0.05</v>
       </c>
       <c r="K29" t="n">
-        <v>0.7776000000000001</v>
-      </c>
-      <c r="L29" t="n">
-        <v>7.2576</v>
-      </c>
-      <c r="M29" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
       <c r="N29" t="n">
-        <v>0.1296</v>
-      </c>
-      <c r="O29" t="n">
-        <v>6.6096</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n">
@@ -4492,46 +4123,31 @@
       <c r="C30" t="n">
         <v>700</v>
       </c>
-      <c r="D30" t="n">
-        <v>7</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>rt_2 dlss_2</t>
-        </is>
-      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr">
         <is>
           <t>monster_size</t>
         </is>
       </c>
-      <c r="G30" t="n">
-        <v>2000</v>
-      </c>
-      <c r="H30" t="n">
-        <v>250000</v>
-      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
       <c r="I30" t="n">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
         <v>-0.05</v>
       </c>
       <c r="K30" t="n">
-        <v>0.8400000000000001</v>
-      </c>
-      <c r="L30" t="n">
-        <v>7.84</v>
-      </c>
-      <c r="M30" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="n">
-        <v>0.14</v>
-      </c>
-      <c r="O30" t="n">
-        <v>7.14</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n">
@@ -4545,46 +4161,31 @@
       <c r="C31" t="n">
         <v>811</v>
       </c>
-      <c r="D31" t="n">
-        <v>8.109999999999999</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>rt_3 dlss_2 dlss_3</t>
-        </is>
-      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>monster_size</t>
         </is>
       </c>
-      <c r="G31" t="n">
-        <v>1200</v>
-      </c>
-      <c r="H31" t="n">
-        <v>150000</v>
-      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
         <v>-0.05</v>
       </c>
       <c r="K31" t="n">
-        <v>1.3787</v>
-      </c>
-      <c r="L31" t="n">
-        <v>9.4887</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
       <c r="N31" t="n">
-        <v>0.1622</v>
-      </c>
-      <c r="O31" t="n">
-        <v>8.2722</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n">
@@ -4598,46 +4199,31 @@
       <c r="C32" t="n">
         <v>1014</v>
       </c>
-      <c r="D32" t="n">
-        <v>10.14</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>rt_3 dlss_2 dlss_3</t>
-        </is>
-      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>monster_size</t>
         </is>
       </c>
-      <c r="G32" t="n">
-        <v>1600</v>
-      </c>
-      <c r="H32" t="n">
-        <v>200000</v>
-      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
       <c r="I32" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="J32" t="n">
         <v>-0.05</v>
       </c>
       <c r="K32" t="n">
-        <v>1.7238</v>
-      </c>
-      <c r="L32" t="n">
-        <v>11.8638</v>
-      </c>
-      <c r="M32" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr"/>
       <c r="N32" t="n">
-        <v>0.2028000000000001</v>
-      </c>
-      <c r="O32" t="n">
-        <v>10.3428</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n">
@@ -4651,42 +4237,27 @@
       <c r="C33" t="n">
         <v>668</v>
       </c>
-      <c r="D33" t="n">
-        <v>6.68</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>rt_3 dlss_2 dlss_3</t>
-        </is>
-      </c>
+      <c r="D33" t="inlineStr"/>
+      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="n">
-        <v>800</v>
-      </c>
-      <c r="H33" t="n">
-        <v>100000</v>
-      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
       <c r="I33" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>1.4696</v>
-      </c>
-      <c r="L33" t="n">
-        <v>8.1496</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0.07000000000000001</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
       <c r="N33" t="n">
-        <v>0.4676</v>
-      </c>
-      <c r="O33" t="n">
-        <v>7.1476</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n">
@@ -4700,9 +4271,7 @@
       <c r="C34" t="n">
         <v>162</v>
       </c>
-      <c r="D34" t="n">
-        <v>1.62</v>
-      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr"/>
@@ -4716,18 +4285,13 @@
       <c r="K34" t="n">
         <v>0</v>
       </c>
-      <c r="L34" t="n">
-        <v>1.62</v>
-      </c>
-      <c r="M34" t="n">
-        <v>0</v>
-      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr"/>
       <c r="N34" t="n">
         <v>0</v>
       </c>
-      <c r="O34" t="n">
-        <v>1.62</v>
-      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n">
@@ -4741,17 +4305,11 @@
       <c r="C35" t="n">
         <v>142</v>
       </c>
-      <c r="D35" t="n">
-        <v>1.42</v>
-      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr"/>
-      <c r="G35" t="n">
-        <v>170</v>
-      </c>
-      <c r="H35" t="n">
-        <v>21250</v>
-      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
       <c r="I35" t="n">
         <v>0</v>
       </c>
@@ -4761,18 +4319,13 @@
       <c r="K35" t="n">
         <v>0</v>
       </c>
-      <c r="L35" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="M35" t="n">
-        <v>0</v>
-      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
       <c r="N35" t="n">
         <v>0</v>
       </c>
-      <c r="O35" t="n">
-        <v>1.42</v>
-      </c>
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n">
@@ -4786,17 +4339,11 @@
       <c r="C36" t="n">
         <v>165</v>
       </c>
-      <c r="D36" t="n">
-        <v>1.65</v>
-      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
-      <c r="G36" t="n">
-        <v>200</v>
-      </c>
-      <c r="H36" t="n">
-        <v>25000</v>
-      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
       <c r="I36" t="n">
         <v>0</v>
       </c>
@@ -4806,18 +4353,13 @@
       <c r="K36" t="n">
         <v>0</v>
       </c>
-      <c r="L36" t="n">
-        <v>1.65</v>
-      </c>
-      <c r="M36" t="n">
-        <v>0</v>
-      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
       <c r="N36" t="n">
         <v>0</v>
       </c>
-      <c r="O36" t="n">
-        <v>1.65</v>
-      </c>
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n">
@@ -4831,17 +4373,11 @@
       <c r="C37" t="n">
         <v>246</v>
       </c>
-      <c r="D37" t="n">
-        <v>2.46</v>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr"/>
-      <c r="G37" t="n">
-        <v>280</v>
-      </c>
-      <c r="H37" t="n">
-        <v>35000</v>
-      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
       <c r="I37" t="n">
         <v>0</v>
       </c>
@@ -4851,18 +4387,13 @@
       <c r="K37" t="n">
         <v>0</v>
       </c>
-      <c r="L37" t="n">
-        <v>2.46</v>
-      </c>
-      <c r="M37" t="n">
-        <v>0</v>
-      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr"/>
       <c r="N37" t="n">
         <v>0</v>
       </c>
-      <c r="O37" t="n">
-        <v>2.46</v>
-      </c>
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n">
@@ -4876,17 +4407,11 @@
       <c r="C38" t="n">
         <v>142</v>
       </c>
-      <c r="D38" t="n">
-        <v>1.42</v>
-      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr"/>
-      <c r="G38" t="n">
-        <v>170</v>
-      </c>
-      <c r="H38" t="n">
-        <v>21250</v>
-      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
       <c r="I38" t="n">
         <v>0</v>
       </c>
@@ -4896,18 +4421,13 @@
       <c r="K38" t="n">
         <v>0</v>
       </c>
-      <c r="L38" t="n">
-        <v>1.42</v>
-      </c>
-      <c r="M38" t="n">
-        <v>0</v>
-      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
       <c r="N38" t="n">
         <v>0</v>
       </c>
-      <c r="O38" t="n">
-        <v>1.42</v>
-      </c>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n">
@@ -4921,17 +4441,11 @@
       <c r="C39" t="n">
         <v>263</v>
       </c>
-      <c r="D39" t="n">
-        <v>2.63</v>
-      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr"/>
-      <c r="G39" t="n">
-        <v>350</v>
-      </c>
-      <c r="H39" t="n">
-        <v>43750</v>
-      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
       <c r="I39" t="n">
         <v>0</v>
       </c>
@@ -4941,18 +4455,13 @@
       <c r="K39" t="n">
         <v>0</v>
       </c>
-      <c r="L39" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="M39" t="n">
-        <v>0</v>
-      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr"/>
       <c r="N39" t="n">
         <v>0</v>
       </c>
-      <c r="O39" t="n">
-        <v>2.63</v>
-      </c>
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n">
@@ -4966,17 +4475,11 @@
       <c r="C40" t="n">
         <v>302</v>
       </c>
-      <c r="D40" t="n">
-        <v>3.02</v>
-      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr"/>
-      <c r="G40" t="n">
-        <v>400</v>
-      </c>
-      <c r="H40" t="n">
-        <v>50000</v>
-      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
       <c r="I40" t="n">
         <v>0</v>
       </c>
@@ -4986,18 +4489,13 @@
       <c r="K40" t="n">
         <v>0</v>
       </c>
-      <c r="L40" t="n">
-        <v>3.02</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0</v>
-      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
       <c r="N40" t="n">
         <v>0</v>
       </c>
-      <c r="O40" t="n">
-        <v>3.02</v>
-      </c>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n">
@@ -5011,17 +4509,11 @@
       <c r="C41" t="n">
         <v>164</v>
       </c>
-      <c r="D41" t="n">
-        <v>1.64</v>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr"/>
-      <c r="G41" t="n">
-        <v>230</v>
-      </c>
-      <c r="H41" t="n">
-        <v>28750</v>
-      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
       <c r="I41" t="n">
         <v>0</v>
       </c>
@@ -5031,18 +4523,13 @@
       <c r="K41" t="n">
         <v>0</v>
       </c>
-      <c r="L41" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="M41" t="n">
-        <v>0</v>
-      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr"/>
       <c r="N41" t="n">
         <v>0</v>
       </c>
-      <c r="O41" t="n">
-        <v>1.64</v>
-      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n">
@@ -5056,17 +4543,11 @@
       <c r="C42" t="n">
         <v>177</v>
       </c>
-      <c r="D42" t="n">
-        <v>1.77</v>
-      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr"/>
-      <c r="G42" t="n">
-        <v>280</v>
-      </c>
-      <c r="H42" t="n">
-        <v>35000</v>
-      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
       <c r="I42" t="n">
         <v>0</v>
       </c>
@@ -5076,18 +4557,13 @@
       <c r="K42" t="n">
         <v>0</v>
       </c>
-      <c r="L42" t="n">
-        <v>1.77</v>
-      </c>
-      <c r="M42" t="n">
-        <v>0</v>
-      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr"/>
       <c r="N42" t="n">
         <v>0</v>
       </c>
-      <c r="O42" t="n">
-        <v>1.77</v>
-      </c>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n">
@@ -5101,9 +4577,7 @@
       <c r="C43" t="n">
         <v>282</v>
       </c>
-      <c r="D43" t="n">
-        <v>2.82</v>
-      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
           <t>rt_1</t>
@@ -5113,9 +4587,7 @@
       <c r="G43" t="n">
         <v>330</v>
       </c>
-      <c r="H43" t="n">
-        <v>41250</v>
-      </c>
+      <c r="H43" t="inlineStr"/>
       <c r="I43" t="n">
         <v>0.05</v>
       </c>
@@ -5123,20 +4595,15 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>0.141</v>
-      </c>
-      <c r="L43" t="n">
-        <v>2.961</v>
-      </c>
-      <c r="M43" t="n">
-        <v>0</v>
-      </c>
+        <v>0.05</v>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
       <c r="N43" t="n">
         <v>0</v>
       </c>
-      <c r="O43" t="n">
-        <v>2.82</v>
-      </c>
+      <c r="O43" t="inlineStr"/>
+      <c r="P43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n">
@@ -5150,42 +4617,27 @@
       <c r="C44" t="n">
         <v>336</v>
       </c>
-      <c r="D44" t="n">
-        <v>3.36</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D44" t="inlineStr"/>
+      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr"/>
-      <c r="G44" t="n">
-        <v>380</v>
-      </c>
-      <c r="H44" t="n">
-        <v>47500</v>
-      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
       <c r="I44" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J44" t="n">
         <v>0</v>
       </c>
       <c r="K44" t="n">
-        <v>0.168</v>
-      </c>
-      <c r="L44" t="n">
-        <v>3.528</v>
-      </c>
-      <c r="M44" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr"/>
       <c r="N44" t="n">
         <v>0</v>
       </c>
-      <c r="O44" t="n">
-        <v>3.36</v>
-      </c>
+      <c r="O44" t="inlineStr"/>
+      <c r="P44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n">
@@ -5199,42 +4651,27 @@
       <c r="C45" t="n">
         <v>343</v>
       </c>
-      <c r="D45" t="n">
-        <v>3.43</v>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr"/>
-      <c r="G45" t="n">
-        <v>400</v>
-      </c>
-      <c r="H45" t="n">
-        <v>50000</v>
-      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
       <c r="I45" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J45" t="n">
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>0.1715</v>
-      </c>
-      <c r="L45" t="n">
-        <v>3.6015</v>
-      </c>
-      <c r="M45" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr"/>
       <c r="N45" t="n">
         <v>0</v>
       </c>
-      <c r="O45" t="n">
-        <v>3.43</v>
-      </c>
+      <c r="O45" t="inlineStr"/>
+      <c r="P45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n">
@@ -5248,42 +4685,27 @@
       <c r="C46" t="n">
         <v>383</v>
       </c>
-      <c r="D46" t="n">
-        <v>3.83</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="n">
-        <v>480</v>
-      </c>
-      <c r="H46" t="n">
-        <v>60000</v>
-      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
       <c r="I46" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J46" t="n">
         <v>0</v>
       </c>
       <c r="K46" t="n">
-        <v>0.1915</v>
-      </c>
-      <c r="L46" t="n">
-        <v>4.0215</v>
-      </c>
-      <c r="M46" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
       <c r="N46" t="n">
         <v>0</v>
       </c>
-      <c r="O46" t="n">
-        <v>3.83</v>
-      </c>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n">
@@ -5297,42 +4719,27 @@
       <c r="C47" t="n">
         <v>414</v>
       </c>
-      <c r="D47" t="n">
-        <v>4.14</v>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
+      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr"/>
-      <c r="G47" t="n">
-        <v>550</v>
-      </c>
-      <c r="H47" t="n">
-        <v>68750</v>
-      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
       <c r="I47" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J47" t="n">
         <v>0</v>
       </c>
       <c r="K47" t="n">
-        <v>0.207</v>
-      </c>
-      <c r="L47" t="n">
-        <v>4.347</v>
-      </c>
-      <c r="M47" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
       <c r="N47" t="n">
         <v>0</v>
       </c>
-      <c r="O47" t="n">
-        <v>4.14</v>
-      </c>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n">
@@ -5346,42 +4753,27 @@
       <c r="C48" t="n">
         <v>486</v>
       </c>
-      <c r="D48" t="n">
-        <v>4.86</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D48" t="inlineStr"/>
+      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr"/>
-      <c r="G48" t="n">
-        <v>580</v>
-      </c>
-      <c r="H48" t="n">
-        <v>72500</v>
-      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
       <c r="I48" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>0.243</v>
-      </c>
-      <c r="L48" t="n">
-        <v>5.103000000000001</v>
-      </c>
-      <c r="M48" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr"/>
       <c r="N48" t="n">
         <v>0</v>
       </c>
-      <c r="O48" t="n">
-        <v>4.86</v>
-      </c>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n">
@@ -5395,42 +4787,27 @@
       <c r="C49" t="n">
         <v>558</v>
       </c>
-      <c r="D49" t="n">
-        <v>5.58</v>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D49" t="inlineStr"/>
+      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
-      <c r="G49" t="n">
-        <v>650</v>
-      </c>
-      <c r="H49" t="n">
-        <v>81250</v>
-      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
       <c r="I49" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J49" t="n">
         <v>0</v>
       </c>
       <c r="K49" t="n">
-        <v>0.279</v>
-      </c>
-      <c r="L49" t="n">
-        <v>5.859</v>
-      </c>
-      <c r="M49" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr"/>
       <c r="N49" t="n">
         <v>0</v>
       </c>
-      <c r="O49" t="n">
-        <v>5.58</v>
-      </c>
+      <c r="O49" t="inlineStr"/>
+      <c r="P49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n">
@@ -5444,42 +4821,27 @@
       <c r="C50" t="n">
         <v>606</v>
       </c>
-      <c r="D50" t="n">
-        <v>6.06</v>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D50" t="inlineStr"/>
+      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr"/>
-      <c r="G50" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H50" t="n">
-        <v>125000</v>
-      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
       <c r="I50" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J50" t="n">
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>0.303</v>
-      </c>
-      <c r="L50" t="n">
-        <v>6.363</v>
-      </c>
-      <c r="M50" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr"/>
       <c r="N50" t="n">
         <v>0</v>
       </c>
-      <c r="O50" t="n">
-        <v>6.06</v>
-      </c>
+      <c r="O50" t="inlineStr"/>
+      <c r="P50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n">
@@ -5493,42 +4855,27 @@
       <c r="C51" t="n">
         <v>643</v>
       </c>
-      <c r="D51" t="n">
-        <v>6.43</v>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_1  </t>
-        </is>
-      </c>
+      <c r="D51" t="inlineStr"/>
+      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="n">
-        <v>1100</v>
-      </c>
-      <c r="H51" t="n">
-        <v>137500</v>
-      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
       <c r="I51" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>0.3215</v>
-      </c>
-      <c r="L51" t="n">
-        <v>6.7515</v>
-      </c>
-      <c r="M51" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="L51" t="inlineStr"/>
+      <c r="M51" t="inlineStr"/>
       <c r="N51" t="n">
         <v>0</v>
       </c>
-      <c r="O51" t="n">
-        <v>6.43</v>
-      </c>
+      <c r="O51" t="inlineStr"/>
+      <c r="P51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n">
@@ -5542,46 +4889,31 @@
       <c r="C52" t="n">
         <v>706</v>
       </c>
-      <c r="D52" t="n">
-        <v>7.06</v>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_2  </t>
-        </is>
-      </c>
+      <c r="D52" t="inlineStr"/>
+      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>radeon_high_temp</t>
         </is>
       </c>
-      <c r="G52" t="n">
-        <v>900</v>
-      </c>
-      <c r="H52" t="n">
-        <v>112500</v>
-      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
       <c r="I52" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J52" t="n">
         <v>-0.05</v>
       </c>
       <c r="K52" t="n">
-        <v>0.353</v>
-      </c>
-      <c r="L52" t="n">
-        <v>7.412999999999999</v>
-      </c>
-      <c r="M52" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L52" t="inlineStr"/>
+      <c r="M52" t="inlineStr"/>
       <c r="N52" t="n">
-        <v>-0.353</v>
-      </c>
-      <c r="O52" t="n">
-        <v>6.707</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O52" t="inlineStr"/>
+      <c r="P52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n">
@@ -5595,46 +4927,31 @@
       <c r="C53" t="n">
         <v>844</v>
       </c>
-      <c r="D53" t="n">
-        <v>8.44</v>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t xml:space="preserve">rt_2  </t>
-        </is>
-      </c>
+      <c r="D53" t="inlineStr"/>
+      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>radeon_high_temp</t>
         </is>
       </c>
-      <c r="G53" t="n">
-        <v>1000</v>
-      </c>
-      <c r="H53" t="n">
-        <v>125000</v>
-      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
       <c r="I53" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J53" t="n">
         <v>-0.05</v>
       </c>
       <c r="K53" t="n">
-        <v>0.422</v>
-      </c>
-      <c r="L53" t="n">
-        <v>8.862</v>
-      </c>
-      <c r="M53" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L53" t="inlineStr"/>
+      <c r="M53" t="inlineStr"/>
       <c r="N53" t="n">
-        <v>-0.422</v>
-      </c>
-      <c r="O53" t="n">
-        <v>8.017999999999999</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n">
@@ -5648,9 +4965,7 @@
       <c r="C54" t="n">
         <v>166</v>
       </c>
-      <c r="D54" t="n">
-        <v>1.66</v>
-      </c>
+      <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
           <t>rt_1</t>
@@ -5664,9 +4979,7 @@
       <c r="G54" t="n">
         <v>200</v>
       </c>
-      <c r="H54" t="n">
-        <v>25000</v>
-      </c>
+      <c r="H54" t="inlineStr"/>
       <c r="I54" t="n">
         <v>0.05</v>
       </c>
@@ -5674,20 +4987,15 @@
         <v>-0.1</v>
       </c>
       <c r="K54" t="n">
-        <v>-0.083</v>
-      </c>
-      <c r="L54" t="n">
-        <v>1.577</v>
-      </c>
-      <c r="M54" t="n">
-        <v>0</v>
-      </c>
+        <v>-0.05</v>
+      </c>
+      <c r="L54" t="inlineStr"/>
+      <c r="M54" t="inlineStr"/>
       <c r="N54" t="n">
-        <v>-0.166</v>
-      </c>
-      <c r="O54" t="n">
-        <v>1.494</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="O54" t="inlineStr"/>
+      <c r="P54" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
now includes both 3060 8gb and 12gb tier scores
</commit_message>
<xml_diff>
--- a/tier_score.xlsx
+++ b/tier_score.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12330"/>
   </bookViews>
   <sheets>
     <sheet name="tier_score_sheet" sheetId="1" r:id="rId1"/>
@@ -17,12 +17,12 @@
     <sheet name="overall_tier_scores" sheetId="3" r:id="rId3"/>
     <sheet name="tier_score_sheet_copy" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="108">
   <si>
     <t>gpu_unit_name</t>
   </si>
@@ -48,6 +48,9 @@
     <t>Intel Arc A380</t>
   </si>
   <si>
+    <t>rt_1</t>
+  </si>
+  <si>
     <t>arc_driver_issues</t>
   </si>
   <si>
@@ -114,223 +117,229 @@
     <t>rt_2 dlss_2</t>
   </si>
   <si>
+    <t>Geforce RTX 3060 8GB</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3060 12GB</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3060 Ti</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3070</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3070 Ti</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3080 10GB</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3080 12GB</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3080 Ti</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3090</t>
+  </si>
+  <si>
+    <t>monster_size</t>
+  </si>
+  <si>
+    <t>Geforce RTX 3090 Ti</t>
+  </si>
+  <si>
+    <t>Geforce RTX 4080</t>
+  </si>
+  <si>
+    <t>rt_3 dlss_2 dlss_3</t>
+  </si>
+  <si>
+    <t>Geforce RTX 4090</t>
+  </si>
+  <si>
+    <t>Geforce RTX 4070 Ti</t>
+  </si>
+  <si>
+    <t>Radeon RX 5500 OEM</t>
+  </si>
+  <si>
+    <t>Radeon RX 5500 XT 4GB</t>
+  </si>
+  <si>
+    <t>Radeon RX 5500 XT 8GB</t>
+  </si>
+  <si>
+    <t>Radeon RX 5600 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 570</t>
+  </si>
+  <si>
+    <t>Radeon RX 5700</t>
+  </si>
+  <si>
+    <t>Radeon RX 5700 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 580</t>
+  </si>
+  <si>
+    <t>Radeon RX 590</t>
+  </si>
+  <si>
+    <t>Radeon RX 6600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rt_1 </t>
+  </si>
+  <si>
+    <t>Radeon RX 6600 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 6650 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 6700 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 6750 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 6800</t>
+  </si>
+  <si>
+    <t>Radeon RX 6800 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 6900 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 6950 XT</t>
+  </si>
+  <si>
+    <t>Radeon RX 7900 XT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rt_2 </t>
+  </si>
+  <si>
+    <t>radeon_high_temp</t>
+  </si>
+  <si>
+    <t>Radeon RX 7900 XTX</t>
+  </si>
+  <si>
+    <t>Radeon RX 6500 XT</t>
+  </si>
+  <si>
+    <t>rx_6500_xt_problems</t>
+  </si>
+  <si>
+    <t>comment_code</t>
+  </si>
+  <si>
+    <t>comment_desc</t>
+  </si>
+  <si>
+    <t>weight_score</t>
+  </si>
+  <si>
+    <t>1st generation ray tracing capabilities or equivalent/limited ray tracing capabilities</t>
+  </si>
+  <si>
+    <t>rt_2</t>
+  </si>
+  <si>
+    <t>2nd generation ray tracing capabilities or equivalent</t>
+  </si>
+  <si>
+    <t>rt_3</t>
+  </si>
+  <si>
+    <t>3rd generation ray tracing capabilities or equivalent</t>
+  </si>
+  <si>
+    <t>dlss_2</t>
+  </si>
+  <si>
+    <t>supports Nvidia's DLSS (Deep Learning Super Sampling) 2 upscaling technology, increasing FPS in supported games</t>
+  </si>
+  <si>
+    <t>dlss_3</t>
+  </si>
+  <si>
+    <t>supports Nvidia's DLSS (Deep Learning Super Sampling) 3.0 upscaling technology, currently the technology can potentially noticably degrade visual quality, and increase input latency unlike DLSS 2</t>
+  </si>
+  <si>
+    <t>low_power</t>
+  </si>
+  <si>
+    <t>low power consumption (just 75 watts), no need for external power connection</t>
+  </si>
+  <si>
+    <t>currently Intel Arc GPU drivers have several issues affecting performance and stability</t>
+  </si>
+  <si>
+    <t>some of the Radeon RX 7900 XT and 7900 XTX currently having high junction temperature issues; AMD has acknowledged them and replace them under warranty</t>
+  </si>
+  <si>
+    <t>low_profile</t>
+  </si>
+  <si>
+    <t>low profile graphics card, should fit a mini-ITX case easily</t>
+  </si>
+  <si>
+    <t>graphics card is very large and may require a case upgrade (over 300 mm in length and/or 60 mm in height)</t>
+  </si>
+  <si>
+    <t>radeon_high_idle_power</t>
+  </si>
+  <si>
+    <t>when connecting to high resolution and high refresh rate monitors (sometimes up to 100 W); this is a known issue and AMD is working on a driver fix for this</t>
+  </si>
+  <si>
+    <t>poor PCI. E 3.0 performance, no hardware encoding ( thus, screen capturing on gpu not supported), only 2 display output ports; it's basically a laptop card turned into a desktop card)</t>
+  </si>
+  <si>
+    <t>positive_score_multiplier</t>
+  </si>
+  <si>
+    <t>negative_score_multiplier</t>
+  </si>
+  <si>
+    <t>overall_score_multiplier</t>
+  </si>
+  <si>
+    <t>overall_additional_score</t>
+  </si>
+  <si>
+    <t>net_tier_score</t>
+  </si>
+  <si>
+    <t>non_rt_positive_score_multiplier</t>
+  </si>
+  <si>
+    <t>non_rt_additional_score</t>
+  </si>
+  <si>
+    <t>non_rt_net_score</t>
+  </si>
+  <si>
+    <t>gpu_name_tpu</t>
+  </si>
+  <si>
+    <t>Geforce GTX 1650 SUPER</t>
+  </si>
+  <si>
+    <t>Geforce GTX 1660 SUPER</t>
+  </si>
+  <si>
+    <t>Geforce RTX 2060 SUPER</t>
+  </si>
+  <si>
     <t>Geforce RTX 3060</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3060 Ti</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3070</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3070 Ti</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3080 10GB</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3080 12GB</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3080 Ti</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3090</t>
-  </si>
-  <si>
-    <t>monster_size</t>
-  </si>
-  <si>
-    <t>Geforce RTX 3090 Ti</t>
-  </si>
-  <si>
-    <t>Geforce RTX 4080</t>
-  </si>
-  <si>
-    <t>rt_3 dlss_2 dlss_3</t>
-  </si>
-  <si>
-    <t>Geforce RTX 4090</t>
-  </si>
-  <si>
-    <t>Geforce RTX 4070 Ti</t>
-  </si>
-  <si>
-    <t>Radeon RX 5500 OEM</t>
-  </si>
-  <si>
-    <t>Radeon RX 5500 XT 4GB</t>
-  </si>
-  <si>
-    <t>Radeon RX 5500 XT 8GB</t>
-  </si>
-  <si>
-    <t>Radeon RX 5600 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 570</t>
-  </si>
-  <si>
-    <t>Radeon RX 5700</t>
-  </si>
-  <si>
-    <t>Radeon RX 5700 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 580</t>
-  </si>
-  <si>
-    <t>Radeon RX 590</t>
-  </si>
-  <si>
-    <t>Radeon RX 6600</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rt_1 </t>
-  </si>
-  <si>
-    <t>Radeon RX 6600 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 6650 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 6700 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 6750 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 6800</t>
-  </si>
-  <si>
-    <t>Radeon RX 6800 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 6900 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 6950 XT</t>
-  </si>
-  <si>
-    <t>Radeon RX 7900 XT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rt_2 </t>
-  </si>
-  <si>
-    <t>radeon_high_temp</t>
-  </si>
-  <si>
-    <t>Radeon RX 7900 XTX</t>
-  </si>
-  <si>
-    <t>comment_code</t>
-  </si>
-  <si>
-    <t>comment_desc</t>
-  </si>
-  <si>
-    <t>weight_score</t>
-  </si>
-  <si>
-    <t>rt_1</t>
-  </si>
-  <si>
-    <t>1st generation ray tracing capabilities or equivalent/limited ray tracing capabilities</t>
-  </si>
-  <si>
-    <t>rt_2</t>
-  </si>
-  <si>
-    <t>2nd generation ray tracing capabilities or equivalent</t>
-  </si>
-  <si>
-    <t>rt_3</t>
-  </si>
-  <si>
-    <t>3rd generation ray tracing capabilities or equivalent</t>
-  </si>
-  <si>
-    <t>dlss_2</t>
-  </si>
-  <si>
-    <t>supports Nvidia's DLSS (Deep Learning Super Sampling) 2 upscaling technology, increasing FPS in supported games</t>
-  </si>
-  <si>
-    <t>dlss_3</t>
-  </si>
-  <si>
-    <t>supports Nvidia's DLSS (Deep Learning Super Sampling) 3.0 upscaling technology, currently the technology can potentially noticably degrade visual quality, and increase input latency unlike DLSS 2</t>
-  </si>
-  <si>
-    <t>low_power</t>
-  </si>
-  <si>
-    <t>low power consumption (just 75 watts), no need for external power connection</t>
-  </si>
-  <si>
-    <t>currently Intel Arc GPU drivers have several issues affecting performance and stability</t>
-  </si>
-  <si>
-    <t>some of the Radeon RX 7900 XT and 7900 XTX currently having high junction temperature issues; AMD has acknowledged them and replace them under warranty</t>
-  </si>
-  <si>
-    <t>low_profile</t>
-  </si>
-  <si>
-    <t>low profile graphics card, should fit a mini-ITX case easily</t>
-  </si>
-  <si>
-    <t>graphics card is very large and may require a case upgrade (over 300 mm in length and/or 60 mm in height)</t>
-  </si>
-  <si>
-    <t>radeon_high_idle_power</t>
-  </si>
-  <si>
-    <t>when connecting to high resolution and high refresh rate monitors (sometimes up to 100 W); this is a known issue and AMD is working on a driver fix for this</t>
-  </si>
-  <si>
-    <t>rx_6500_xt_problems</t>
-  </si>
-  <si>
-    <t>poor PCI. E 3.0 performance, no hardware encoding ( thus, screen capturing on gpu not supported), only 2 display output ports; it's basically a laptop card turned into a desktop card)</t>
-  </si>
-  <si>
-    <t>positive_score_multiplier</t>
-  </si>
-  <si>
-    <t>negative_score_multiplier</t>
-  </si>
-  <si>
-    <t>overall_score_multiplier</t>
-  </si>
-  <si>
-    <t>overall_additional_score</t>
-  </si>
-  <si>
-    <t>net_tier_score</t>
-  </si>
-  <si>
-    <t>non_rt_positive_score_multiplier</t>
-  </si>
-  <si>
-    <t>non_rt_additional_score</t>
-  </si>
-  <si>
-    <t>non_rt_net_score</t>
-  </si>
-  <si>
-    <t>gpu_name_tpu</t>
-  </si>
-  <si>
-    <t>Geforce GTX 1650 SUPER</t>
-  </si>
-  <si>
-    <t>Geforce GTX 1660 SUPER</t>
-  </si>
-  <si>
-    <t>Geforce RTX 2060 SUPER</t>
   </si>
   <si>
     <t>Geforce RTX 2070 SUPER</t>
@@ -740,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G52"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.140625" style="2" bestFit="1" customWidth="1"/>
@@ -785,8 +794,11 @@
       <c r="C2">
         <v>1.21</v>
       </c>
+      <c r="D2" t="s">
+        <v>8</v>
+      </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2">
         <v>140</v>
@@ -797,7 +809,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3">
         <v>281</v>
@@ -805,13 +817,23 @@
       <c r="C3">
         <v>2.81</v>
       </c>
+      <c r="D3" t="s">
+        <v>8</v>
+      </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="F3" s="2">
+        <v>290</v>
+      </c>
+      <c r="G3" s="2">
+        <f>F3*125</f>
+        <v>36250</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4">
         <v>301</v>
@@ -819,13 +841,23 @@
       <c r="C4">
         <v>3.01</v>
       </c>
+      <c r="D4" t="s">
+        <v>8</v>
+      </c>
       <c r="E4" t="s">
-        <v>8</v>
+        <v>9</v>
+      </c>
+      <c r="F4" s="2">
+        <v>350</v>
+      </c>
+      <c r="G4" s="2">
+        <f>F4*125</f>
+        <v>43750</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5">
         <v>100</v>
@@ -842,7 +874,7 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>160</v>
@@ -859,7 +891,7 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7">
         <v>125</v>
@@ -868,7 +900,7 @@
         <v>1.25</v>
       </c>
       <c r="D7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7">
         <v>150</v>
@@ -879,7 +911,7 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B8">
         <v>139</v>
@@ -888,7 +920,7 @@
         <v>1.39</v>
       </c>
       <c r="D8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F8">
         <v>150</v>
@@ -899,7 +931,7 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B9">
         <v>169</v>
@@ -916,7 +948,7 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B10">
         <v>187</v>
@@ -933,7 +965,7 @@
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B11">
         <v>210</v>
@@ -950,7 +982,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B12">
         <v>215</v>
@@ -967,7 +999,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B13">
         <v>253</v>
@@ -976,7 +1008,7 @@
         <v>2.5299999999999998</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F13">
         <v>300</v>
@@ -987,7 +1019,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14">
         <v>284</v>
@@ -996,7 +1028,7 @@
         <v>2.84</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F14">
         <v>400</v>
@@ -1007,7 +1039,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15">
         <v>295</v>
@@ -1024,7 +1056,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B16">
         <v>326</v>
@@ -1033,7 +1065,7 @@
         <v>3.26</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F16">
         <v>500</v>
@@ -1044,7 +1076,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B17">
         <v>350</v>
@@ -1053,7 +1085,7 @@
         <v>3.5</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F17">
         <v>700</v>
@@ -1064,7 +1096,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B18">
         <v>367</v>
@@ -1073,7 +1105,7 @@
         <v>3.67</v>
       </c>
       <c r="D18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F18">
         <v>700</v>
@@ -1084,7 +1116,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B19">
         <v>413</v>
@@ -1093,7 +1125,7 @@
         <v>4.13</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F19">
         <v>1000</v>
@@ -1104,7 +1136,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B20">
         <v>218</v>
@@ -1113,7 +1145,7 @@
         <v>2.1800000000000002</v>
       </c>
       <c r="D20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F20">
         <v>250</v>
@@ -1124,16 +1156,16 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>31</v>
+      </c>
+      <c r="B21">
+        <v>270</v>
+      </c>
+      <c r="C21">
+        <v>2.7</v>
+      </c>
+      <c r="D21" t="s">
         <v>30</v>
-      </c>
-      <c r="B21">
-        <v>301</v>
-      </c>
-      <c r="C21">
-        <v>3.01</v>
-      </c>
-      <c r="D21" t="s">
-        <v>29</v>
       </c>
       <c r="F21">
         <v>330</v>
@@ -1144,142 +1176,139 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B22">
-        <v>376</v>
+        <v>301</v>
       </c>
       <c r="C22">
-        <v>3.76</v>
+        <v>3.01</v>
       </c>
       <c r="D22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F22">
-        <v>400</v>
+        <v>330</v>
       </c>
       <c r="G22">
-        <v>50000</v>
+        <v>41250</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B23">
-        <v>441</v>
+        <v>376</v>
       </c>
       <c r="C23">
-        <v>4.41</v>
+        <v>3.76</v>
       </c>
       <c r="D23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F23">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="G23">
-        <v>62500</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B24">
-        <v>472</v>
+        <v>441</v>
       </c>
       <c r="C24">
-        <v>4.72</v>
+        <v>4.41</v>
       </c>
       <c r="D24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F24">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="G24">
-        <v>75000</v>
+        <v>62500</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B25">
-        <v>546</v>
+        <v>472</v>
       </c>
       <c r="C25">
-        <v>5.46</v>
+        <v>4.72</v>
       </c>
       <c r="D25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F25">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="G25">
-        <v>87500</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B26">
-        <v>573</v>
+        <v>546</v>
       </c>
       <c r="C26">
-        <v>5.73</v>
+        <v>5.46</v>
+      </c>
+      <c r="D26" t="s">
+        <v>30</v>
       </c>
       <c r="F26">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="G26">
-        <v>100000</v>
+        <v>87500</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B27">
-        <v>642</v>
+        <v>573</v>
       </c>
       <c r="C27">
-        <v>6.42</v>
-      </c>
-      <c r="D27" t="s">
-        <v>29</v>
+        <v>5.73</v>
       </c>
       <c r="F27">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="G27">
-        <v>150000</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B28">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="C28">
-        <v>6.48</v>
+        <v>6.42</v>
       </c>
       <c r="D28" t="s">
-        <v>29</v>
-      </c>
-      <c r="E28" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="F28">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="G28">
-        <v>187500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -1287,45 +1316,45 @@
         <v>39</v>
       </c>
       <c r="B29">
-        <v>700</v>
+        <v>648</v>
       </c>
       <c r="C29">
-        <v>7</v>
+        <v>6.48</v>
       </c>
       <c r="D29" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E29" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F29">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="G29">
-        <v>250000</v>
+        <v>187500</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30">
+        <v>700</v>
+      </c>
+      <c r="C30">
+        <v>7</v>
+      </c>
+      <c r="D30" t="s">
+        <v>30</v>
+      </c>
+      <c r="E30" t="s">
         <v>40</v>
       </c>
-      <c r="B30">
-        <v>811</v>
-      </c>
-      <c r="C30">
-        <v>8.11</v>
-      </c>
-      <c r="D30" t="s">
-        <v>41</v>
-      </c>
-      <c r="E30" t="s">
-        <v>38</v>
-      </c>
       <c r="F30">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="G30">
-        <v>150000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
@@ -1333,209 +1362,212 @@
         <v>42</v>
       </c>
       <c r="B31">
-        <v>1014</v>
+        <v>811</v>
       </c>
       <c r="C31">
-        <v>10.14</v>
+        <v>8.11</v>
       </c>
       <c r="D31" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E31" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F31">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="G31">
-        <v>200000</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
+        <v>44</v>
+      </c>
+      <c r="B32">
+        <v>1014</v>
+      </c>
+      <c r="C32">
+        <v>10.14</v>
+      </c>
+      <c r="D32" t="s">
         <v>43</v>
       </c>
-      <c r="B32">
-        <v>668</v>
-      </c>
-      <c r="C32">
-        <v>6.68</v>
-      </c>
-      <c r="D32" t="s">
-        <v>41</v>
+      <c r="E32" t="s">
+        <v>40</v>
       </c>
       <c r="F32">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="G32">
-        <v>100000</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B33">
-        <v>162</v>
+        <v>668</v>
       </c>
       <c r="C33">
-        <v>1.62</v>
+        <v>6.68</v>
+      </c>
+      <c r="D33" t="s">
+        <v>43</v>
+      </c>
+      <c r="F33">
+        <v>800</v>
+      </c>
+      <c r="G33">
+        <v>100000</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B34">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="C34">
-        <v>1.42</v>
-      </c>
-      <c r="F34">
-        <v>170</v>
-      </c>
-      <c r="G34">
-        <v>21250</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B35">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="C35">
-        <v>1.65</v>
+        <v>1.42</v>
       </c>
       <c r="F35">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="G35">
-        <v>25000</v>
+        <v>21250</v>
       </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B36">
-        <v>246</v>
+        <v>165</v>
       </c>
       <c r="C36">
-        <v>2.46</v>
+        <v>1.65</v>
       </c>
       <c r="F36">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="G36">
-        <v>35000</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B37">
-        <v>142</v>
+        <v>246</v>
       </c>
       <c r="C37">
-        <v>1.42</v>
+        <v>2.46</v>
       </c>
       <c r="F37">
-        <v>170</v>
+        <v>280</v>
       </c>
       <c r="G37">
-        <v>21250</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B38">
-        <v>263</v>
+        <v>142</v>
       </c>
       <c r="C38">
-        <v>2.63</v>
+        <v>1.42</v>
       </c>
       <c r="F38">
-        <v>350</v>
+        <v>170</v>
       </c>
       <c r="G38">
-        <v>43750</v>
+        <v>21250</v>
       </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B39">
-        <v>302</v>
+        <v>263</v>
       </c>
       <c r="C39">
-        <v>3.02</v>
+        <v>2.63</v>
       </c>
       <c r="F39">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="G39">
-        <v>50000</v>
+        <v>43750</v>
       </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B40">
-        <v>164</v>
+        <v>302</v>
       </c>
       <c r="C40">
-        <v>1.64</v>
+        <v>3.02</v>
       </c>
       <c r="F40">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="G40">
-        <v>28750</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B41">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="C41">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
       <c r="F41">
-        <v>280</v>
+        <v>230</v>
       </c>
       <c r="G41">
-        <v>35000</v>
+        <v>28750</v>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B42">
-        <v>282</v>
+        <v>177</v>
       </c>
       <c r="C42">
-        <v>2.82</v>
-      </c>
-      <c r="D42" t="s">
-        <v>54</v>
+        <v>1.77</v>
       </c>
       <c r="F42">
-        <v>330</v>
+        <v>280</v>
       </c>
       <c r="G42">
-        <v>41250</v>
+        <v>35000</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
@@ -1543,205 +1575,249 @@
         <v>55</v>
       </c>
       <c r="B43">
-        <v>336</v>
+        <v>282</v>
       </c>
       <c r="C43">
-        <v>3.36</v>
+        <v>2.82</v>
       </c>
       <c r="D43" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F43">
-        <v>380</v>
+        <v>330</v>
       </c>
       <c r="G43">
-        <v>47500</v>
+        <v>41250</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
+        <v>57</v>
+      </c>
+      <c r="B44">
+        <v>336</v>
+      </c>
+      <c r="C44">
+        <v>3.36</v>
+      </c>
+      <c r="D44" t="s">
         <v>56</v>
       </c>
-      <c r="B44">
-        <v>343</v>
-      </c>
-      <c r="C44">
-        <v>3.43</v>
-      </c>
-      <c r="D44" t="s">
-        <v>54</v>
-      </c>
       <c r="F44">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="G44">
-        <v>50000</v>
+        <v>47500</v>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B45">
-        <v>383</v>
+        <v>343</v>
       </c>
       <c r="C45">
-        <v>3.83</v>
+        <v>3.43</v>
       </c>
       <c r="D45" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F45">
-        <v>480</v>
+        <v>400</v>
       </c>
       <c r="G45">
-        <v>60000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B46">
-        <v>414</v>
+        <v>383</v>
       </c>
       <c r="C46">
-        <v>4.1399999999999997</v>
+        <v>3.83</v>
       </c>
       <c r="D46" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F46">
-        <v>550</v>
+        <v>480</v>
       </c>
       <c r="G46">
-        <v>68750</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B47">
-        <v>486</v>
+        <v>414</v>
       </c>
       <c r="C47">
-        <v>4.8600000000000003</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="D47" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F47">
-        <v>580</v>
+        <v>550</v>
       </c>
       <c r="G47">
-        <v>72500</v>
+        <v>68750</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B48">
-        <v>558</v>
+        <v>486</v>
       </c>
       <c r="C48">
-        <v>5.58</v>
+        <v>4.8600000000000003</v>
       </c>
       <c r="D48" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F48">
-        <v>650</v>
+        <v>580</v>
       </c>
       <c r="G48">
-        <v>81250</v>
+        <v>72500</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B49">
-        <v>606</v>
+        <v>558</v>
       </c>
       <c r="C49">
-        <v>6.06</v>
+        <v>5.58</v>
       </c>
       <c r="D49" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F49">
-        <v>1000</v>
+        <v>650</v>
       </c>
       <c r="G49">
-        <v>125000</v>
+        <v>81250</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B50">
-        <v>643</v>
+        <v>606</v>
       </c>
       <c r="C50">
-        <v>6.43</v>
+        <v>6.06</v>
       </c>
       <c r="D50" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F50">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="G50">
-        <v>137500</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B51">
-        <v>706</v>
+        <v>643</v>
       </c>
       <c r="C51">
-        <v>7.06</v>
+        <v>6.43</v>
       </c>
       <c r="D51" t="s">
-        <v>64</v>
-      </c>
-      <c r="E51" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="F51">
-        <v>900</v>
+        <v>1100</v>
       </c>
       <c r="G51">
-        <v>112500</v>
+        <v>137500</v>
       </c>
     </row>
     <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>65</v>
+      </c>
+      <c r="B52">
+        <v>706</v>
+      </c>
+      <c r="C52">
+        <v>7.06</v>
+      </c>
+      <c r="D52" t="s">
         <v>66</v>
       </c>
-      <c r="B52">
+      <c r="E52" t="s">
+        <v>67</v>
+      </c>
+      <c r="F52">
+        <v>900</v>
+      </c>
+      <c r="G52">
+        <v>112500</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>68</v>
+      </c>
+      <c r="B53">
         <v>844</v>
       </c>
-      <c r="C52">
+      <c r="C53">
         <v>8.44</v>
       </c>
-      <c r="D52" t="s">
-        <v>64</v>
-      </c>
-      <c r="E52" t="s">
-        <v>65</v>
-      </c>
-      <c r="F52">
+      <c r="D53" t="s">
+        <v>66</v>
+      </c>
+      <c r="E53" t="s">
+        <v>67</v>
+      </c>
+      <c r="F53">
         <v>1000</v>
       </c>
-      <c r="G52">
+      <c r="G53">
         <v>125000</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>69</v>
+      </c>
+      <c r="B54">
+        <v>166</v>
+      </c>
+      <c r="C54">
+        <v>1.66</v>
+      </c>
+      <c r="D54" t="s">
+        <v>8</v>
+      </c>
+      <c r="E54" t="s">
+        <v>70</v>
+      </c>
+      <c r="F54">
+        <v>200</v>
+      </c>
+      <c r="G54">
+        <f>F54*125</f>
+        <v>25000</v>
       </c>
     </row>
   </sheetData>
@@ -1761,21 +1837,21 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C2">
         <v>5</v>
@@ -1783,10 +1859,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C3">
         <v>10</v>
@@ -1794,10 +1870,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B4" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C4">
         <v>15</v>
@@ -1805,10 +1881,10 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C5">
         <v>7</v>
@@ -1816,10 +1892,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1827,10 +1903,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C7">
         <v>5</v>
@@ -1838,10 +1914,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C8">
         <v>-10</v>
@@ -1849,10 +1925,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C9">
         <v>-5</v>
@@ -1860,10 +1936,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1871,10 +1947,10 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C11">
         <v>-5</v>
@@ -1882,10 +1958,10 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B12" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1893,10 +1969,10 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>89</v>
+        <v>70</v>
       </c>
       <c r="B13" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C13">
         <v>-10</v>
@@ -1909,15 +1985,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P52"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.5703125" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
@@ -1943,28 +2014,28 @@
         <v>6</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.25">
@@ -1980,8 +2051,11 @@
       <c r="D2">
         <v>1.21</v>
       </c>
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G2">
         <v>140</v>
@@ -1990,28 +2064,28 @@
         <v>17500</v>
       </c>
       <c r="I2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J2">
         <v>-0.1</v>
       </c>
       <c r="K2">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="L2">
-        <v>-0.121</v>
+        <v>-6.0499999999999998E-2</v>
       </c>
       <c r="M2">
-        <v>1.089</v>
+        <v>1.1495</v>
       </c>
       <c r="N2">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="O2">
-        <v>-0.121</v>
+        <v>-6.0499999999999998E-2</v>
       </c>
       <c r="P2">
-        <v>1.089</v>
+        <v>1.1495</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.25">
@@ -2019,7 +2093,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C3">
         <v>281</v>
@@ -2027,32 +2101,35 @@
       <c r="D3">
         <v>2.81</v>
       </c>
+      <c r="E3" t="s">
+        <v>8</v>
+      </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I3">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J3">
         <v>-0.1</v>
       </c>
       <c r="K3">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="L3">
-        <v>-0.28100000000000003</v>
+        <v>-0.14050000000000001</v>
       </c>
       <c r="M3">
-        <v>2.5289999999999999</v>
+        <v>2.6695000000000002</v>
       </c>
       <c r="N3">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="O3">
-        <v>-0.28100000000000003</v>
+        <v>-0.14050000000000001</v>
       </c>
       <c r="P3">
-        <v>2.5289999999999999</v>
+        <v>2.6695000000000002</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.25">
@@ -2060,7 +2137,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4">
         <v>301</v>
@@ -2068,32 +2145,35 @@
       <c r="D4">
         <v>3.01</v>
       </c>
+      <c r="E4" t="s">
+        <v>8</v>
+      </c>
       <c r="F4" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J4">
         <v>-0.1</v>
       </c>
       <c r="K4">
-        <v>-0.1</v>
+        <v>-0.05</v>
       </c>
       <c r="L4">
-        <v>-0.30099999999999999</v>
+        <v>-0.15049999999999999</v>
       </c>
       <c r="M4">
-        <v>2.7090000000000001</v>
+        <v>2.8595000000000002</v>
       </c>
       <c r="N4">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="O4">
-        <v>-0.30099999999999999</v>
+        <v>-0.15049999999999999</v>
       </c>
       <c r="P4">
-        <v>2.7090000000000001</v>
+        <v>2.8595000000000002</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.25">
@@ -2101,7 +2181,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C5">
         <v>100</v>
@@ -2145,7 +2225,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C6">
         <v>160</v>
@@ -2189,7 +2269,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7">
         <v>125</v>
@@ -2198,7 +2278,7 @@
         <v>1.25</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G7">
         <v>150</v>
@@ -2236,7 +2316,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C8">
         <v>139</v>
@@ -2245,7 +2325,7 @@
         <v>1.39</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G8">
         <v>150</v>
@@ -2283,7 +2363,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C9">
         <v>169</v>
@@ -2327,7 +2407,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>187</v>
@@ -2371,7 +2451,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C11">
         <v>210</v>
@@ -2415,7 +2495,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C12">
         <v>215</v>
@@ -2459,7 +2539,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13">
         <v>253</v>
@@ -2468,7 +2548,7 @@
         <v>2.5299999999999998</v>
       </c>
       <c r="E13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G13">
         <v>300</v>
@@ -2506,7 +2586,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C14">
         <v>284</v>
@@ -2515,7 +2595,7 @@
         <v>2.84</v>
       </c>
       <c r="E14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G14">
         <v>400</v>
@@ -2553,7 +2633,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C15">
         <v>295</v>
@@ -2597,7 +2677,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C16">
         <v>326</v>
@@ -2606,7 +2686,7 @@
         <v>3.26</v>
       </c>
       <c r="E16" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G16">
         <v>500</v>
@@ -2644,7 +2724,7 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C17">
         <v>350</v>
@@ -2653,7 +2733,7 @@
         <v>3.5</v>
       </c>
       <c r="E17" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G17">
         <v>700</v>
@@ -2691,7 +2771,7 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C18">
         <v>367</v>
@@ -2700,7 +2780,7 @@
         <v>3.67</v>
       </c>
       <c r="E18" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G18">
         <v>700</v>
@@ -2738,7 +2818,7 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C19">
         <v>413</v>
@@ -2747,7 +2827,7 @@
         <v>4.13</v>
       </c>
       <c r="E19" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G19">
         <v>1000</v>
@@ -2785,7 +2865,7 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C20">
         <v>218</v>
@@ -2794,7 +2874,7 @@
         <v>2.1800000000000002</v>
       </c>
       <c r="E20" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G20">
         <v>250</v>
@@ -2832,16 +2912,16 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>31</v>
+      </c>
+      <c r="C21">
+        <v>270</v>
+      </c>
+      <c r="D21">
+        <v>2.7</v>
+      </c>
+      <c r="E21" t="s">
         <v>30</v>
-      </c>
-      <c r="C21">
-        <v>301</v>
-      </c>
-      <c r="D21">
-        <v>3.01</v>
-      </c>
-      <c r="E21" t="s">
-        <v>29</v>
       </c>
       <c r="G21">
         <v>330</v>
@@ -2859,19 +2939,19 @@
         <v>0.17</v>
       </c>
       <c r="L21">
-        <v>0.51170000000000004</v>
+        <v>0.45900000000000007</v>
       </c>
       <c r="M21">
-        <v>3.5217000000000001</v>
+        <v>3.1589999999999998</v>
       </c>
       <c r="N21">
         <v>0.17</v>
       </c>
       <c r="O21">
-        <v>0.51170000000000004</v>
+        <v>0.45900000000000007</v>
       </c>
       <c r="P21">
-        <v>3.5217000000000001</v>
+        <v>3.1589999999999998</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.25">
@@ -2879,22 +2959,22 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C22">
-        <v>376</v>
+        <v>301</v>
       </c>
       <c r="D22">
-        <v>3.76</v>
+        <v>3.01</v>
       </c>
       <c r="E22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G22">
-        <v>400</v>
+        <v>330</v>
       </c>
       <c r="H22">
-        <v>50000</v>
+        <v>41250</v>
       </c>
       <c r="I22">
         <v>0.17</v>
@@ -2906,19 +2986,19 @@
         <v>0.17</v>
       </c>
       <c r="L22">
-        <v>0.63919999999999999</v>
+        <v>0.51170000000000004</v>
       </c>
       <c r="M22">
-        <v>4.3992000000000004</v>
+        <v>3.5217000000000001</v>
       </c>
       <c r="N22">
         <v>0.17</v>
       </c>
       <c r="O22">
-        <v>0.63919999999999999</v>
+        <v>0.51170000000000004</v>
       </c>
       <c r="P22">
-        <v>4.3992000000000004</v>
+        <v>3.5217000000000001</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.25">
@@ -2926,22 +3006,22 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C23">
-        <v>441</v>
+        <v>376</v>
       </c>
       <c r="D23">
-        <v>4.41</v>
+        <v>3.76</v>
       </c>
       <c r="E23" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G23">
-        <v>500</v>
+        <v>400</v>
       </c>
       <c r="H23">
-        <v>62500</v>
+        <v>50000</v>
       </c>
       <c r="I23">
         <v>0.17</v>
@@ -2953,19 +3033,19 @@
         <v>0.17</v>
       </c>
       <c r="L23">
-        <v>0.74970000000000003</v>
+        <v>0.63919999999999999</v>
       </c>
       <c r="M23">
-        <v>5.1597</v>
+        <v>4.3992000000000004</v>
       </c>
       <c r="N23">
         <v>0.17</v>
       </c>
       <c r="O23">
-        <v>0.74970000000000003</v>
+        <v>0.63919999999999999</v>
       </c>
       <c r="P23">
-        <v>5.1597</v>
+        <v>4.3992000000000004</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.25">
@@ -2973,22 +3053,22 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C24">
-        <v>472</v>
+        <v>441</v>
       </c>
       <c r="D24">
-        <v>4.72</v>
+        <v>4.41</v>
       </c>
       <c r="E24" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G24">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="H24">
-        <v>75000</v>
+        <v>62500</v>
       </c>
       <c r="I24">
         <v>0.17</v>
@@ -3000,19 +3080,19 @@
         <v>0.17</v>
       </c>
       <c r="L24">
-        <v>0.8024</v>
+        <v>0.74970000000000003</v>
       </c>
       <c r="M24">
-        <v>5.5223999999999993</v>
+        <v>5.1597</v>
       </c>
       <c r="N24">
         <v>0.17</v>
       </c>
       <c r="O24">
-        <v>0.8024</v>
+        <v>0.74970000000000003</v>
       </c>
       <c r="P24">
-        <v>5.5223999999999993</v>
+        <v>5.1597</v>
       </c>
     </row>
     <row r="25" spans="1:16" x14ac:dyDescent="0.25">
@@ -3020,22 +3100,22 @@
         <v>23</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C25">
-        <v>546</v>
+        <v>472</v>
       </c>
       <c r="D25">
-        <v>5.46</v>
+        <v>4.72</v>
       </c>
       <c r="E25" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G25">
-        <v>700</v>
+        <v>600</v>
       </c>
       <c r="H25">
-        <v>87500</v>
+        <v>75000</v>
       </c>
       <c r="I25">
         <v>0.17</v>
@@ -3047,19 +3127,19 @@
         <v>0.17</v>
       </c>
       <c r="L25">
-        <v>0.92820000000000003</v>
+        <v>0.8024</v>
       </c>
       <c r="M25">
-        <v>6.3882000000000003</v>
+        <v>5.5223999999999993</v>
       </c>
       <c r="N25">
         <v>0.17</v>
       </c>
       <c r="O25">
-        <v>0.92820000000000003</v>
+        <v>0.8024</v>
       </c>
       <c r="P25">
-        <v>6.3882000000000003</v>
+        <v>5.5223999999999993</v>
       </c>
     </row>
     <row r="26" spans="1:16" x14ac:dyDescent="0.25">
@@ -3067,43 +3147,46 @@
         <v>24</v>
       </c>
       <c r="B26" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C26">
-        <v>573</v>
+        <v>546</v>
       </c>
       <c r="D26">
-        <v>5.73</v>
+        <v>5.46</v>
+      </c>
+      <c r="E26" t="s">
+        <v>30</v>
       </c>
       <c r="G26">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="H26">
-        <v>100000</v>
+        <v>87500</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="J26">
         <v>0</v>
       </c>
       <c r="K26">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="L26">
-        <v>0</v>
+        <v>0.92820000000000003</v>
       </c>
       <c r="M26">
-        <v>5.73</v>
+        <v>6.3882000000000003</v>
       </c>
       <c r="N26">
-        <v>0</v>
+        <v>0.17</v>
       </c>
       <c r="O26">
-        <v>0</v>
+        <v>0.92820000000000003</v>
       </c>
       <c r="P26">
-        <v>5.73</v>
+        <v>6.3882000000000003</v>
       </c>
     </row>
     <row r="27" spans="1:16" x14ac:dyDescent="0.25">
@@ -3111,46 +3194,43 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C27">
-        <v>642</v>
+        <v>573</v>
       </c>
       <c r="D27">
-        <v>6.42</v>
-      </c>
-      <c r="E27" t="s">
-        <v>29</v>
+        <v>5.73</v>
       </c>
       <c r="G27">
-        <v>1200</v>
+        <v>800</v>
       </c>
       <c r="H27">
-        <v>150000</v>
+        <v>100000</v>
       </c>
       <c r="I27">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="J27">
         <v>0</v>
       </c>
       <c r="K27">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="L27">
-        <v>1.0913999999999999</v>
+        <v>0</v>
       </c>
       <c r="M27">
-        <v>7.5114000000000001</v>
+        <v>5.73</v>
       </c>
       <c r="N27">
-        <v>0.17</v>
+        <v>0</v>
       </c>
       <c r="O27">
-        <v>1.0913999999999999</v>
+        <v>0</v>
       </c>
       <c r="P27">
-        <v>7.5114000000000001</v>
+        <v>5.73</v>
       </c>
     </row>
     <row r="28" spans="1:16" x14ac:dyDescent="0.25">
@@ -3158,49 +3238,46 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C28">
-        <v>648</v>
+        <v>642</v>
       </c>
       <c r="D28">
-        <v>6.48</v>
+        <v>6.42</v>
       </c>
       <c r="E28" t="s">
-        <v>29</v>
-      </c>
-      <c r="F28" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="G28">
-        <v>1500</v>
+        <v>1200</v>
       </c>
       <c r="H28">
-        <v>187500</v>
+        <v>150000</v>
       </c>
       <c r="I28">
         <v>0.17</v>
       </c>
       <c r="J28">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="K28">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="L28">
-        <v>0.77760000000000007</v>
+        <v>1.0913999999999999</v>
       </c>
       <c r="M28">
-        <v>7.2576000000000001</v>
+        <v>7.5114000000000001</v>
       </c>
       <c r="N28">
         <v>0.17</v>
       </c>
       <c r="O28">
-        <v>0.77760000000000007</v>
+        <v>1.0913999999999999</v>
       </c>
       <c r="P28">
-        <v>7.2576000000000001</v>
+        <v>7.5114000000000001</v>
       </c>
     </row>
     <row r="29" spans="1:16" x14ac:dyDescent="0.25">
@@ -3211,22 +3288,22 @@
         <v>39</v>
       </c>
       <c r="C29">
-        <v>700</v>
+        <v>648</v>
       </c>
       <c r="D29">
-        <v>7</v>
+        <v>6.48</v>
       </c>
       <c r="E29" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F29" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G29">
-        <v>2000</v>
+        <v>1500</v>
       </c>
       <c r="H29">
-        <v>250000</v>
+        <v>187500</v>
       </c>
       <c r="I29">
         <v>0.17</v>
@@ -3238,19 +3315,19 @@
         <v>0.12</v>
       </c>
       <c r="L29">
-        <v>0.84000000000000008</v>
+        <v>0.77760000000000007</v>
       </c>
       <c r="M29">
-        <v>7.84</v>
+        <v>7.2576000000000001</v>
       </c>
       <c r="N29">
         <v>0.17</v>
       </c>
       <c r="O29">
-        <v>0.84000000000000008</v>
+        <v>0.77760000000000007</v>
       </c>
       <c r="P29">
-        <v>7.84</v>
+        <v>7.2576000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:16" x14ac:dyDescent="0.25">
@@ -3258,49 +3335,49 @@
         <v>28</v>
       </c>
       <c r="B30" t="s">
+        <v>41</v>
+      </c>
+      <c r="C30">
+        <v>700</v>
+      </c>
+      <c r="D30">
+        <v>7</v>
+      </c>
+      <c r="E30" t="s">
+        <v>30</v>
+      </c>
+      <c r="F30" t="s">
         <v>40</v>
       </c>
-      <c r="C30">
-        <v>811</v>
-      </c>
-      <c r="D30">
-        <v>8.11</v>
-      </c>
-      <c r="E30" t="s">
-        <v>41</v>
-      </c>
-      <c r="F30" t="s">
-        <v>38</v>
-      </c>
       <c r="G30">
-        <v>1200</v>
+        <v>2000</v>
       </c>
       <c r="H30">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="I30">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="J30">
         <v>-0.05</v>
       </c>
       <c r="K30">
+        <v>0.12</v>
+      </c>
+      <c r="L30">
+        <v>0.84000000000000008</v>
+      </c>
+      <c r="M30">
+        <v>7.84</v>
+      </c>
+      <c r="N30">
         <v>0.17</v>
       </c>
-      <c r="L30">
-        <v>1.3787</v>
-      </c>
-      <c r="M30">
-        <v>9.4886999999999997</v>
-      </c>
-      <c r="N30">
-        <v>0.22</v>
-      </c>
       <c r="O30">
-        <v>1.3787</v>
+        <v>0.84000000000000008</v>
       </c>
       <c r="P30">
-        <v>9.4886999999999997</v>
+        <v>7.84</v>
       </c>
     </row>
     <row r="31" spans="1:16" x14ac:dyDescent="0.25">
@@ -3311,22 +3388,22 @@
         <v>42</v>
       </c>
       <c r="C31">
-        <v>1014</v>
+        <v>811</v>
       </c>
       <c r="D31">
-        <v>10.14</v>
+        <v>8.11</v>
       </c>
       <c r="E31" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F31" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G31">
-        <v>1600</v>
+        <v>1200</v>
       </c>
       <c r="H31">
-        <v>200000</v>
+        <v>150000</v>
       </c>
       <c r="I31">
         <v>0.22</v>
@@ -3338,19 +3415,19 @@
         <v>0.17</v>
       </c>
       <c r="L31">
-        <v>1.7238</v>
+        <v>1.3787</v>
       </c>
       <c r="M31">
-        <v>11.863799999999999</v>
+        <v>9.4886999999999997</v>
       </c>
       <c r="N31">
         <v>0.22</v>
       </c>
       <c r="O31">
-        <v>1.7238</v>
+        <v>1.3787</v>
       </c>
       <c r="P31">
-        <v>11.863799999999999</v>
+        <v>9.4886999999999997</v>
       </c>
     </row>
     <row r="32" spans="1:16" x14ac:dyDescent="0.25">
@@ -3358,46 +3435,49 @@
         <v>30</v>
       </c>
       <c r="B32" t="s">
+        <v>44</v>
+      </c>
+      <c r="C32">
+        <v>1014</v>
+      </c>
+      <c r="D32">
+        <v>10.14</v>
+      </c>
+      <c r="E32" t="s">
         <v>43</v>
       </c>
-      <c r="C32">
-        <v>668</v>
-      </c>
-      <c r="D32">
-        <v>6.68</v>
-      </c>
-      <c r="E32" t="s">
-        <v>41</v>
+      <c r="F32" t="s">
+        <v>40</v>
       </c>
       <c r="G32">
-        <v>800</v>
+        <v>1600</v>
       </c>
       <c r="H32">
-        <v>100000</v>
+        <v>200000</v>
       </c>
       <c r="I32">
         <v>0.22</v>
       </c>
       <c r="J32">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="K32">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="L32">
-        <v>1.4696</v>
+        <v>1.7238</v>
       </c>
       <c r="M32">
-        <v>8.1495999999999995</v>
+        <v>11.863799999999999</v>
       </c>
       <c r="N32">
         <v>0.22</v>
       </c>
       <c r="O32">
-        <v>1.4696</v>
+        <v>1.7238</v>
       </c>
       <c r="P32">
-        <v>8.1495999999999995</v>
+        <v>11.863799999999999</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.25">
@@ -3405,37 +3485,46 @@
         <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C33">
-        <v>162</v>
+        <v>668</v>
       </c>
       <c r="D33">
-        <v>1.62</v>
+        <v>6.68</v>
+      </c>
+      <c r="E33" t="s">
+        <v>43</v>
+      </c>
+      <c r="G33">
+        <v>800</v>
+      </c>
+      <c r="H33">
+        <v>100000</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="J33">
         <v>0</v>
       </c>
       <c r="K33">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="L33">
-        <v>0</v>
+        <v>1.4696</v>
       </c>
       <c r="M33">
-        <v>1.62</v>
+        <v>8.1495999999999995</v>
       </c>
       <c r="N33">
-        <v>0</v>
+        <v>0.22</v>
       </c>
       <c r="O33">
-        <v>0</v>
+        <v>1.4696</v>
       </c>
       <c r="P33">
-        <v>1.62</v>
+        <v>8.1495999999999995</v>
       </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.25">
@@ -3443,19 +3532,13 @@
         <v>32</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C34">
-        <v>142</v>
+        <v>162</v>
       </c>
       <c r="D34">
-        <v>1.42</v>
-      </c>
-      <c r="G34">
-        <v>170</v>
-      </c>
-      <c r="H34">
-        <v>21250</v>
+        <v>1.62</v>
       </c>
       <c r="I34">
         <v>0</v>
@@ -3470,7 +3553,7 @@
         <v>0</v>
       </c>
       <c r="M34">
-        <v>1.42</v>
+        <v>1.62</v>
       </c>
       <c r="N34">
         <v>0</v>
@@ -3479,7 +3562,7 @@
         <v>0</v>
       </c>
       <c r="P34">
-        <v>1.42</v>
+        <v>1.62</v>
       </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.25">
@@ -3487,19 +3570,19 @@
         <v>33</v>
       </c>
       <c r="B35" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C35">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="D35">
-        <v>1.65</v>
+        <v>1.42</v>
       </c>
       <c r="G35">
-        <v>200</v>
+        <v>170</v>
       </c>
       <c r="H35">
-        <v>25000</v>
+        <v>21250</v>
       </c>
       <c r="I35">
         <v>0</v>
@@ -3514,7 +3597,7 @@
         <v>0</v>
       </c>
       <c r="M35">
-        <v>1.65</v>
+        <v>1.42</v>
       </c>
       <c r="N35">
         <v>0</v>
@@ -3523,7 +3606,7 @@
         <v>0</v>
       </c>
       <c r="P35">
-        <v>1.65</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.25">
@@ -3531,19 +3614,19 @@
         <v>34</v>
       </c>
       <c r="B36" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C36">
-        <v>246</v>
+        <v>165</v>
       </c>
       <c r="D36">
-        <v>2.46</v>
+        <v>1.65</v>
       </c>
       <c r="G36">
-        <v>280</v>
+        <v>200</v>
       </c>
       <c r="H36">
-        <v>35000</v>
+        <v>25000</v>
       </c>
       <c r="I36">
         <v>0</v>
@@ -3558,7 +3641,7 @@
         <v>0</v>
       </c>
       <c r="M36">
-        <v>2.46</v>
+        <v>1.65</v>
       </c>
       <c r="N36">
         <v>0</v>
@@ -3567,7 +3650,7 @@
         <v>0</v>
       </c>
       <c r="P36">
-        <v>2.46</v>
+        <v>1.65</v>
       </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.25">
@@ -3575,19 +3658,19 @@
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C37">
-        <v>142</v>
+        <v>246</v>
       </c>
       <c r="D37">
-        <v>1.42</v>
+        <v>2.46</v>
       </c>
       <c r="G37">
-        <v>170</v>
+        <v>280</v>
       </c>
       <c r="H37">
-        <v>21250</v>
+        <v>35000</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -3602,7 +3685,7 @@
         <v>0</v>
       </c>
       <c r="M37">
-        <v>1.42</v>
+        <v>2.46</v>
       </c>
       <c r="N37">
         <v>0</v>
@@ -3611,7 +3694,7 @@
         <v>0</v>
       </c>
       <c r="P37">
-        <v>1.42</v>
+        <v>2.46</v>
       </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.25">
@@ -3619,19 +3702,19 @@
         <v>36</v>
       </c>
       <c r="B38" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C38">
-        <v>263</v>
+        <v>142</v>
       </c>
       <c r="D38">
-        <v>2.63</v>
+        <v>1.42</v>
       </c>
       <c r="G38">
-        <v>350</v>
+        <v>170</v>
       </c>
       <c r="H38">
-        <v>43750</v>
+        <v>21250</v>
       </c>
       <c r="I38">
         <v>0</v>
@@ -3646,7 +3729,7 @@
         <v>0</v>
       </c>
       <c r="M38">
-        <v>2.63</v>
+        <v>1.42</v>
       </c>
       <c r="N38">
         <v>0</v>
@@ -3655,7 +3738,7 @@
         <v>0</v>
       </c>
       <c r="P38">
-        <v>2.63</v>
+        <v>1.42</v>
       </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.25">
@@ -3663,19 +3746,19 @@
         <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C39">
-        <v>302</v>
+        <v>263</v>
       </c>
       <c r="D39">
-        <v>3.02</v>
+        <v>2.63</v>
       </c>
       <c r="G39">
-        <v>400</v>
+        <v>350</v>
       </c>
       <c r="H39">
-        <v>50000</v>
+        <v>43750</v>
       </c>
       <c r="I39">
         <v>0</v>
@@ -3690,7 +3773,7 @@
         <v>0</v>
       </c>
       <c r="M39">
-        <v>3.02</v>
+        <v>2.63</v>
       </c>
       <c r="N39">
         <v>0</v>
@@ -3699,7 +3782,7 @@
         <v>0</v>
       </c>
       <c r="P39">
-        <v>3.02</v>
+        <v>2.63</v>
       </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.25">
@@ -3707,19 +3790,19 @@
         <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C40">
-        <v>164</v>
+        <v>302</v>
       </c>
       <c r="D40">
-        <v>1.64</v>
+        <v>3.02</v>
       </c>
       <c r="G40">
-        <v>230</v>
+        <v>400</v>
       </c>
       <c r="H40">
-        <v>28750</v>
+        <v>50000</v>
       </c>
       <c r="I40">
         <v>0</v>
@@ -3734,7 +3817,7 @@
         <v>0</v>
       </c>
       <c r="M40">
-        <v>1.64</v>
+        <v>3.02</v>
       </c>
       <c r="N40">
         <v>0</v>
@@ -3743,7 +3826,7 @@
         <v>0</v>
       </c>
       <c r="P40">
-        <v>1.64</v>
+        <v>3.02</v>
       </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.25">
@@ -3751,19 +3834,19 @@
         <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C41">
-        <v>177</v>
+        <v>164</v>
       </c>
       <c r="D41">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
       <c r="G41">
-        <v>280</v>
+        <v>230</v>
       </c>
       <c r="H41">
-        <v>35000</v>
+        <v>28750</v>
       </c>
       <c r="I41">
         <v>0</v>
@@ -3778,7 +3861,7 @@
         <v>0</v>
       </c>
       <c r="M41">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
       <c r="N41">
         <v>0</v>
@@ -3787,7 +3870,7 @@
         <v>0</v>
       </c>
       <c r="P41">
-        <v>1.77</v>
+        <v>1.64</v>
       </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.25">
@@ -3795,46 +3878,43 @@
         <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C42">
-        <v>282</v>
+        <v>177</v>
       </c>
       <c r="D42">
-        <v>2.82</v>
-      </c>
-      <c r="E42" t="s">
-        <v>54</v>
+        <v>1.77</v>
       </c>
       <c r="G42">
-        <v>330</v>
+        <v>280</v>
       </c>
       <c r="H42">
-        <v>41250</v>
+        <v>35000</v>
       </c>
       <c r="I42">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J42">
         <v>0</v>
       </c>
       <c r="K42">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="L42">
-        <v>0.14099999999999999</v>
+        <v>0</v>
       </c>
       <c r="M42">
-        <v>2.9609999999999999</v>
+        <v>1.77</v>
       </c>
       <c r="N42">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="O42">
-        <v>0.14099999999999999</v>
+        <v>0</v>
       </c>
       <c r="P42">
-        <v>2.9609999999999999</v>
+        <v>1.77</v>
       </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.25">
@@ -3845,19 +3925,19 @@
         <v>55</v>
       </c>
       <c r="C43">
-        <v>336</v>
+        <v>282</v>
       </c>
       <c r="D43">
-        <v>3.36</v>
+        <v>2.82</v>
       </c>
       <c r="E43" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G43">
-        <v>380</v>
+        <v>330</v>
       </c>
       <c r="H43">
-        <v>47500</v>
+        <v>41250</v>
       </c>
       <c r="I43">
         <v>0.05</v>
@@ -3869,19 +3949,19 @@
         <v>0.05</v>
       </c>
       <c r="L43">
-        <v>0.16800000000000001</v>
+        <v>0.14099999999999999</v>
       </c>
       <c r="M43">
-        <v>3.528</v>
+        <v>2.9609999999999999</v>
       </c>
       <c r="N43">
         <v>0.05</v>
       </c>
       <c r="O43">
-        <v>0.16800000000000001</v>
+        <v>0.14099999999999999</v>
       </c>
       <c r="P43">
-        <v>3.528</v>
+        <v>2.9609999999999999</v>
       </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.25">
@@ -3889,22 +3969,22 @@
         <v>42</v>
       </c>
       <c r="B44" t="s">
+        <v>57</v>
+      </c>
+      <c r="C44">
+        <v>336</v>
+      </c>
+      <c r="D44">
+        <v>3.36</v>
+      </c>
+      <c r="E44" t="s">
         <v>56</v>
       </c>
-      <c r="C44">
-        <v>343</v>
-      </c>
-      <c r="D44">
-        <v>3.43</v>
-      </c>
-      <c r="E44" t="s">
-        <v>54</v>
-      </c>
       <c r="G44">
-        <v>400</v>
+        <v>380</v>
       </c>
       <c r="H44">
-        <v>50000</v>
+        <v>47500</v>
       </c>
       <c r="I44">
         <v>0.05</v>
@@ -3916,19 +3996,19 @@
         <v>0.05</v>
       </c>
       <c r="L44">
-        <v>0.17150000000000001</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="M44">
-        <v>3.6015000000000001</v>
+        <v>3.528</v>
       </c>
       <c r="N44">
         <v>0.05</v>
       </c>
       <c r="O44">
-        <v>0.17150000000000001</v>
+        <v>0.16800000000000001</v>
       </c>
       <c r="P44">
-        <v>3.6015000000000001</v>
+        <v>3.528</v>
       </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.25">
@@ -3936,22 +4016,22 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C45">
-        <v>383</v>
+        <v>343</v>
       </c>
       <c r="D45">
-        <v>3.83</v>
+        <v>3.43</v>
       </c>
       <c r="E45" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G45">
-        <v>480</v>
+        <v>400</v>
       </c>
       <c r="H45">
-        <v>60000</v>
+        <v>50000</v>
       </c>
       <c r="I45">
         <v>0.05</v>
@@ -3963,19 +4043,19 @@
         <v>0.05</v>
       </c>
       <c r="L45">
-        <v>0.1915</v>
+        <v>0.17150000000000001</v>
       </c>
       <c r="M45">
-        <v>4.0214999999999996</v>
+        <v>3.6015000000000001</v>
       </c>
       <c r="N45">
         <v>0.05</v>
       </c>
       <c r="O45">
-        <v>0.1915</v>
+        <v>0.17150000000000001</v>
       </c>
       <c r="P45">
-        <v>4.0214999999999996</v>
+        <v>3.6015000000000001</v>
       </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.25">
@@ -3983,22 +4063,22 @@
         <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C46">
-        <v>414</v>
+        <v>383</v>
       </c>
       <c r="D46">
-        <v>4.1399999999999997</v>
+        <v>3.83</v>
       </c>
       <c r="E46" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G46">
-        <v>550</v>
+        <v>480</v>
       </c>
       <c r="H46">
-        <v>68750</v>
+        <v>60000</v>
       </c>
       <c r="I46">
         <v>0.05</v>
@@ -4010,19 +4090,19 @@
         <v>0.05</v>
       </c>
       <c r="L46">
-        <v>0.20699999999999999</v>
+        <v>0.1915</v>
       </c>
       <c r="M46">
-        <v>4.3470000000000004</v>
+        <v>4.0214999999999996</v>
       </c>
       <c r="N46">
         <v>0.05</v>
       </c>
       <c r="O46">
-        <v>0.20699999999999999</v>
+        <v>0.1915</v>
       </c>
       <c r="P46">
-        <v>4.3470000000000004</v>
+        <v>4.0214999999999996</v>
       </c>
     </row>
     <row r="47" spans="1:16" x14ac:dyDescent="0.25">
@@ -4030,22 +4110,22 @@
         <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C47">
-        <v>486</v>
+        <v>414</v>
       </c>
       <c r="D47">
-        <v>4.8600000000000003</v>
+        <v>4.1399999999999997</v>
       </c>
       <c r="E47" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G47">
-        <v>580</v>
+        <v>550</v>
       </c>
       <c r="H47">
-        <v>72500</v>
+        <v>68750</v>
       </c>
       <c r="I47">
         <v>0.05</v>
@@ -4057,19 +4137,19 @@
         <v>0.05</v>
       </c>
       <c r="L47">
-        <v>0.24299999999999999</v>
+        <v>0.20699999999999999</v>
       </c>
       <c r="M47">
-        <v>5.1030000000000006</v>
+        <v>4.3470000000000004</v>
       </c>
       <c r="N47">
         <v>0.05</v>
       </c>
       <c r="O47">
-        <v>0.24299999999999999</v>
+        <v>0.20699999999999999</v>
       </c>
       <c r="P47">
-        <v>5.1030000000000006</v>
+        <v>4.3470000000000004</v>
       </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.25">
@@ -4077,22 +4157,22 @@
         <v>46</v>
       </c>
       <c r="B48" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C48">
-        <v>558</v>
+        <v>486</v>
       </c>
       <c r="D48">
-        <v>5.58</v>
+        <v>4.8600000000000003</v>
       </c>
       <c r="E48" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G48">
-        <v>650</v>
+        <v>580</v>
       </c>
       <c r="H48">
-        <v>81250</v>
+        <v>72500</v>
       </c>
       <c r="I48">
         <v>0.05</v>
@@ -4104,19 +4184,19 @@
         <v>0.05</v>
       </c>
       <c r="L48">
-        <v>0.27900000000000003</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="M48">
-        <v>5.859</v>
+        <v>5.1030000000000006</v>
       </c>
       <c r="N48">
         <v>0.05</v>
       </c>
       <c r="O48">
-        <v>0.27900000000000003</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="P48">
-        <v>5.859</v>
+        <v>5.1030000000000006</v>
       </c>
     </row>
     <row r="49" spans="1:16" x14ac:dyDescent="0.25">
@@ -4124,22 +4204,22 @@
         <v>47</v>
       </c>
       <c r="B49" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C49">
-        <v>606</v>
+        <v>558</v>
       </c>
       <c r="D49">
-        <v>6.06</v>
+        <v>5.58</v>
       </c>
       <c r="E49" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G49">
-        <v>1000</v>
+        <v>650</v>
       </c>
       <c r="H49">
-        <v>125000</v>
+        <v>81250</v>
       </c>
       <c r="I49">
         <v>0.05</v>
@@ -4151,19 +4231,19 @@
         <v>0.05</v>
       </c>
       <c r="L49">
-        <v>0.30299999999999999</v>
+        <v>0.27900000000000003</v>
       </c>
       <c r="M49">
-        <v>6.3630000000000004</v>
+        <v>5.859</v>
       </c>
       <c r="N49">
         <v>0.05</v>
       </c>
       <c r="O49">
-        <v>0.30299999999999999</v>
+        <v>0.27900000000000003</v>
       </c>
       <c r="P49">
-        <v>6.3630000000000004</v>
+        <v>5.859</v>
       </c>
     </row>
     <row r="50" spans="1:16" x14ac:dyDescent="0.25">
@@ -4171,22 +4251,22 @@
         <v>48</v>
       </c>
       <c r="B50" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C50">
-        <v>643</v>
+        <v>606</v>
       </c>
       <c r="D50">
-        <v>6.43</v>
+        <v>6.06</v>
       </c>
       <c r="E50" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G50">
-        <v>1100</v>
+        <v>1000</v>
       </c>
       <c r="H50">
-        <v>137500</v>
+        <v>125000</v>
       </c>
       <c r="I50">
         <v>0.05</v>
@@ -4198,19 +4278,19 @@
         <v>0.05</v>
       </c>
       <c r="L50">
-        <v>0.32150000000000001</v>
+        <v>0.30299999999999999</v>
       </c>
       <c r="M50">
-        <v>6.7515000000000001</v>
+        <v>6.3630000000000004</v>
       </c>
       <c r="N50">
         <v>0.05</v>
       </c>
       <c r="O50">
-        <v>0.32150000000000001</v>
+        <v>0.30299999999999999</v>
       </c>
       <c r="P50">
-        <v>6.7515000000000001</v>
+        <v>6.3630000000000004</v>
       </c>
     </row>
     <row r="51" spans="1:16" x14ac:dyDescent="0.25">
@@ -4218,49 +4298,46 @@
         <v>49</v>
       </c>
       <c r="B51" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C51">
-        <v>706</v>
+        <v>643</v>
       </c>
       <c r="D51">
-        <v>7.06</v>
+        <v>6.43</v>
       </c>
       <c r="E51" t="s">
-        <v>64</v>
-      </c>
-      <c r="F51" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="G51">
-        <v>900</v>
+        <v>1100</v>
       </c>
       <c r="H51">
-        <v>112500</v>
+        <v>137500</v>
       </c>
       <c r="I51">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="J51">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="K51">
         <v>0.05</v>
       </c>
       <c r="L51">
-        <v>0.35299999999999998</v>
+        <v>0.32150000000000001</v>
       </c>
       <c r="M51">
-        <v>7.4129999999999994</v>
+        <v>6.7515000000000001</v>
       </c>
       <c r="N51">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="O51">
-        <v>0.35299999999999998</v>
+        <v>0.32150000000000001</v>
       </c>
       <c r="P51">
-        <v>7.4129999999999994</v>
+        <v>6.7515000000000001</v>
       </c>
     </row>
     <row r="52" spans="1:16" x14ac:dyDescent="0.25">
@@ -4268,25 +4345,25 @@
         <v>50</v>
       </c>
       <c r="B52" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52">
+        <v>706</v>
+      </c>
+      <c r="D52">
+        <v>7.06</v>
+      </c>
+      <c r="E52" t="s">
         <v>66</v>
       </c>
-      <c r="C52">
-        <v>844</v>
-      </c>
-      <c r="D52">
-        <v>8.44</v>
-      </c>
-      <c r="E52" t="s">
-        <v>64</v>
-      </c>
       <c r="F52" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G52">
-        <v>1000</v>
+        <v>900</v>
       </c>
       <c r="H52">
-        <v>125000</v>
+        <v>112500</v>
       </c>
       <c r="I52">
         <v>0.1</v>
@@ -4298,19 +4375,119 @@
         <v>0.05</v>
       </c>
       <c r="L52">
-        <v>0.42199999999999999</v>
+        <v>0.35299999999999998</v>
       </c>
       <c r="M52">
-        <v>8.8620000000000001</v>
+        <v>7.4129999999999994</v>
       </c>
       <c r="N52">
         <v>0.1</v>
       </c>
       <c r="O52">
+        <v>0.35299999999999998</v>
+      </c>
+      <c r="P52">
+        <v>7.4129999999999994</v>
+      </c>
+    </row>
+    <row r="53" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A53" s="5">
+        <v>51</v>
+      </c>
+      <c r="B53" t="s">
+        <v>68</v>
+      </c>
+      <c r="C53">
+        <v>844</v>
+      </c>
+      <c r="D53">
+        <v>8.44</v>
+      </c>
+      <c r="E53" t="s">
+        <v>66</v>
+      </c>
+      <c r="F53" t="s">
+        <v>67</v>
+      </c>
+      <c r="G53">
+        <v>1000</v>
+      </c>
+      <c r="H53">
+        <v>125000</v>
+      </c>
+      <c r="I53">
+        <v>0.1</v>
+      </c>
+      <c r="J53">
+        <v>-0.05</v>
+      </c>
+      <c r="K53">
+        <v>0.05</v>
+      </c>
+      <c r="L53">
         <v>0.42199999999999999</v>
       </c>
-      <c r="P52">
+      <c r="M53">
         <v>8.8620000000000001</v>
+      </c>
+      <c r="N53">
+        <v>0.1</v>
+      </c>
+      <c r="O53">
+        <v>0.42199999999999999</v>
+      </c>
+      <c r="P53">
+        <v>8.8620000000000001</v>
+      </c>
+    </row>
+    <row r="54" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A54" s="5">
+        <v>52</v>
+      </c>
+      <c r="B54" t="s">
+        <v>69</v>
+      </c>
+      <c r="C54">
+        <v>166</v>
+      </c>
+      <c r="D54">
+        <v>1.66</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="F54" t="s">
+        <v>70</v>
+      </c>
+      <c r="G54">
+        <v>200</v>
+      </c>
+      <c r="H54">
+        <v>25000</v>
+      </c>
+      <c r="I54">
+        <v>0.05</v>
+      </c>
+      <c r="J54">
+        <v>-0.1</v>
+      </c>
+      <c r="K54">
+        <v>-0.05</v>
+      </c>
+      <c r="L54">
+        <v>-8.3000000000000004E-2</v>
+      </c>
+      <c r="M54">
+        <v>1.577</v>
+      </c>
+      <c r="N54">
+        <v>0.05</v>
+      </c>
+      <c r="O54">
+        <v>-8.3000000000000004E-2</v>
+      </c>
+      <c r="P54">
+        <v>1.577</v>
       </c>
     </row>
   </sheetData>
@@ -4332,7 +4509,7 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -4352,7 +4529,7 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2">
         <v>100</v>
@@ -4386,7 +4563,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B4">
         <v>125</v>
@@ -4403,7 +4580,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>139</v>
@@ -4420,7 +4597,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B6">
         <v>142</v>
@@ -4437,7 +4614,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B7">
         <v>142</v>
@@ -4454,7 +4631,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>160</v>
@@ -4471,7 +4648,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B9">
         <v>162</v>
@@ -4482,7 +4659,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B10">
         <v>164</v>
@@ -4499,7 +4676,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B11">
         <v>165</v>
@@ -4516,7 +4693,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B12">
         <v>169</v>
@@ -4533,7 +4710,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B13">
         <v>177</v>
@@ -4550,7 +4727,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>187</v>
@@ -4567,7 +4744,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B15">
         <v>210</v>
@@ -4584,7 +4761,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B16">
         <v>215</v>
@@ -4601,7 +4778,7 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17">
         <v>218</v>
@@ -4618,7 +4795,7 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B18">
         <v>246</v>
@@ -4635,7 +4812,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B19">
         <v>253</v>
@@ -4652,7 +4829,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B20">
         <v>263</v>
@@ -4669,7 +4846,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B21">
         <v>281</v>
@@ -4680,7 +4857,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B22">
         <v>282</v>
@@ -4697,7 +4874,7 @@
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B23">
         <v>284</v>
@@ -4714,7 +4891,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B24">
         <v>295</v>
@@ -4731,7 +4908,7 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B25">
         <v>301</v>
@@ -4742,7 +4919,7 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>30</v>
+        <v>105</v>
       </c>
       <c r="B26">
         <v>301</v>
@@ -4759,7 +4936,7 @@
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B27">
         <v>302</v>
@@ -4776,7 +4953,7 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B28">
         <v>326</v>
@@ -4793,7 +4970,7 @@
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B29">
         <v>336</v>
@@ -4810,7 +4987,7 @@
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B30">
         <v>343</v>
@@ -4827,7 +5004,7 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B31">
         <v>350</v>
@@ -4844,7 +5021,7 @@
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B32">
         <v>367</v>
@@ -4861,7 +5038,7 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B33">
         <v>376</v>
@@ -4878,7 +5055,7 @@
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B34">
         <v>383</v>
@@ -4895,7 +5072,7 @@
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B35">
         <v>413</v>
@@ -4912,7 +5089,7 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B36">
         <v>414</v>
@@ -4929,7 +5106,7 @@
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B37">
         <v>441</v>
@@ -4946,7 +5123,7 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B38">
         <v>472</v>
@@ -4963,7 +5140,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B39">
         <v>486</v>
@@ -4980,7 +5157,7 @@
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B40">
         <v>546</v>
@@ -4997,7 +5174,7 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B41">
         <v>558</v>
@@ -5014,7 +5191,7 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B42">
         <v>573</v>
@@ -5031,7 +5208,7 @@
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B43">
         <v>606</v>
@@ -5048,7 +5225,7 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B44">
         <v>642</v>
@@ -5065,7 +5242,7 @@
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B45">
         <v>643</v>
@@ -5082,7 +5259,7 @@
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B46">
         <v>648</v>
@@ -5099,7 +5276,7 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B47">
         <v>700</v>
@@ -5116,7 +5293,7 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B48">
         <v>706</v>
@@ -5133,7 +5310,7 @@
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B49">
         <v>811</v>
@@ -5150,7 +5327,7 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B50">
         <v>844</v>
@@ -5167,7 +5344,7 @@
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B51">
         <v>1014</v>

</xml_diff>